<commit_message>
Güncel tahmin tablosu: 3-8 Ekim maçları (53 satır, Dixon-Coles + LOO düzeltmeli)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBfpyxGus5xRHHn8xK9mQE
</commit_message>
<xml_diff>
--- a/maclar_ve_tahminler.xlsx
+++ b/maclar_ve_tahminler.xlsx
@@ -61,13 +61,13 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00922B21"/>
+      <color rgb="00707B7C"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00707B7C"/>
+      <color rgb="00922B21"/>
       <sz val="11"/>
     </font>
     <font>
@@ -331,7 +331,7 @@
     <xf numFmtId="0" fontId="4" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -352,7 +352,7 @@
     <xf numFmtId="0" fontId="5" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1075,56 +1075,56 @@
         </is>
       </c>
       <c r="N3" s="37" t="n">
-        <v>77.2</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="O3" s="37" t="n">
-        <v>12.8</v>
+        <v>15.8</v>
       </c>
       <c r="P3" s="37" t="n">
-        <v>10</v>
+        <v>15.3</v>
       </c>
       <c r="Q3" s="38" t="n">
-        <v>3.18</v>
+        <v>2.85</v>
       </c>
       <c r="R3" s="38" t="n">
-        <v>1.14</v>
+        <v>1.33</v>
       </c>
       <c r="S3" s="37" t="n">
-        <v>80.40000000000001</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="T3" s="37" t="n">
-        <v>19.6</v>
+        <v>21.4</v>
       </c>
       <c r="U3" s="37" t="n">
-        <v>65.09999999999999</v>
+        <v>69.2</v>
       </c>
       <c r="V3" s="37" t="n">
-        <v>34.9</v>
+        <v>30.8</v>
       </c>
       <c r="W3" s="37" t="n">
-        <v>92.90000000000001</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="X3" s="37" t="n">
-        <v>90</v>
+        <v>84.7</v>
       </c>
       <c r="Y3" s="37" t="n">
-        <v>22.8</v>
+        <v>31.1</v>
       </c>
       <c r="Z3" s="37" t="n">
-        <v>87.2</v>
+        <v>84.2</v>
       </c>
       <c r="AA3" s="37" t="n">
-        <v>59.9</v>
+        <v>53.3</v>
       </c>
       <c r="AB3" s="37" t="n">
-        <v>26.9</v>
+        <v>29.4</v>
       </c>
       <c r="AC3" s="37" t="n">
-        <v>13.2</v>
+        <v>17.3</v>
       </c>
       <c r="AD3" s="34" t="inlineStr">
         <is>
-          <t>3-1 (%8)</t>
+          <t>2-1 (%8)</t>
         </is>
       </c>
       <c r="AE3" s="34" t="n"/>
@@ -1212,52 +1212,52 @@
         </is>
       </c>
       <c r="N4" s="37" t="n">
-        <v>54.6</v>
+        <v>56.5</v>
       </c>
       <c r="O4" s="37" t="n">
-        <v>20.6</v>
+        <v>19.7</v>
       </c>
       <c r="P4" s="37" t="n">
-        <v>24.9</v>
+        <v>23.9</v>
       </c>
       <c r="Q4" s="38" t="n">
-        <v>2.17</v>
+        <v>2.32</v>
       </c>
       <c r="R4" s="38" t="n">
-        <v>1.42</v>
+        <v>1.47</v>
       </c>
       <c r="S4" s="37" t="n">
-        <v>69.59999999999999</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="T4" s="37" t="n">
-        <v>30.4</v>
+        <v>27.1</v>
       </c>
       <c r="U4" s="37" t="n">
-        <v>67.2</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="V4" s="37" t="n">
-        <v>32.8</v>
+        <v>30.6</v>
       </c>
       <c r="W4" s="37" t="n">
-        <v>87.3</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="X4" s="37" t="n">
-        <v>75.09999999999999</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="Y4" s="37" t="n">
-        <v>45.4</v>
+        <v>43.5</v>
       </c>
       <c r="Z4" s="37" t="n">
-        <v>79.40000000000001</v>
+        <v>80.3</v>
       </c>
       <c r="AA4" s="37" t="n">
-        <v>42.4</v>
+        <v>44</v>
       </c>
       <c r="AB4" s="37" t="n">
-        <v>34.4</v>
+        <v>33.1</v>
       </c>
       <c r="AC4" s="37" t="n">
-        <v>23.3</v>
+        <v>22.9</v>
       </c>
       <c r="AD4" s="34" t="inlineStr">
         <is>
@@ -1343,62 +1343,62 @@
       <c r="L5" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="M5" s="36" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="M5" s="39" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
       <c r="N5" s="37" t="n">
-        <v>71.90000000000001</v>
+        <v>11.7</v>
       </c>
       <c r="O5" s="37" t="n">
-        <v>19.1</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="P5" s="37" t="n">
-        <v>8.9</v>
+        <v>11.7</v>
       </c>
       <c r="Q5" s="38" t="n">
-        <v>1.98</v>
+        <v>0.15</v>
       </c>
       <c r="R5" s="38" t="n">
-        <v>0.53</v>
+        <v>0.15</v>
       </c>
       <c r="S5" s="37" t="n">
-        <v>46.1</v>
+        <v>0.4</v>
       </c>
       <c r="T5" s="37" t="n">
-        <v>53.9</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="U5" s="37" t="n">
-        <v>35.6</v>
+        <v>2.4</v>
       </c>
       <c r="V5" s="37" t="n">
-        <v>64.40000000000001</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="W5" s="37" t="n">
-        <v>71.59999999999999</v>
+        <v>4.1</v>
       </c>
       <c r="X5" s="37" t="n">
-        <v>91.09999999999999</v>
+        <v>88.3</v>
       </c>
       <c r="Y5" s="37" t="n">
-        <v>28.1</v>
+        <v>88.3</v>
       </c>
       <c r="Z5" s="37" t="n">
-        <v>80.90000000000001</v>
+        <v>23.4</v>
       </c>
       <c r="AA5" s="37" t="n">
-        <v>50.8</v>
+        <v>6.1</v>
       </c>
       <c r="AB5" s="37" t="n">
-        <v>39.5</v>
+        <v>87.8</v>
       </c>
       <c r="AC5" s="37" t="n">
-        <v>9.699999999999999</v>
+        <v>6.1</v>
       </c>
       <c r="AD5" s="34" t="inlineStr">
         <is>
-          <t>1-0 (%16)</t>
+          <t>0-0 (%74)</t>
         </is>
       </c>
       <c r="AE5" s="34" t="n"/>
@@ -1480,62 +1480,62 @@
       <c r="L6" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="M6" s="36" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="M6" s="39" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
       <c r="N6" s="37" t="n">
-        <v>99.2</v>
+        <v>11.7</v>
       </c>
       <c r="O6" s="37" t="n">
-        <v>0.7</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="P6" s="37" t="n">
-        <v>0.1</v>
+        <v>11.7</v>
       </c>
       <c r="Q6" s="38" t="n">
-        <v>5.5</v>
+        <v>0.15</v>
       </c>
       <c r="R6" s="38" t="n">
         <v>0.15</v>
       </c>
       <c r="S6" s="37" t="n">
-        <v>91.59999999999999</v>
+        <v>0.4</v>
       </c>
       <c r="T6" s="37" t="n">
-        <v>8.4</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="U6" s="37" t="n">
-        <v>13.9</v>
+        <v>2.4</v>
       </c>
       <c r="V6" s="37" t="n">
-        <v>86.09999999999999</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="W6" s="37" t="n">
-        <v>97.5</v>
+        <v>4.1</v>
       </c>
       <c r="X6" s="37" t="n">
-        <v>99.90000000000001</v>
+        <v>88.3</v>
       </c>
       <c r="Y6" s="37" t="n">
-        <v>0.8</v>
+        <v>88.3</v>
       </c>
       <c r="Z6" s="37" t="n">
-        <v>99.3</v>
+        <v>23.4</v>
       </c>
       <c r="AA6" s="37" t="n">
-        <v>90.2</v>
+        <v>6.1</v>
       </c>
       <c r="AB6" s="37" t="n">
-        <v>9.199999999999999</v>
+        <v>87.8</v>
       </c>
       <c r="AC6" s="37" t="n">
-        <v>0.6</v>
+        <v>6.1</v>
       </c>
       <c r="AD6" s="34" t="inlineStr">
         <is>
-          <t>5-0 (%16)</t>
+          <t>0-0 (%74)</t>
         </is>
       </c>
       <c r="AE6" s="34" t="n"/>
@@ -1617,62 +1617,62 @@
       <c r="L7" s="34" t="n">
         <v>7</v>
       </c>
-      <c r="M7" s="39" t="inlineStr">
+      <c r="M7" s="40" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
       <c r="N7" s="37" t="n">
-        <v>1.5</v>
+        <v>17.5</v>
       </c>
       <c r="O7" s="37" t="n">
-        <v>3</v>
+        <v>13.6</v>
       </c>
       <c r="P7" s="37" t="n">
-        <v>95.59999999999999</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="Q7" s="38" t="n">
-        <v>0.92</v>
+        <v>2.32</v>
       </c>
       <c r="R7" s="38" t="n">
-        <v>5.5</v>
+        <v>4.12</v>
       </c>
       <c r="S7" s="37" t="n">
-        <v>95.2</v>
+        <v>95.5</v>
       </c>
       <c r="T7" s="37" t="n">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="U7" s="37" t="n">
-        <v>59.7</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="V7" s="37" t="n">
-        <v>40.3</v>
+        <v>10.9</v>
       </c>
       <c r="W7" s="37" t="n">
-        <v>98.7</v>
+        <v>99.2</v>
       </c>
       <c r="X7" s="37" t="n">
-        <v>4.4</v>
+        <v>31.1</v>
       </c>
       <c r="Y7" s="37" t="n">
-        <v>98.5</v>
+        <v>82.5</v>
       </c>
       <c r="Z7" s="37" t="n">
-        <v>97</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="AA7" s="37" t="n">
-        <v>4.4</v>
+        <v>21</v>
       </c>
       <c r="AB7" s="37" t="n">
-        <v>12.9</v>
+        <v>22.6</v>
       </c>
       <c r="AC7" s="37" t="n">
-        <v>82.7</v>
+        <v>56.4</v>
       </c>
       <c r="AD7" s="34" t="inlineStr">
         <is>
-          <t>0-5 (%7)</t>
+          <t>2-4 (%5)</t>
         </is>
       </c>
       <c r="AE7" s="34" t="n"/>
@@ -1760,56 +1760,56 @@
         </is>
       </c>
       <c r="N8" s="37" t="n">
-        <v>59.5</v>
+        <v>43.8</v>
       </c>
       <c r="O8" s="37" t="n">
-        <v>34.2</v>
+        <v>42.6</v>
       </c>
       <c r="P8" s="37" t="n">
-        <v>6.3</v>
+        <v>13.6</v>
       </c>
       <c r="Q8" s="38" t="n">
-        <v>1.08</v>
+        <v>0.91</v>
       </c>
       <c r="R8" s="38" t="n">
-        <v>0.19</v>
+        <v>0.41</v>
       </c>
       <c r="S8" s="37" t="n">
-        <v>13.5</v>
+        <v>14.9</v>
       </c>
       <c r="T8" s="37" t="n">
-        <v>86.5</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="U8" s="37" t="n">
-        <v>11.2</v>
+        <v>22.8</v>
       </c>
       <c r="V8" s="37" t="n">
-        <v>88.8</v>
+        <v>77.2</v>
       </c>
       <c r="W8" s="37" t="n">
-        <v>36.1</v>
+        <v>40.8</v>
       </c>
       <c r="X8" s="37" t="n">
-        <v>93.7</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="Y8" s="37" t="n">
-        <v>40.5</v>
+        <v>56.2</v>
       </c>
       <c r="Z8" s="37" t="n">
-        <v>65.8</v>
+        <v>57.4</v>
       </c>
       <c r="AA8" s="37" t="n">
-        <v>36.1</v>
+        <v>29</v>
       </c>
       <c r="AB8" s="37" t="n">
-        <v>58.9</v>
+        <v>59.3</v>
       </c>
       <c r="AC8" s="37" t="n">
-        <v>5</v>
+        <v>11.7</v>
       </c>
       <c r="AD8" s="34" t="inlineStr">
         <is>
-          <t>1-0 (%30)</t>
+          <t>0-0 (%29)</t>
         </is>
       </c>
       <c r="AE8" s="34" t="n"/>
@@ -1897,56 +1897,56 @@
         </is>
       </c>
       <c r="N9" s="37" t="n">
-        <v>96.5</v>
+        <v>76</v>
       </c>
       <c r="O9" s="37" t="n">
-        <v>3.1</v>
+        <v>21.5</v>
       </c>
       <c r="P9" s="37" t="n">
-        <v>0.4</v>
+        <v>2.5</v>
       </c>
       <c r="Q9" s="38" t="n">
-        <v>3.85</v>
+        <v>1.8</v>
       </c>
       <c r="R9" s="38" t="n">
-        <v>0.15</v>
+        <v>0.21</v>
       </c>
       <c r="S9" s="37" t="n">
-        <v>76</v>
+        <v>32.6</v>
       </c>
       <c r="T9" s="37" t="n">
+        <v>67.40000000000001</v>
+      </c>
+      <c r="U9" s="37" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="V9" s="37" t="n">
+        <v>82.8</v>
+      </c>
+      <c r="W9" s="37" t="n">
+        <v>61</v>
+      </c>
+      <c r="X9" s="37" t="n">
+        <v>97.5</v>
+      </c>
+      <c r="Y9" s="37" t="n">
         <v>24</v>
       </c>
-      <c r="U9" s="37" t="n">
-        <v>13.6</v>
-      </c>
-      <c r="V9" s="37" t="n">
-        <v>86.40000000000001</v>
-      </c>
-      <c r="W9" s="37" t="n">
-        <v>90.8</v>
-      </c>
-      <c r="X9" s="37" t="n">
-        <v>99.59999999999999</v>
-      </c>
-      <c r="Y9" s="37" t="n">
-        <v>3.5</v>
-      </c>
       <c r="Z9" s="37" t="n">
-        <v>96.90000000000001</v>
+        <v>78.5</v>
       </c>
       <c r="AA9" s="37" t="n">
-        <v>80.2</v>
+        <v>52.2</v>
       </c>
       <c r="AB9" s="37" t="n">
-        <v>18.5</v>
+        <v>43.6</v>
       </c>
       <c r="AC9" s="37" t="n">
-        <v>1.2</v>
+        <v>4.2</v>
       </c>
       <c r="AD9" s="34" t="inlineStr">
         <is>
-          <t>3-0 (%18)</t>
+          <t>1-0 (%23)</t>
         </is>
       </c>
       <c r="AE9" s="34" t="n"/>
@@ -2034,56 +2034,56 @@
         </is>
       </c>
       <c r="N10" s="37" t="n">
-        <v>69.8</v>
+        <v>59.1</v>
       </c>
       <c r="O10" s="37" t="n">
-        <v>21.8</v>
+        <v>28.3</v>
       </c>
       <c r="P10" s="37" t="n">
-        <v>8.4</v>
+        <v>12.5</v>
       </c>
       <c r="Q10" s="38" t="n">
-        <v>1.73</v>
+        <v>1.36</v>
       </c>
       <c r="R10" s="38" t="n">
-        <v>0.42</v>
+        <v>0.47</v>
       </c>
       <c r="S10" s="37" t="n">
-        <v>36.2</v>
+        <v>27.6</v>
       </c>
       <c r="T10" s="37" t="n">
-        <v>63.8</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="U10" s="37" t="n">
-        <v>28.1</v>
+        <v>27.8</v>
       </c>
       <c r="V10" s="37" t="n">
-        <v>71.90000000000001</v>
+        <v>72.2</v>
       </c>
       <c r="W10" s="37" t="n">
-        <v>63.2</v>
+        <v>54.6</v>
       </c>
       <c r="X10" s="37" t="n">
-        <v>91.59999999999999</v>
+        <v>87.5</v>
       </c>
       <c r="Y10" s="37" t="n">
-        <v>30.2</v>
+        <v>40.9</v>
       </c>
       <c r="Z10" s="37" t="n">
-        <v>78.2</v>
+        <v>71.7</v>
       </c>
       <c r="AA10" s="37" t="n">
-        <v>47.7</v>
+        <v>39.3</v>
       </c>
       <c r="AB10" s="37" t="n">
-        <v>43.9</v>
+        <v>49.8</v>
       </c>
       <c r="AC10" s="37" t="n">
-        <v>8.4</v>
+        <v>10.9</v>
       </c>
       <c r="AD10" s="34" t="inlineStr">
         <is>
-          <t>1-0 (%20)</t>
+          <t>1-0 (%22)</t>
         </is>
       </c>
       <c r="AE10" s="34" t="n"/>
@@ -2167,60 +2167,60 @@
       </c>
       <c r="M11" s="39" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>X</t>
         </is>
       </c>
       <c r="N11" s="37" t="n">
-        <v>4.4</v>
+        <v>11.7</v>
       </c>
       <c r="O11" s="37" t="n">
-        <v>29.8</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="P11" s="37" t="n">
-        <v>65.8</v>
+        <v>11.7</v>
       </c>
       <c r="Q11" s="38" t="n">
         <v>0.15</v>
       </c>
       <c r="R11" s="38" t="n">
-        <v>1.24</v>
+        <v>0.15</v>
       </c>
       <c r="S11" s="37" t="n">
-        <v>16.4</v>
+        <v>0.4</v>
       </c>
       <c r="T11" s="37" t="n">
-        <v>83.59999999999999</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="U11" s="37" t="n">
-        <v>9.9</v>
+        <v>2.4</v>
       </c>
       <c r="V11" s="37" t="n">
-        <v>90.09999999999999</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="W11" s="37" t="n">
-        <v>40.5</v>
+        <v>4.1</v>
       </c>
       <c r="X11" s="37" t="n">
-        <v>34.2</v>
+        <v>88.3</v>
       </c>
       <c r="Y11" s="37" t="n">
-        <v>95.59999999999999</v>
+        <v>88.3</v>
       </c>
       <c r="Z11" s="37" t="n">
-        <v>70.2</v>
+        <v>23.4</v>
       </c>
       <c r="AA11" s="37" t="n">
-        <v>3.8</v>
+        <v>6.1</v>
       </c>
       <c r="AB11" s="37" t="n">
-        <v>55.5</v>
+        <v>87.8</v>
       </c>
       <c r="AC11" s="37" t="n">
-        <v>40.7</v>
+        <v>6.1</v>
       </c>
       <c r="AD11" s="34" t="inlineStr">
         <is>
-          <t>0-1 (%31)</t>
+          <t>0-0 (%74)</t>
         </is>
       </c>
       <c r="AE11" s="34" t="n"/>
@@ -2308,52 +2308,52 @@
         </is>
       </c>
       <c r="N12" s="37" t="n">
-        <v>96.59999999999999</v>
+        <v>96.7</v>
       </c>
       <c r="O12" s="37" t="n">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="P12" s="37" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="Q12" s="38" t="n">
         <v>5.5</v>
       </c>
       <c r="R12" s="38" t="n">
-        <v>0.74</v>
+        <v>0.67</v>
       </c>
       <c r="S12" s="37" t="n">
-        <v>94.5</v>
+        <v>94.2</v>
       </c>
       <c r="T12" s="37" t="n">
-        <v>5.5</v>
+        <v>5.8</v>
       </c>
       <c r="U12" s="37" t="n">
-        <v>52.2</v>
+        <v>48.9</v>
       </c>
       <c r="V12" s="37" t="n">
-        <v>47.8</v>
+        <v>51.1</v>
       </c>
       <c r="W12" s="37" t="n">
-        <v>98.5</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="X12" s="37" t="n">
-        <v>99</v>
+        <v>99.3</v>
       </c>
       <c r="Y12" s="37" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="Z12" s="37" t="n">
-        <v>97.59999999999999</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="AA12" s="37" t="n">
-        <v>84.40000000000001</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="AB12" s="37" t="n">
-        <v>12.1</v>
+        <v>11.8</v>
       </c>
       <c r="AC12" s="37" t="n">
-        <v>3.5</v>
+        <v>3.1</v>
       </c>
       <c r="AD12" s="34" t="inlineStr">
         <is>
@@ -2439,62 +2439,62 @@
       <c r="L13" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="M13" s="36" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="M13" s="39" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
       <c r="N13" s="37" t="n">
-        <v>74.8</v>
+        <v>11.7</v>
       </c>
       <c r="O13" s="37" t="n">
-        <v>20.1</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="P13" s="37" t="n">
-        <v>5.1</v>
+        <v>11.7</v>
       </c>
       <c r="Q13" s="38" t="n">
-        <v>1.77</v>
+        <v>0.15</v>
       </c>
       <c r="R13" s="38" t="n">
-        <v>0.27</v>
+        <v>0.15</v>
       </c>
       <c r="S13" s="37" t="n">
-        <v>33.4</v>
+        <v>0.4</v>
       </c>
       <c r="T13" s="37" t="n">
-        <v>66.59999999999999</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="U13" s="37" t="n">
-        <v>19.8</v>
+        <v>2.4</v>
       </c>
       <c r="V13" s="37" t="n">
-        <v>80.2</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="W13" s="37" t="n">
-        <v>60.5</v>
+        <v>4.1</v>
       </c>
       <c r="X13" s="37" t="n">
-        <v>94.90000000000001</v>
+        <v>88.3</v>
       </c>
       <c r="Y13" s="37" t="n">
-        <v>25.2</v>
+        <v>88.3</v>
       </c>
       <c r="Z13" s="37" t="n">
-        <v>79.90000000000001</v>
+        <v>23.4</v>
       </c>
       <c r="AA13" s="37" t="n">
-        <v>50.6</v>
+        <v>6.1</v>
       </c>
       <c r="AB13" s="37" t="n">
-        <v>43.9</v>
+        <v>87.8</v>
       </c>
       <c r="AC13" s="37" t="n">
-        <v>5.5</v>
+        <v>6.1</v>
       </c>
       <c r="AD13" s="34" t="inlineStr">
         <is>
-          <t>1-0 (%23)</t>
+          <t>0-0 (%74)</t>
         </is>
       </c>
       <c r="AE13" s="34" t="n"/>
@@ -2582,56 +2582,56 @@
         </is>
       </c>
       <c r="N14" s="37" t="n">
-        <v>46</v>
+        <v>46.4</v>
       </c>
       <c r="O14" s="37" t="n">
-        <v>34.5</v>
+        <v>41.1</v>
       </c>
       <c r="P14" s="37" t="n">
-        <v>19.5</v>
+        <v>12.5</v>
       </c>
       <c r="Q14" s="38" t="n">
-        <v>1.01</v>
+        <v>0.83</v>
       </c>
       <c r="R14" s="38" t="n">
-        <v>0.54</v>
+        <v>0.29</v>
       </c>
       <c r="S14" s="37" t="n">
-        <v>20.4</v>
+        <v>10.4</v>
       </c>
       <c r="T14" s="37" t="n">
-        <v>79.59999999999999</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="U14" s="37" t="n">
-        <v>26.6</v>
+        <v>14.4</v>
       </c>
       <c r="V14" s="37" t="n">
-        <v>73.40000000000001</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="W14" s="37" t="n">
-        <v>45.8</v>
+        <v>30.9</v>
       </c>
       <c r="X14" s="37" t="n">
-        <v>80.5</v>
+        <v>87.5</v>
       </c>
       <c r="Y14" s="37" t="n">
-        <v>54</v>
+        <v>53.6</v>
       </c>
       <c r="Z14" s="37" t="n">
-        <v>65.5</v>
+        <v>58.9</v>
       </c>
       <c r="AA14" s="37" t="n">
-        <v>30</v>
+        <v>27.8</v>
       </c>
       <c r="AB14" s="37" t="n">
-        <v>55.5</v>
+        <v>63.4</v>
       </c>
       <c r="AC14" s="37" t="n">
-        <v>14.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AD14" s="34" t="inlineStr">
         <is>
-          <t>1-0 (%21)</t>
+          <t>0-0 (%33)</t>
         </is>
       </c>
       <c r="AE14" s="34" t="n"/>
@@ -2719,56 +2719,56 @@
         </is>
       </c>
       <c r="N15" s="37" t="n">
-        <v>43.3</v>
+        <v>45.6</v>
       </c>
       <c r="O15" s="37" t="n">
-        <v>34.8</v>
+        <v>31.4</v>
       </c>
       <c r="P15" s="37" t="n">
-        <v>21.9</v>
+        <v>23</v>
       </c>
       <c r="Q15" s="38" t="n">
-        <v>0.97</v>
+        <v>1.14</v>
       </c>
       <c r="R15" s="38" t="n">
-        <v>0.6</v>
+        <v>0.72</v>
       </c>
       <c r="S15" s="37" t="n">
-        <v>20.9</v>
+        <v>28.3</v>
       </c>
       <c r="T15" s="37" t="n">
-        <v>79.09999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="U15" s="37" t="n">
-        <v>27.9</v>
+        <v>34.7</v>
       </c>
       <c r="V15" s="37" t="n">
-        <v>72.09999999999999</v>
+        <v>65.3</v>
       </c>
       <c r="W15" s="37" t="n">
-        <v>46.5</v>
+        <v>55.3</v>
       </c>
       <c r="X15" s="37" t="n">
-        <v>78.09999999999999</v>
+        <v>77</v>
       </c>
       <c r="Y15" s="37" t="n">
-        <v>56.7</v>
+        <v>54.4</v>
       </c>
       <c r="Z15" s="37" t="n">
-        <v>65.2</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="AA15" s="37" t="n">
-        <v>28.6</v>
+        <v>31.3</v>
       </c>
       <c r="AB15" s="37" t="n">
-        <v>55.3</v>
+        <v>50.9</v>
       </c>
       <c r="AC15" s="37" t="n">
-        <v>16.1</v>
+        <v>17.8</v>
       </c>
       <c r="AD15" s="34" t="inlineStr">
         <is>
-          <t>0-0 (%21)</t>
+          <t>1-0 (%18)</t>
         </is>
       </c>
       <c r="AE15" s="34" t="n"/>
@@ -2852,56 +2852,56 @@
         </is>
       </c>
       <c r="N16" s="37" t="n">
-        <v>70.59999999999999</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="O16" s="37" t="n">
-        <v>19.1</v>
+        <v>17.3</v>
       </c>
       <c r="P16" s="37" t="n">
-        <v>10.3</v>
+        <v>13.2</v>
       </c>
       <c r="Q16" s="38" t="n">
-        <v>2.04</v>
+        <v>2.42</v>
       </c>
       <c r="R16" s="38" t="n">
-        <v>0.63</v>
+        <v>0.97</v>
       </c>
       <c r="S16" s="37" t="n">
-        <v>49.8</v>
+        <v>65.8</v>
       </c>
       <c r="T16" s="37" t="n">
-        <v>50.2</v>
+        <v>34.2</v>
       </c>
       <c r="U16" s="37" t="n">
-        <v>40.6</v>
+        <v>56.4</v>
       </c>
       <c r="V16" s="37" t="n">
-        <v>59.4</v>
+        <v>43.6</v>
       </c>
       <c r="W16" s="37" t="n">
-        <v>74.5</v>
+        <v>85.2</v>
       </c>
       <c r="X16" s="37" t="n">
-        <v>89.7</v>
+        <v>86.8</v>
       </c>
       <c r="Y16" s="37" t="n">
-        <v>29.4</v>
+        <v>30.6</v>
       </c>
       <c r="Z16" s="37" t="n">
-        <v>80.90000000000001</v>
+        <v>82.7</v>
       </c>
       <c r="AA16" s="37" t="n">
-        <v>49.4</v>
+        <v>50.7</v>
       </c>
       <c r="AB16" s="37" t="n">
-        <v>39.6</v>
+        <v>34.7</v>
       </c>
       <c r="AC16" s="37" t="n">
-        <v>11</v>
+        <v>14.6</v>
       </c>
       <c r="AD16" s="34" t="inlineStr">
         <is>
-          <t>2-0 (%14)</t>
+          <t>2-0 (%10)</t>
         </is>
       </c>
       <c r="AE16" s="34" t="n"/>
@@ -2983,62 +2983,62 @@
       <c r="L17" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="M17" s="40" t="inlineStr">
+      <c r="M17" s="39" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
       <c r="N17" s="37" t="n">
-        <v>28.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="O17" s="37" t="n">
-        <v>54.9</v>
+        <v>51.5</v>
       </c>
       <c r="P17" s="37" t="n">
-        <v>17</v>
+        <v>38.6</v>
       </c>
       <c r="Q17" s="38" t="n">
-        <v>0.43</v>
+        <v>0.22</v>
       </c>
       <c r="R17" s="38" t="n">
-        <v>0.28</v>
+        <v>0.64</v>
       </c>
       <c r="S17" s="37" t="n">
-        <v>3.7</v>
+        <v>5.7</v>
       </c>
       <c r="T17" s="37" t="n">
-        <v>96.3</v>
+        <v>94.3</v>
       </c>
       <c r="U17" s="37" t="n">
-        <v>8.699999999999999</v>
+        <v>11</v>
       </c>
       <c r="V17" s="37" t="n">
-        <v>91.3</v>
+        <v>89</v>
       </c>
       <c r="W17" s="37" t="n">
-        <v>16.3</v>
+        <v>22.9</v>
       </c>
       <c r="X17" s="37" t="n">
-        <v>83</v>
+        <v>61.4</v>
       </c>
       <c r="Y17" s="37" t="n">
-        <v>71.90000000000001</v>
+        <v>90.2</v>
       </c>
       <c r="Z17" s="37" t="n">
-        <v>45.1</v>
+        <v>48.5</v>
       </c>
       <c r="AA17" s="37" t="n">
-        <v>15.8</v>
+        <v>7.3</v>
       </c>
       <c r="AB17" s="37" t="n">
-        <v>74.2</v>
+        <v>69.8</v>
       </c>
       <c r="AC17" s="37" t="n">
-        <v>10</v>
+        <v>22.9</v>
       </c>
       <c r="AD17" s="34" t="inlineStr">
         <is>
-          <t>0-0 (%49)</t>
+          <t>0-0 (%44)</t>
         </is>
       </c>
       <c r="AE17" s="34" t="n"/>
@@ -3120,62 +3120,62 @@
       <c r="L18" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="M18" s="39" t="inlineStr">
+      <c r="M18" s="40" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
       <c r="N18" s="37" t="n">
-        <v>17.6</v>
+        <v>10.3</v>
       </c>
       <c r="O18" s="37" t="n">
-        <v>21.6</v>
+        <v>21.7</v>
       </c>
       <c r="P18" s="37" t="n">
-        <v>60.7</v>
+        <v>68</v>
       </c>
       <c r="Q18" s="38" t="n">
-        <v>0.93</v>
+        <v>0.87</v>
       </c>
       <c r="R18" s="38" t="n">
-        <v>1.93</v>
+        <v>2.33</v>
       </c>
       <c r="S18" s="37" t="n">
-        <v>54.6</v>
+        <v>61.9</v>
       </c>
       <c r="T18" s="37" t="n">
-        <v>45.4</v>
+        <v>38.1</v>
       </c>
       <c r="U18" s="37" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="V18" s="37" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="W18" s="37" t="n">
+        <v>84.90000000000001</v>
+      </c>
+      <c r="X18" s="37" t="n">
+        <v>32</v>
+      </c>
+      <c r="Y18" s="37" t="n">
+        <v>89.7</v>
+      </c>
+      <c r="Z18" s="37" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="AA18" s="37" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="AB18" s="37" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="AC18" s="37" t="n">
         <v>51.9</v>
       </c>
-      <c r="V18" s="37" t="n">
-        <v>48.1</v>
-      </c>
-      <c r="W18" s="37" t="n">
-        <v>78</v>
-      </c>
-      <c r="X18" s="37" t="n">
-        <v>39.3</v>
-      </c>
-      <c r="Y18" s="37" t="n">
-        <v>82.40000000000001</v>
-      </c>
-      <c r="Z18" s="37" t="n">
-        <v>78.40000000000001</v>
-      </c>
-      <c r="AA18" s="37" t="n">
-        <v>17</v>
-      </c>
-      <c r="AB18" s="37" t="n">
-        <v>38.6</v>
-      </c>
-      <c r="AC18" s="37" t="n">
-        <v>44.5</v>
-      </c>
       <c r="AD18" s="34" t="inlineStr">
         <is>
-          <t>0-1 (%11)</t>
+          <t>0-2 (%11)</t>
         </is>
       </c>
       <c r="AE18" s="34" t="n"/>
@@ -3263,56 +3263,56 @@
         </is>
       </c>
       <c r="N19" s="37" t="n">
-        <v>65.90000000000001</v>
+        <v>58.3</v>
       </c>
       <c r="O19" s="37" t="n">
-        <v>28.7</v>
+        <v>32.6</v>
       </c>
       <c r="P19" s="37" t="n">
-        <v>5.4</v>
+        <v>9.1</v>
       </c>
       <c r="Q19" s="38" t="n">
-        <v>1.29</v>
+        <v>1.37</v>
       </c>
       <c r="R19" s="38" t="n">
-        <v>0.19</v>
+        <v>0.43</v>
       </c>
       <c r="S19" s="37" t="n">
-        <v>18.7</v>
+        <v>27.1</v>
       </c>
       <c r="T19" s="37" t="n">
-        <v>81.3</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="U19" s="37" t="n">
-        <v>12.7</v>
+        <v>28.6</v>
       </c>
       <c r="V19" s="37" t="n">
-        <v>87.3</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="W19" s="37" t="n">
-        <v>43.6</v>
+        <v>56.3</v>
       </c>
       <c r="X19" s="37" t="n">
-        <v>94.59999999999999</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="Y19" s="37" t="n">
-        <v>34.1</v>
+        <v>41.7</v>
       </c>
       <c r="Z19" s="37" t="n">
-        <v>71.3</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="AA19" s="37" t="n">
-        <v>41.3</v>
+        <v>40.1</v>
       </c>
       <c r="AB19" s="37" t="n">
-        <v>53.9</v>
+        <v>49.9</v>
       </c>
       <c r="AC19" s="37" t="n">
-        <v>4.7</v>
+        <v>10.1</v>
       </c>
       <c r="AD19" s="34" t="inlineStr">
         <is>
-          <t>1-0 (%29)</t>
+          <t>1-0 (%20)</t>
         </is>
       </c>
       <c r="AE19" s="34" t="n"/>
@@ -3400,56 +3400,56 @@
         </is>
       </c>
       <c r="N20" s="37" t="n">
-        <v>64.09999999999999</v>
+        <v>62.9</v>
       </c>
       <c r="O20" s="37" t="n">
-        <v>22.8</v>
+        <v>22.5</v>
       </c>
       <c r="P20" s="37" t="n">
-        <v>13.1</v>
+        <v>14.6</v>
       </c>
       <c r="Q20" s="38" t="n">
-        <v>1.74</v>
+        <v>1.83</v>
       </c>
       <c r="R20" s="38" t="n">
-        <v>0.64</v>
+        <v>0.75</v>
       </c>
       <c r="S20" s="37" t="n">
-        <v>42.4</v>
+        <v>47.6</v>
       </c>
       <c r="T20" s="37" t="n">
-        <v>57.6</v>
+        <v>52.4</v>
       </c>
       <c r="U20" s="37" t="n">
-        <v>38.8</v>
+        <v>44.4</v>
       </c>
       <c r="V20" s="37" t="n">
-        <v>61.2</v>
+        <v>55.6</v>
       </c>
       <c r="W20" s="37" t="n">
-        <v>68.59999999999999</v>
+        <v>73</v>
       </c>
       <c r="X20" s="37" t="n">
-        <v>86.90000000000001</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="Y20" s="37" t="n">
-        <v>35.9</v>
+        <v>37.1</v>
       </c>
       <c r="Z20" s="37" t="n">
-        <v>77.2</v>
+        <v>77.5</v>
       </c>
       <c r="AA20" s="37" t="n">
-        <v>44.9</v>
+        <v>45.1</v>
       </c>
       <c r="AB20" s="37" t="n">
-        <v>42.5</v>
+        <v>40.7</v>
       </c>
       <c r="AC20" s="37" t="n">
-        <v>12.6</v>
+        <v>14.3</v>
       </c>
       <c r="AD20" s="34" t="inlineStr">
         <is>
-          <t>1-0 (%16)</t>
+          <t>1-0 (%14)</t>
         </is>
       </c>
       <c r="AE20" s="34" t="n"/>
@@ -3531,62 +3531,62 @@
       <c r="L21" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="M21" s="40" t="inlineStr">
+      <c r="M21" s="39" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
       <c r="N21" s="37" t="n">
-        <v>32.3</v>
+        <v>37.2</v>
       </c>
       <c r="O21" s="37" t="n">
-        <v>44.5</v>
+        <v>38.2</v>
       </c>
       <c r="P21" s="37" t="n">
-        <v>23.2</v>
+        <v>24.6</v>
       </c>
       <c r="Q21" s="38" t="n">
-        <v>0.61</v>
+        <v>1.06</v>
       </c>
       <c r="R21" s="38" t="n">
-        <v>0.47</v>
+        <v>0.83</v>
       </c>
       <c r="S21" s="37" t="n">
-        <v>9.5</v>
+        <v>29.5</v>
       </c>
       <c r="T21" s="37" t="n">
-        <v>90.5</v>
+        <v>70.5</v>
       </c>
       <c r="U21" s="37" t="n">
-        <v>17.1</v>
+        <v>40.2</v>
       </c>
       <c r="V21" s="37" t="n">
-        <v>82.90000000000001</v>
+        <v>59.8</v>
       </c>
       <c r="W21" s="37" t="n">
-        <v>29.3</v>
+        <v>59.8</v>
       </c>
       <c r="X21" s="37" t="n">
-        <v>76.8</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="Y21" s="37" t="n">
-        <v>67.7</v>
+        <v>62.8</v>
       </c>
       <c r="Z21" s="37" t="n">
-        <v>55.5</v>
+        <v>61.8</v>
       </c>
       <c r="AA21" s="37" t="n">
-        <v>19.9</v>
+        <v>28.4</v>
       </c>
       <c r="AB21" s="37" t="n">
-        <v>65.2</v>
+        <v>50.6</v>
       </c>
       <c r="AC21" s="37" t="n">
-        <v>14.9</v>
+        <v>21</v>
       </c>
       <c r="AD21" s="34" t="inlineStr">
         <is>
-          <t>0-0 (%34)</t>
+          <t>0-0 (%18)</t>
         </is>
       </c>
       <c r="AE21" s="34" t="n"/>
@@ -3674,56 +3674,56 @@
         </is>
       </c>
       <c r="N22" s="37" t="n">
-        <v>84.3</v>
+        <v>91.7</v>
       </c>
       <c r="O22" s="37" t="n">
-        <v>11.8</v>
+        <v>7.6</v>
       </c>
       <c r="P22" s="37" t="n">
-        <v>3.9</v>
+        <v>0.7</v>
       </c>
       <c r="Q22" s="38" t="n">
-        <v>2.58</v>
+        <v>3.23</v>
       </c>
       <c r="R22" s="38" t="n">
-        <v>0.4</v>
+        <v>0.26</v>
       </c>
       <c r="S22" s="37" t="n">
-        <v>57.2</v>
+        <v>67.8</v>
       </c>
       <c r="T22" s="37" t="n">
-        <v>42.8</v>
+        <v>32.2</v>
       </c>
       <c r="U22" s="37" t="n">
-        <v>30.3</v>
+        <v>23</v>
       </c>
       <c r="V22" s="37" t="n">
-        <v>69.7</v>
+        <v>77</v>
       </c>
       <c r="W22" s="37" t="n">
-        <v>79.7</v>
+        <v>87</v>
       </c>
       <c r="X22" s="37" t="n">
-        <v>96.09999999999999</v>
+        <v>99.3</v>
       </c>
       <c r="Y22" s="37" t="n">
-        <v>15.7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="Z22" s="37" t="n">
-        <v>88.2</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="AA22" s="37" t="n">
-        <v>62.4</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="AB22" s="37" t="n">
-        <v>31.9</v>
+        <v>24.5</v>
       </c>
       <c r="AC22" s="37" t="n">
-        <v>5.7</v>
+        <v>2.9</v>
       </c>
       <c r="AD22" s="34" t="inlineStr">
         <is>
-          <t>2-0 (%17)</t>
+          <t>3-0 (%17)</t>
         </is>
       </c>
       <c r="AE22" s="34" t="n"/>
@@ -3811,52 +3811,52 @@
         </is>
       </c>
       <c r="N23" s="37" t="n">
-        <v>85.59999999999999</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="O23" s="37" t="n">
-        <v>9.300000000000001</v>
+        <v>13.2</v>
       </c>
       <c r="P23" s="37" t="n">
-        <v>5.1</v>
+        <v>4.9</v>
       </c>
       <c r="Q23" s="38" t="n">
-        <v>3.41</v>
+        <v>3.15</v>
       </c>
       <c r="R23" s="38" t="n">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="S23" s="37" t="n">
-        <v>79</v>
+        <v>75.2</v>
       </c>
       <c r="T23" s="37" t="n">
-        <v>21</v>
+        <v>24.8</v>
       </c>
       <c r="U23" s="37" t="n">
-        <v>53.1</v>
+        <v>53.5</v>
       </c>
       <c r="V23" s="37" t="n">
-        <v>46.9</v>
+        <v>46.5</v>
       </c>
       <c r="W23" s="37" t="n">
-        <v>92.2</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="X23" s="37" t="n">
-        <v>94.90000000000001</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="Y23" s="37" t="n">
-        <v>14.4</v>
+        <v>18.1</v>
       </c>
       <c r="Z23" s="37" t="n">
-        <v>90.7</v>
+        <v>86.8</v>
       </c>
       <c r="AA23" s="37" t="n">
-        <v>67.09999999999999</v>
+        <v>64.2</v>
       </c>
       <c r="AB23" s="37" t="n">
-        <v>24.6</v>
+        <v>26.7</v>
       </c>
       <c r="AC23" s="37" t="n">
-        <v>8.300000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="AD23" s="34" t="inlineStr">
         <is>
@@ -3948,52 +3948,52 @@
         </is>
       </c>
       <c r="N24" s="37" t="n">
-        <v>86.5</v>
+        <v>83.7</v>
       </c>
       <c r="O24" s="37" t="n">
-        <v>7.7</v>
+        <v>9.5</v>
       </c>
       <c r="P24" s="37" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="Q24" s="38" t="n">
-        <v>4.35</v>
+        <v>4.39</v>
       </c>
       <c r="R24" s="38" t="n">
-        <v>1.29</v>
+        <v>1.49</v>
       </c>
       <c r="S24" s="37" t="n">
-        <v>91.90000000000001</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="T24" s="37" t="n">
-        <v>8.1</v>
+        <v>6.9</v>
       </c>
       <c r="U24" s="37" t="n">
-        <v>71.5</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="V24" s="37" t="n">
-        <v>28.5</v>
+        <v>23.1</v>
       </c>
       <c r="W24" s="37" t="n">
-        <v>97.59999999999999</v>
+        <v>98.5</v>
       </c>
       <c r="X24" s="37" t="n">
-        <v>94.2</v>
+        <v>93.2</v>
       </c>
       <c r="Y24" s="37" t="n">
-        <v>13.5</v>
+        <v>16.3</v>
       </c>
       <c r="Z24" s="37" t="n">
-        <v>92.3</v>
+        <v>90.5</v>
       </c>
       <c r="AA24" s="37" t="n">
-        <v>70.2</v>
+        <v>68.2</v>
       </c>
       <c r="AB24" s="37" t="n">
-        <v>19.8</v>
+        <v>20.1</v>
       </c>
       <c r="AC24" s="37" t="n">
-        <v>10</v>
+        <v>11.7</v>
       </c>
       <c r="AD24" s="34" t="inlineStr">
         <is>
@@ -4079,62 +4079,62 @@
       <c r="L25" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="M25" s="39" t="inlineStr">
+      <c r="M25" s="40" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
       <c r="N25" s="37" t="n">
-        <v>17.4</v>
+        <v>24.7</v>
       </c>
       <c r="O25" s="37" t="n">
-        <v>22.3</v>
+        <v>24</v>
       </c>
       <c r="P25" s="37" t="n">
-        <v>60.2</v>
+        <v>51.3</v>
       </c>
       <c r="Q25" s="38" t="n">
-        <v>0.88</v>
+        <v>1.57</v>
       </c>
       <c r="R25" s="38" t="n">
-        <v>1.85</v>
+        <v>2.25</v>
       </c>
       <c r="S25" s="37" t="n">
-        <v>51.3</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="T25" s="37" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="U25" s="37" t="n">
+        <v>72.7</v>
+      </c>
+      <c r="V25" s="37" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="W25" s="37" t="n">
+        <v>91.3</v>
+      </c>
+      <c r="X25" s="37" t="n">
         <v>48.7</v>
       </c>
-      <c r="U25" s="37" t="n">
-        <v>49.3</v>
-      </c>
-      <c r="V25" s="37" t="n">
-        <v>50.7</v>
-      </c>
-      <c r="W25" s="37" t="n">
-        <v>75.7</v>
-      </c>
-      <c r="X25" s="37" t="n">
-        <v>39.8</v>
-      </c>
       <c r="Y25" s="37" t="n">
-        <v>82.59999999999999</v>
+        <v>75.3</v>
       </c>
       <c r="Z25" s="37" t="n">
-        <v>77.7</v>
+        <v>76</v>
       </c>
       <c r="AA25" s="37" t="n">
-        <v>16.5</v>
+        <v>24.8</v>
       </c>
       <c r="AB25" s="37" t="n">
-        <v>39.8</v>
+        <v>33.2</v>
       </c>
       <c r="AC25" s="37" t="n">
-        <v>43.7</v>
+        <v>41.9</v>
       </c>
       <c r="AD25" s="34" t="inlineStr">
         <is>
-          <t>0-1 (%12)</t>
+          <t>1-1 (%10)</t>
         </is>
       </c>
       <c r="AE25" s="34" t="n"/>
@@ -4211,67 +4211,67 @@
         </is>
       </c>
       <c r="K26" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="L26" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="L26" s="41" t="n">
-        <v>0</v>
-      </c>
       <c r="M26" s="43" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="N26" s="44" t="n">
-        <v>53.2</v>
+        <v>53</v>
       </c>
       <c r="O26" s="44" t="n">
-        <v>29.4</v>
+        <v>29.5</v>
       </c>
       <c r="P26" s="44" t="n">
-        <v>17.4</v>
+        <v>17.5</v>
       </c>
       <c r="Q26" s="45" t="n">
         <v>1.28</v>
       </c>
       <c r="R26" s="45" t="n">
-        <v>0.6</v>
+        <v>0.61</v>
       </c>
       <c r="S26" s="44" t="n">
-        <v>29.1</v>
+        <v>29.4</v>
       </c>
       <c r="T26" s="44" t="n">
-        <v>70.90000000000001</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="U26" s="44" t="n">
-        <v>32.5</v>
+        <v>33</v>
       </c>
       <c r="V26" s="44" t="n">
-        <v>67.5</v>
+        <v>67</v>
       </c>
       <c r="W26" s="44" t="n">
-        <v>56</v>
+        <v>56.5</v>
       </c>
       <c r="X26" s="44" t="n">
-        <v>82.59999999999999</v>
+        <v>82.5</v>
       </c>
       <c r="Y26" s="44" t="n">
-        <v>46.8</v>
+        <v>47</v>
       </c>
       <c r="Z26" s="44" t="n">
-        <v>70.59999999999999</v>
+        <v>70.5</v>
       </c>
       <c r="AA26" s="44" t="n">
         <v>35.9</v>
       </c>
       <c r="AB26" s="44" t="n">
-        <v>49.9</v>
+        <v>49.7</v>
       </c>
       <c r="AC26" s="44" t="n">
-        <v>14.3</v>
+        <v>14.4</v>
       </c>
       <c r="AD26" s="41" t="inlineStr">
         <is>
-          <t>1-0 (%20)</t>
+          <t>1-0 (%19)</t>
         </is>
       </c>
       <c r="AE26" s="41" t="n"/>
@@ -4364,52 +4364,52 @@
         </is>
       </c>
       <c r="N27" s="49" t="n">
-        <v>27.8</v>
+        <v>28.9</v>
       </c>
       <c r="O27" s="49" t="n">
         <v>30.7</v>
       </c>
       <c r="P27" s="49" t="n">
-        <v>41.4</v>
+        <v>40.4</v>
       </c>
       <c r="Q27" s="50" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="R27" s="50" t="n">
         <v>1.12</v>
       </c>
       <c r="S27" s="49" t="n">
-        <v>31.7</v>
+        <v>32.8</v>
       </c>
       <c r="T27" s="49" t="n">
-        <v>68.3</v>
+        <v>67.2</v>
       </c>
       <c r="U27" s="49" t="n">
-        <v>38.8</v>
+        <v>40</v>
       </c>
       <c r="V27" s="49" t="n">
-        <v>61.2</v>
+        <v>60</v>
       </c>
       <c r="W27" s="49" t="n">
-        <v>58.8</v>
+        <v>60</v>
       </c>
       <c r="X27" s="49" t="n">
-        <v>58.6</v>
+        <v>59.6</v>
       </c>
       <c r="Y27" s="49" t="n">
-        <v>72.2</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="Z27" s="49" t="n">
         <v>69.3</v>
       </c>
       <c r="AA27" s="49" t="n">
-        <v>21.2</v>
+        <v>22.1</v>
       </c>
       <c r="AB27" s="49" t="n">
-        <v>49.5</v>
+        <v>49</v>
       </c>
       <c r="AC27" s="49" t="n">
-        <v>29.3</v>
+        <v>28.9</v>
       </c>
       <c r="AD27" s="51" t="inlineStr">
         <is>
@@ -4506,13 +4506,13 @@
         </is>
       </c>
       <c r="N28" s="49" t="n">
-        <v>66.5</v>
+        <v>65.2</v>
       </c>
       <c r="O28" s="49" t="n">
-        <v>28.1</v>
+        <v>30.8</v>
       </c>
       <c r="P28" s="49" t="n">
-        <v>5.4</v>
+        <v>4</v>
       </c>
       <c r="Q28" s="50" t="n">
         <v>1.32</v>
@@ -4521,31 +4521,31 @@
         <v>0.2</v>
       </c>
       <c r="S28" s="49" t="n">
-        <v>19.5</v>
+        <v>19.6</v>
       </c>
       <c r="T28" s="49" t="n">
-        <v>80.5</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="U28" s="49" t="n">
-        <v>13.2</v>
+        <v>14.6</v>
       </c>
       <c r="V28" s="49" t="n">
-        <v>86.8</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="W28" s="49" t="n">
-        <v>44.8</v>
+        <v>46.3</v>
       </c>
       <c r="X28" s="49" t="n">
-        <v>94.59999999999999</v>
+        <v>96</v>
       </c>
       <c r="Y28" s="49" t="n">
-        <v>33.5</v>
+        <v>34.8</v>
       </c>
       <c r="Z28" s="49" t="n">
-        <v>71.90000000000001</v>
+        <v>69.2</v>
       </c>
       <c r="AA28" s="49" t="n">
-        <v>41.9</v>
+        <v>42</v>
       </c>
       <c r="AB28" s="49" t="n">
         <v>53.2</v>
@@ -4555,7 +4555,7 @@
       </c>
       <c r="AD28" s="51" t="inlineStr">
         <is>
-          <t>1-0 (%29)</t>
+          <t>1-0 (%27)</t>
         </is>
       </c>
       <c r="AE28" s="52" t="n"/>
@@ -4647,56 +4647,56 @@
         </is>
       </c>
       <c r="N29" s="49" t="n">
-        <v>32</v>
+        <v>29.7</v>
       </c>
       <c r="O29" s="49" t="n">
-        <v>21.4</v>
+        <v>25.5</v>
       </c>
       <c r="P29" s="49" t="n">
-        <v>46.6</v>
+        <v>44.8</v>
       </c>
       <c r="Q29" s="50" t="n">
         <v>1.65</v>
       </c>
       <c r="R29" s="50" t="n">
-        <v>2.02</v>
+        <v>2.03</v>
       </c>
       <c r="S29" s="49" t="n">
-        <v>70.90000000000001</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="T29" s="49" t="n">
-        <v>29.1</v>
+        <v>28.9</v>
       </c>
       <c r="U29" s="49" t="n">
-        <v>70.09999999999999</v>
+        <v>72.3</v>
       </c>
       <c r="V29" s="49" t="n">
-        <v>29.9</v>
+        <v>27.7</v>
       </c>
       <c r="W29" s="49" t="n">
-        <v>88.09999999999999</v>
+        <v>90.3</v>
       </c>
       <c r="X29" s="49" t="n">
-        <v>53.4</v>
+        <v>55.2</v>
       </c>
       <c r="Y29" s="49" t="n">
-        <v>68</v>
+        <v>70.3</v>
       </c>
       <c r="Z29" s="49" t="n">
-        <v>78.59999999999999</v>
+        <v>74.5</v>
       </c>
       <c r="AA29" s="49" t="n">
-        <v>28.1</v>
+        <v>28</v>
       </c>
       <c r="AB29" s="49" t="n">
-        <v>34.5</v>
+        <v>34.4</v>
       </c>
       <c r="AC29" s="49" t="n">
-        <v>37.4</v>
+        <v>37.6</v>
       </c>
       <c r="AD29" s="51" t="inlineStr">
         <is>
-          <t>1-2 (%9)</t>
+          <t>1-1 (%11)</t>
         </is>
       </c>
       <c r="AE29" s="46" t="n"/>
@@ -4788,56 +4788,56 @@
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>18.2</v>
+        <v>16.5</v>
       </c>
       <c r="O30" s="49" t="n">
-        <v>53.4</v>
+        <v>56.5</v>
       </c>
       <c r="P30" s="49" t="n">
-        <v>28.4</v>
+        <v>26.9</v>
       </c>
       <c r="Q30" s="50" t="n">
         <v>0.31</v>
       </c>
       <c r="R30" s="50" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
       <c r="S30" s="49" t="n">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
       <c r="T30" s="49" t="n">
-        <v>95.8</v>
+        <v>95.7</v>
       </c>
       <c r="U30" s="49" t="n">
-        <v>9.699999999999999</v>
+        <v>11.5</v>
       </c>
       <c r="V30" s="49" t="n">
-        <v>90.3</v>
+        <v>88.5</v>
       </c>
       <c r="W30" s="49" t="n">
-        <v>17.8</v>
+        <v>19.6</v>
       </c>
       <c r="X30" s="49" t="n">
-        <v>71.59999999999999</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="Y30" s="49" t="n">
-        <v>81.8</v>
+        <v>83.5</v>
       </c>
       <c r="Z30" s="49" t="n">
-        <v>46.6</v>
+        <v>43.5</v>
       </c>
       <c r="AA30" s="49" t="n">
         <v>10.8</v>
       </c>
       <c r="AB30" s="49" t="n">
-        <v>72.90000000000001</v>
+        <v>72.8</v>
       </c>
       <c r="AC30" s="49" t="n">
-        <v>16.2</v>
+        <v>16.3</v>
       </c>
       <c r="AD30" s="51" t="inlineStr">
         <is>
-          <t>0-0 (%47)</t>
+          <t>0-0 (%48)</t>
         </is>
       </c>
       <c r="AE30" s="52" t="n"/>
@@ -4929,49 +4929,49 @@
         </is>
       </c>
       <c r="N31" s="49" t="n">
-        <v>95.40000000000001</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="O31" s="49" t="n">
-        <v>3.6</v>
+        <v>4.4</v>
       </c>
       <c r="P31" s="49" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="Q31" s="50" t="n">
-        <v>4.17</v>
+        <v>4.19</v>
       </c>
       <c r="R31" s="50" t="n">
         <v>0.38</v>
       </c>
       <c r="S31" s="49" t="n">
-        <v>83.09999999999999</v>
+        <v>83.2</v>
       </c>
       <c r="T31" s="49" t="n">
-        <v>16.9</v>
+        <v>16.8</v>
       </c>
       <c r="U31" s="49" t="n">
-        <v>31.4</v>
+        <v>31.7</v>
       </c>
       <c r="V31" s="49" t="n">
-        <v>68.59999999999999</v>
+        <v>68.3</v>
       </c>
       <c r="W31" s="49" t="n">
-        <v>94.09999999999999</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="X31" s="49" t="n">
-        <v>99</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="Y31" s="49" t="n">
-        <v>4.6</v>
+        <v>4.9</v>
       </c>
       <c r="Z31" s="49" t="n">
-        <v>96.40000000000001</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="AA31" s="49" t="n">
-        <v>79.8</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="AB31" s="49" t="n">
-        <v>17.4</v>
+        <v>17.3</v>
       </c>
       <c r="AC31" s="49" t="n">
         <v>2.8</v>
@@ -5070,19 +5070,19 @@
         </is>
       </c>
       <c r="N32" s="49" t="n">
-        <v>76.59999999999999</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="O32" s="49" t="n">
-        <v>11.8</v>
+        <v>13.2</v>
       </c>
       <c r="P32" s="49" t="n">
-        <v>11.6</v>
+        <v>10.7</v>
       </c>
       <c r="Q32" s="50" t="n">
-        <v>3.73</v>
+        <v>3.74</v>
       </c>
       <c r="R32" s="50" t="n">
-        <v>1.56</v>
+        <v>1.55</v>
       </c>
       <c r="S32" s="49" t="n">
         <v>89.7</v>
@@ -5091,31 +5091,31 @@
         <v>10.3</v>
       </c>
       <c r="U32" s="49" t="n">
-        <v>77.09999999999999</v>
+        <v>77.7</v>
       </c>
       <c r="V32" s="49" t="n">
-        <v>22.9</v>
+        <v>22.3</v>
       </c>
       <c r="W32" s="49" t="n">
-        <v>96.8</v>
+        <v>97.5</v>
       </c>
       <c r="X32" s="49" t="n">
-        <v>88.40000000000001</v>
+        <v>89.3</v>
       </c>
       <c r="Y32" s="49" t="n">
-        <v>23.4</v>
+        <v>23.9</v>
       </c>
       <c r="Z32" s="49" t="n">
-        <v>88.2</v>
+        <v>86.8</v>
       </c>
       <c r="AA32" s="49" t="n">
-        <v>60.8</v>
+        <v>61.1</v>
       </c>
       <c r="AB32" s="49" t="n">
         <v>23.8</v>
       </c>
       <c r="AC32" s="49" t="n">
-        <v>15.3</v>
+        <v>15.2</v>
       </c>
       <c r="AD32" s="51" t="inlineStr">
         <is>
@@ -5211,16 +5211,16 @@
         </is>
       </c>
       <c r="N33" s="49" t="n">
-        <v>51.7</v>
+        <v>50.7</v>
       </c>
       <c r="O33" s="49" t="n">
-        <v>42</v>
+        <v>44.1</v>
       </c>
       <c r="P33" s="49" t="n">
-        <v>6.4</v>
+        <v>5.2</v>
       </c>
       <c r="Q33" s="50" t="n">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="R33" s="50" t="n">
         <v>0.15</v>
@@ -5232,35 +5232,35 @@
         <v>92.09999999999999</v>
       </c>
       <c r="U33" s="49" t="n">
-        <v>7.9</v>
+        <v>9.1</v>
       </c>
       <c r="V33" s="49" t="n">
-        <v>92.09999999999999</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="W33" s="49" t="n">
-        <v>26.1</v>
+        <v>27.4</v>
       </c>
       <c r="X33" s="49" t="n">
-        <v>93.59999999999999</v>
+        <v>94.8</v>
       </c>
       <c r="Y33" s="49" t="n">
-        <v>48.3</v>
+        <v>49.3</v>
       </c>
       <c r="Z33" s="49" t="n">
-        <v>58</v>
+        <v>55.9</v>
       </c>
       <c r="AA33" s="49" t="n">
-        <v>29.8</v>
+        <v>29.9</v>
       </c>
       <c r="AB33" s="49" t="n">
-        <v>65.7</v>
+        <v>65.5</v>
       </c>
       <c r="AC33" s="49" t="n">
         <v>4.5</v>
       </c>
       <c r="AD33" s="51" t="inlineStr">
         <is>
-          <t>0-0 (%37)</t>
+          <t>0-0 (%38)</t>
         </is>
       </c>
       <c r="AE33" s="46" t="n"/>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="AH33" s="46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14°C, Bulutlu, 3 km/sa</t>
         </is>
       </c>
       <c r="AI33" s="46" t="inlineStr">
@@ -5352,13 +5352,13 @@
         </is>
       </c>
       <c r="N34" s="49" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="O34" s="49" t="n">
-        <v>3.2</v>
+        <v>3.6</v>
       </c>
       <c r="P34" s="49" t="n">
-        <v>95.09999999999999</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="Q34" s="50" t="n">
         <v>0.98</v>
@@ -5367,28 +5367,28 @@
         <v>5.5</v>
       </c>
       <c r="S34" s="49" t="n">
-        <v>95.40000000000001</v>
+        <v>95.3</v>
       </c>
       <c r="T34" s="49" t="n">
-        <v>4.6</v>
+        <v>4.7</v>
       </c>
       <c r="U34" s="49" t="n">
-        <v>62.1</v>
+        <v>62.3</v>
       </c>
       <c r="V34" s="49" t="n">
-        <v>37.9</v>
+        <v>37.7</v>
       </c>
       <c r="W34" s="49" t="n">
-        <v>98.8</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="X34" s="49" t="n">
-        <v>4.9</v>
+        <v>5.1</v>
       </c>
       <c r="Y34" s="49" t="n">
-        <v>98.3</v>
+        <v>98.5</v>
       </c>
       <c r="Z34" s="49" t="n">
-        <v>96.8</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="AA34" s="49" t="n">
         <v>4.8</v>
@@ -5493,13 +5493,13 @@
         </is>
       </c>
       <c r="N35" s="49" t="n">
-        <v>10.8</v>
+        <v>10</v>
       </c>
       <c r="O35" s="49" t="n">
-        <v>67.90000000000001</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="P35" s="49" t="n">
-        <v>21.3</v>
+        <v>20.9</v>
       </c>
       <c r="Q35" s="50" t="n">
         <v>0.15</v>
@@ -5514,35 +5514,35 @@
         <v>99</v>
       </c>
       <c r="U35" s="49" t="n">
-        <v>3.4</v>
+        <v>4.1</v>
       </c>
       <c r="V35" s="49" t="n">
-        <v>96.59999999999999</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="W35" s="49" t="n">
-        <v>6.9</v>
+        <v>7.7</v>
       </c>
       <c r="X35" s="49" t="n">
-        <v>78.7</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="Y35" s="49" t="n">
-        <v>89.2</v>
+        <v>90</v>
       </c>
       <c r="Z35" s="49" t="n">
-        <v>32.1</v>
+        <v>30.9</v>
       </c>
       <c r="AA35" s="49" t="n">
         <v>5.8</v>
       </c>
       <c r="AB35" s="49" t="n">
-        <v>83.2</v>
+        <v>83</v>
       </c>
       <c r="AC35" s="49" t="n">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="AD35" s="51" t="inlineStr">
         <is>
-          <t>0-0 (%65)</t>
+          <t>0-0 (%66)</t>
         </is>
       </c>
       <c r="AE35" s="46" t="n"/>
@@ -5634,13 +5634,13 @@
         </is>
       </c>
       <c r="N36" s="49" t="n">
-        <v>9.699999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="O36" s="49" t="n">
-        <v>61.7</v>
+        <v>63.4</v>
       </c>
       <c r="P36" s="49" t="n">
-        <v>28.6</v>
+        <v>27.7</v>
       </c>
       <c r="Q36" s="50" t="n">
         <v>0.15</v>
@@ -5655,35 +5655,35 @@
         <v>98.2</v>
       </c>
       <c r="U36" s="49" t="n">
-        <v>4.5</v>
+        <v>5.4</v>
       </c>
       <c r="V36" s="49" t="n">
-        <v>95.5</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="W36" s="49" t="n">
-        <v>10.3</v>
+        <v>11.1</v>
       </c>
       <c r="X36" s="49" t="n">
-        <v>71.40000000000001</v>
+        <v>72.3</v>
       </c>
       <c r="Y36" s="49" t="n">
-        <v>90.3</v>
+        <v>91.2</v>
       </c>
       <c r="Z36" s="49" t="n">
-        <v>38.3</v>
+        <v>36.6</v>
       </c>
       <c r="AA36" s="49" t="n">
         <v>5.5</v>
       </c>
       <c r="AB36" s="49" t="n">
-        <v>79.3</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="AC36" s="49" t="n">
-        <v>15.2</v>
+        <v>15.1</v>
       </c>
       <c r="AD36" s="51" t="inlineStr">
         <is>
-          <t>0-0 (%58)</t>
+          <t>0-0 (%59)</t>
         </is>
       </c>
       <c r="AE36" s="52" t="n"/>
@@ -5775,52 +5775,52 @@
         </is>
       </c>
       <c r="N37" s="49" t="n">
-        <v>50.6</v>
+        <v>50</v>
       </c>
       <c r="O37" s="49" t="n">
         <v>32.8</v>
       </c>
       <c r="P37" s="49" t="n">
-        <v>16.7</v>
+        <v>17.2</v>
       </c>
       <c r="Q37" s="50" t="n">
         <v>1.11</v>
       </c>
       <c r="R37" s="50" t="n">
-        <v>0.5</v>
+        <v>0.52</v>
       </c>
       <c r="S37" s="49" t="n">
-        <v>21.9</v>
+        <v>22.5</v>
       </c>
       <c r="T37" s="49" t="n">
-        <v>78.09999999999999</v>
+        <v>77.5</v>
       </c>
       <c r="U37" s="49" t="n">
-        <v>26.4</v>
+        <v>27.4</v>
       </c>
       <c r="V37" s="49" t="n">
-        <v>73.59999999999999</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="W37" s="49" t="n">
-        <v>47.8</v>
+        <v>48.7</v>
       </c>
       <c r="X37" s="49" t="n">
-        <v>83.3</v>
+        <v>82.8</v>
       </c>
       <c r="Y37" s="49" t="n">
-        <v>49.4</v>
+        <v>50</v>
       </c>
       <c r="Z37" s="49" t="n">
         <v>67.2</v>
       </c>
       <c r="AA37" s="49" t="n">
-        <v>33</v>
+        <v>32.8</v>
       </c>
       <c r="AB37" s="49" t="n">
-        <v>54.1</v>
+        <v>53.7</v>
       </c>
       <c r="AC37" s="49" t="n">
-        <v>13</v>
+        <v>13.4</v>
       </c>
       <c r="AD37" s="51" t="inlineStr">
         <is>
@@ -5916,52 +5916,52 @@
         </is>
       </c>
       <c r="N38" s="49" t="n">
-        <v>43.6</v>
+        <v>41.6</v>
       </c>
       <c r="O38" s="49" t="n">
-        <v>27.6</v>
+        <v>28.1</v>
       </c>
       <c r="P38" s="49" t="n">
-        <v>28.9</v>
+        <v>30.2</v>
       </c>
       <c r="Q38" s="50" t="n">
-        <v>1.33</v>
+        <v>1.28</v>
       </c>
       <c r="R38" s="50" t="n">
-        <v>1.03</v>
+        <v>1.05</v>
       </c>
       <c r="S38" s="49" t="n">
-        <v>41.9</v>
+        <v>41.1</v>
       </c>
       <c r="T38" s="49" t="n">
-        <v>58.1</v>
+        <v>58.9</v>
       </c>
       <c r="U38" s="49" t="n">
-        <v>47.2</v>
+        <v>47</v>
       </c>
       <c r="V38" s="49" t="n">
-        <v>52.8</v>
+        <v>53</v>
       </c>
       <c r="W38" s="49" t="n">
-        <v>68.2</v>
+        <v>67.7</v>
       </c>
       <c r="X38" s="49" t="n">
-        <v>71.09999999999999</v>
+        <v>69.8</v>
       </c>
       <c r="Y38" s="49" t="n">
-        <v>56.4</v>
+        <v>58.4</v>
       </c>
       <c r="Z38" s="49" t="n">
-        <v>72.40000000000001</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="AA38" s="49" t="n">
-        <v>32</v>
+        <v>30.8</v>
       </c>
       <c r="AB38" s="49" t="n">
-        <v>44.9</v>
+        <v>45.3</v>
       </c>
       <c r="AC38" s="49" t="n">
-        <v>23.1</v>
+        <v>23.9</v>
       </c>
       <c r="AD38" s="51" t="inlineStr">
         <is>
@@ -6057,43 +6057,43 @@
         </is>
       </c>
       <c r="N39" s="49" t="n">
-        <v>81</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="O39" s="49" t="n">
-        <v>12.7</v>
+        <v>12.8</v>
       </c>
       <c r="P39" s="49" t="n">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="Q39" s="50" t="n">
-        <v>2.71</v>
+        <v>2.72</v>
       </c>
       <c r="R39" s="50" t="n">
-        <v>0.63</v>
+        <v>0.64</v>
       </c>
       <c r="S39" s="49" t="n">
-        <v>64.90000000000001</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="T39" s="49" t="n">
-        <v>35.1</v>
+        <v>34.9</v>
       </c>
       <c r="U39" s="49" t="n">
-        <v>43.8</v>
+        <v>44.1</v>
       </c>
       <c r="V39" s="49" t="n">
-        <v>56.2</v>
+        <v>55.9</v>
       </c>
       <c r="W39" s="49" t="n">
-        <v>84.7</v>
+        <v>84.8</v>
       </c>
       <c r="X39" s="49" t="n">
-        <v>93.7</v>
+        <v>93.8</v>
       </c>
       <c r="Y39" s="49" t="n">
-        <v>19</v>
+        <v>19.1</v>
       </c>
       <c r="Z39" s="49" t="n">
-        <v>87.3</v>
+        <v>87.2</v>
       </c>
       <c r="AA39" s="49" t="n">
         <v>60.8</v>
@@ -6198,52 +6198,52 @@
         </is>
       </c>
       <c r="N40" s="49" t="n">
-        <v>34.2</v>
+        <v>33.3</v>
       </c>
       <c r="O40" s="49" t="n">
-        <v>25.3</v>
+        <v>25.6</v>
       </c>
       <c r="P40" s="49" t="n">
-        <v>40.4</v>
+        <v>41.1</v>
       </c>
       <c r="Q40" s="50" t="n">
-        <v>1.32</v>
+        <v>1.29</v>
       </c>
       <c r="R40" s="50" t="n">
         <v>1.46</v>
       </c>
       <c r="S40" s="49" t="n">
-        <v>52.5</v>
+        <v>52</v>
       </c>
       <c r="T40" s="49" t="n">
-        <v>47.5</v>
+        <v>48</v>
       </c>
       <c r="U40" s="49" t="n">
-        <v>56.2</v>
+        <v>55.9</v>
       </c>
       <c r="V40" s="49" t="n">
-        <v>43.8</v>
+        <v>44.1</v>
       </c>
       <c r="W40" s="49" t="n">
-        <v>76.5</v>
+        <v>76.2</v>
       </c>
       <c r="X40" s="49" t="n">
-        <v>59.6</v>
+        <v>58.9</v>
       </c>
       <c r="Y40" s="49" t="n">
-        <v>65.8</v>
+        <v>66.7</v>
       </c>
       <c r="Z40" s="49" t="n">
-        <v>74.7</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="AA40" s="49" t="n">
-        <v>27.6</v>
+        <v>27</v>
       </c>
       <c r="AB40" s="49" t="n">
-        <v>41</v>
+        <v>41.1</v>
       </c>
       <c r="AC40" s="49" t="n">
-        <v>31.5</v>
+        <v>31.9</v>
       </c>
       <c r="AD40" s="51" t="inlineStr">
         <is>
@@ -6339,13 +6339,13 @@
         </is>
       </c>
       <c r="N41" s="49" t="n">
-        <v>25.4</v>
+        <v>22.3</v>
       </c>
       <c r="O41" s="49" t="n">
-        <v>26.9</v>
+        <v>33.2</v>
       </c>
       <c r="P41" s="49" t="n">
-        <v>47.7</v>
+        <v>44.5</v>
       </c>
       <c r="Q41" s="50" t="n">
         <v>0.96</v>
@@ -6360,22 +6360,22 @@
         <v>57.6</v>
       </c>
       <c r="U41" s="49" t="n">
-        <v>46.7</v>
+        <v>49.9</v>
       </c>
       <c r="V41" s="49" t="n">
-        <v>53.3</v>
+        <v>50.1</v>
       </c>
       <c r="W41" s="49" t="n">
-        <v>68.59999999999999</v>
+        <v>71.8</v>
       </c>
       <c r="X41" s="49" t="n">
-        <v>52.3</v>
+        <v>55.5</v>
       </c>
       <c r="Y41" s="49" t="n">
-        <v>74.59999999999999</v>
+        <v>77.7</v>
       </c>
       <c r="Z41" s="49" t="n">
-        <v>73.09999999999999</v>
+        <v>66.8</v>
       </c>
       <c r="AA41" s="49" t="n">
         <v>21</v>
@@ -6388,7 +6388,7 @@
       </c>
       <c r="AD41" s="51" t="inlineStr">
         <is>
-          <t>0-1 (%13)</t>
+          <t>1-1 (%16)</t>
         </is>
       </c>
       <c r="AE41" s="46" t="n"/>
@@ -6480,13 +6480,13 @@
         </is>
       </c>
       <c r="N42" s="49" t="n">
-        <v>99.2</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="O42" s="49" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="P42" s="49" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="Q42" s="50" t="n">
         <v>5.5</v>
@@ -6507,16 +6507,16 @@
         <v>86.09999999999999</v>
       </c>
       <c r="W42" s="49" t="n">
-        <v>97.5</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="X42" s="49" t="n">
-        <v>99.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="Y42" s="49" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="Z42" s="49" t="n">
-        <v>99.3</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="AA42" s="49" t="n">
         <v>90.2</v>
@@ -6621,56 +6621,56 @@
         </is>
       </c>
       <c r="N43" s="49" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="O43" s="49" t="n">
-        <v>22.4</v>
+        <v>27.1</v>
       </c>
       <c r="P43" s="49" t="n">
-        <v>68.7</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="Q43" s="50" t="n">
-        <v>0.43</v>
+        <v>0.44</v>
       </c>
       <c r="R43" s="50" t="n">
-        <v>1.7</v>
+        <v>1.68</v>
       </c>
       <c r="S43" s="49" t="n">
-        <v>35.8</v>
+        <v>35.5</v>
       </c>
       <c r="T43" s="49" t="n">
-        <v>64.2</v>
+        <v>64.5</v>
       </c>
       <c r="U43" s="49" t="n">
-        <v>28.8</v>
+        <v>31.2</v>
       </c>
       <c r="V43" s="49" t="n">
-        <v>71.2</v>
+        <v>68.8</v>
       </c>
       <c r="W43" s="49" t="n">
-        <v>62.8</v>
+        <v>64.7</v>
       </c>
       <c r="X43" s="49" t="n">
-        <v>31.3</v>
+        <v>34.1</v>
       </c>
       <c r="Y43" s="49" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="Z43" s="49" t="n">
-        <v>77.59999999999999</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="AA43" s="49" t="n">
-        <v>8.9</v>
+        <v>9.1</v>
       </c>
       <c r="AB43" s="49" t="n">
-        <v>44.3</v>
+        <v>44.5</v>
       </c>
       <c r="AC43" s="49" t="n">
-        <v>46.8</v>
+        <v>46.4</v>
       </c>
       <c r="AD43" s="51" t="inlineStr">
         <is>
-          <t>0-1 (%20)</t>
+          <t>0-1 (%18)</t>
         </is>
       </c>
       <c r="AE43" s="46" t="n"/>
@@ -6762,13 +6762,13 @@
         </is>
       </c>
       <c r="N44" s="49" t="n">
-        <v>2.7</v>
+        <v>2.5</v>
       </c>
       <c r="O44" s="49" t="n">
-        <v>4.2</v>
+        <v>4.6</v>
       </c>
       <c r="P44" s="49" t="n">
-        <v>93.09999999999999</v>
+        <v>92.8</v>
       </c>
       <c r="Q44" s="50" t="n">
         <v>1.26</v>
@@ -6777,10 +6777,10 @@
         <v>5.5</v>
       </c>
       <c r="S44" s="49" t="n">
-        <v>96.3</v>
+        <v>96.2</v>
       </c>
       <c r="T44" s="49" t="n">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="U44" s="49" t="n">
         <v>71.40000000000001</v>
@@ -6789,16 +6789,16 @@
         <v>28.6</v>
       </c>
       <c r="W44" s="49" t="n">
-        <v>99.09999999999999</v>
+        <v>99.2</v>
       </c>
       <c r="X44" s="49" t="n">
-        <v>6.9</v>
+        <v>7.2</v>
       </c>
       <c r="Y44" s="49" t="n">
-        <v>97.3</v>
+        <v>97.5</v>
       </c>
       <c r="Z44" s="49" t="n">
-        <v>95.8</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="AA44" s="49" t="n">
         <v>6.5</v>
@@ -6807,7 +6807,7 @@
         <v>14.2</v>
       </c>
       <c r="AC44" s="49" t="n">
-        <v>79.2</v>
+        <v>79.3</v>
       </c>
       <c r="AD44" s="51" t="inlineStr">
         <is>
@@ -6903,13 +6903,13 @@
         </is>
       </c>
       <c r="N45" s="49" t="n">
-        <v>97.7</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="O45" s="49" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="P45" s="49" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="Q45" s="50" t="n">
         <v>5.5</v>
@@ -6930,16 +6930,16 @@
         <v>58.5</v>
       </c>
       <c r="W45" s="49" t="n">
-        <v>98.2</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="X45" s="49" t="n">
-        <v>99.40000000000001</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="Y45" s="49" t="n">
-        <v>2.3</v>
+        <v>2.6</v>
       </c>
       <c r="Z45" s="49" t="n">
-        <v>98.2</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="AA45" s="49" t="n">
         <v>86.40000000000001</v>
@@ -7044,13 +7044,13 @@
         </is>
       </c>
       <c r="N46" s="49" t="n">
-        <v>10.3</v>
+        <v>8.9</v>
       </c>
       <c r="O46" s="49" t="n">
-        <v>47.3</v>
+        <v>50.4</v>
       </c>
       <c r="P46" s="49" t="n">
-        <v>42.3</v>
+        <v>40.7</v>
       </c>
       <c r="Q46" s="50" t="n">
         <v>0.21</v>
@@ -7065,35 +7065,35 @@
         <v>94</v>
       </c>
       <c r="U46" s="49" t="n">
-        <v>9.300000000000001</v>
+        <v>10.7</v>
       </c>
       <c r="V46" s="49" t="n">
-        <v>90.7</v>
+        <v>89.3</v>
       </c>
       <c r="W46" s="49" t="n">
-        <v>22.2</v>
+        <v>23.5</v>
       </c>
       <c r="X46" s="49" t="n">
-        <v>57.7</v>
+        <v>59.3</v>
       </c>
       <c r="Y46" s="49" t="n">
-        <v>89.7</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="Z46" s="49" t="n">
-        <v>52.7</v>
+        <v>49.6</v>
       </c>
       <c r="AA46" s="49" t="n">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="AB46" s="49" t="n">
-        <v>69.09999999999999</v>
+        <v>69.2</v>
       </c>
       <c r="AC46" s="49" t="n">
-        <v>24.1</v>
+        <v>24</v>
       </c>
       <c r="AD46" s="51" t="inlineStr">
         <is>
-          <t>0-0 (%41)</t>
+          <t>0-0 (%43)</t>
         </is>
       </c>
       <c r="AE46" s="52" t="n"/>
@@ -7185,56 +7185,56 @@
         </is>
       </c>
       <c r="N47" s="49" t="n">
-        <v>49.7</v>
+        <v>46.9</v>
       </c>
       <c r="O47" s="49" t="n">
-        <v>33.9</v>
+        <v>39.4</v>
       </c>
       <c r="P47" s="49" t="n">
-        <v>16.5</v>
+        <v>13.7</v>
       </c>
       <c r="Q47" s="50" t="n">
-        <v>1.06</v>
+        <v>1.05</v>
       </c>
       <c r="R47" s="50" t="n">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
       <c r="S47" s="49" t="n">
-        <v>20</v>
+        <v>19.8</v>
       </c>
       <c r="T47" s="49" t="n">
-        <v>80</v>
+        <v>80.2</v>
       </c>
       <c r="U47" s="49" t="n">
-        <v>24.7</v>
+        <v>27.3</v>
       </c>
       <c r="V47" s="49" t="n">
-        <v>75.3</v>
+        <v>72.7</v>
       </c>
       <c r="W47" s="49" t="n">
-        <v>45.4</v>
+        <v>47.8</v>
       </c>
       <c r="X47" s="49" t="n">
-        <v>83.5</v>
+        <v>86.3</v>
       </c>
       <c r="Y47" s="49" t="n">
-        <v>50.3</v>
+        <v>53.1</v>
       </c>
       <c r="Z47" s="49" t="n">
-        <v>66.09999999999999</v>
+        <v>60.6</v>
       </c>
       <c r="AA47" s="49" t="n">
         <v>32</v>
       </c>
       <c r="AB47" s="49" t="n">
-        <v>55.4</v>
+        <v>55.5</v>
       </c>
       <c r="AC47" s="49" t="n">
-        <v>12.6</v>
+        <v>12.5</v>
       </c>
       <c r="AD47" s="51" t="inlineStr">
         <is>
-          <t>1-0 (%23)</t>
+          <t>0-0 (%24)</t>
         </is>
       </c>
       <c r="AE47" s="46" t="n"/>
@@ -7326,56 +7326,56 @@
         </is>
       </c>
       <c r="N48" s="49" t="n">
-        <v>11.6</v>
+        <v>9.4</v>
       </c>
       <c r="O48" s="49" t="n">
-        <v>20.5</v>
+        <v>25.4</v>
       </c>
       <c r="P48" s="49" t="n">
-        <v>67.8</v>
+        <v>65.2</v>
       </c>
       <c r="Q48" s="50" t="n">
         <v>0.65</v>
       </c>
       <c r="R48" s="50" t="n">
-        <v>1.93</v>
+        <v>1.92</v>
       </c>
       <c r="S48" s="49" t="n">
-        <v>47.4</v>
+        <v>47.3</v>
       </c>
       <c r="T48" s="49" t="n">
-        <v>52.6</v>
+        <v>52.7</v>
       </c>
       <c r="U48" s="49" t="n">
-        <v>40.6</v>
+        <v>43.1</v>
       </c>
       <c r="V48" s="49" t="n">
-        <v>59.4</v>
+        <v>56.9</v>
       </c>
       <c r="W48" s="49" t="n">
-        <v>72.7</v>
+        <v>75</v>
       </c>
       <c r="X48" s="49" t="n">
-        <v>32.2</v>
+        <v>34.8</v>
       </c>
       <c r="Y48" s="49" t="n">
-        <v>88.40000000000001</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="Z48" s="49" t="n">
-        <v>79.5</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="AA48" s="49" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="AB48" s="49" t="n">
-        <v>39.9</v>
+        <v>40</v>
       </c>
       <c r="AC48" s="49" t="n">
-        <v>48.2</v>
+        <v>48</v>
       </c>
       <c r="AD48" s="51" t="inlineStr">
         <is>
-          <t>0-1 (%15)</t>
+          <t>0-2 (%14)</t>
         </is>
       </c>
       <c r="AE48" s="52" t="n"/>
@@ -7461,62 +7461,62 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M49" s="48" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="M49" s="55" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
       <c r="N49" s="49" t="n">
-        <v>18.3</v>
+        <v>15.9</v>
       </c>
       <c r="O49" s="49" t="n">
-        <v>39.7</v>
+        <v>44.7</v>
       </c>
       <c r="P49" s="49" t="n">
-        <v>42</v>
+        <v>39.3</v>
       </c>
       <c r="Q49" s="50" t="n">
-        <v>0.43</v>
+        <v>0.44</v>
       </c>
       <c r="R49" s="50" t="n">
         <v>0.82</v>
       </c>
       <c r="S49" s="49" t="n">
-        <v>13.2</v>
+        <v>13.3</v>
       </c>
       <c r="T49" s="49" t="n">
-        <v>86.8</v>
+        <v>86.7</v>
       </c>
       <c r="U49" s="49" t="n">
-        <v>19.7</v>
+        <v>22.5</v>
       </c>
       <c r="V49" s="49" t="n">
-        <v>80.3</v>
+        <v>77.5</v>
       </c>
       <c r="W49" s="49" t="n">
-        <v>35.6</v>
+        <v>38.4</v>
       </c>
       <c r="X49" s="49" t="n">
-        <v>58</v>
+        <v>60.7</v>
       </c>
       <c r="Y49" s="49" t="n">
-        <v>81.7</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="Z49" s="49" t="n">
-        <v>60.3</v>
+        <v>55.3</v>
       </c>
       <c r="AA49" s="49" t="n">
-        <v>12.7</v>
+        <v>12.9</v>
       </c>
       <c r="AB49" s="49" t="n">
-        <v>61.1</v>
+        <v>61</v>
       </c>
       <c r="AC49" s="49" t="n">
-        <v>26.2</v>
+        <v>26.1</v>
       </c>
       <c r="AD49" s="51" t="inlineStr">
         <is>
-          <t>0-0 (%29)</t>
+          <t>0-0 (%31)</t>
         </is>
       </c>
       <c r="AE49" s="46" t="n"/>
@@ -7608,13 +7608,13 @@
         </is>
       </c>
       <c r="N50" s="49" t="n">
-        <v>99.2</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="O50" s="49" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="P50" s="49" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="Q50" s="50" t="n">
         <v>5.5</v>
@@ -7635,16 +7635,16 @@
         <v>86.09999999999999</v>
       </c>
       <c r="W50" s="49" t="n">
-        <v>97.5</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="X50" s="49" t="n">
-        <v>99.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="Y50" s="49" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="Z50" s="49" t="n">
-        <v>99.3</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="AA50" s="49" t="n">
         <v>90.2</v>
@@ -7749,52 +7749,52 @@
         </is>
       </c>
       <c r="N51" s="49" t="n">
-        <v>36.2</v>
+        <v>35.8</v>
       </c>
       <c r="O51" s="49" t="n">
-        <v>26.5</v>
+        <v>26.6</v>
       </c>
       <c r="P51" s="49" t="n">
-        <v>37.3</v>
+        <v>37.6</v>
       </c>
       <c r="Q51" s="50" t="n">
-        <v>1.28</v>
+        <v>1.26</v>
       </c>
       <c r="R51" s="50" t="n">
         <v>1.3</v>
       </c>
       <c r="S51" s="49" t="n">
-        <v>47.5</v>
+        <v>47.1</v>
       </c>
       <c r="T51" s="49" t="n">
-        <v>52.5</v>
+        <v>52.9</v>
       </c>
       <c r="U51" s="49" t="n">
-        <v>52.4</v>
+        <v>52.1</v>
       </c>
       <c r="V51" s="49" t="n">
-        <v>47.6</v>
+        <v>47.9</v>
       </c>
       <c r="W51" s="49" t="n">
-        <v>72.8</v>
+        <v>72.5</v>
       </c>
       <c r="X51" s="49" t="n">
-        <v>62.7</v>
+        <v>62.4</v>
       </c>
       <c r="Y51" s="49" t="n">
-        <v>63.8</v>
+        <v>64.2</v>
       </c>
       <c r="Z51" s="49" t="n">
-        <v>73.5</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="AA51" s="49" t="n">
-        <v>27.7</v>
+        <v>27.4</v>
       </c>
       <c r="AB51" s="49" t="n">
-        <v>43.9</v>
+        <v>44</v>
       </c>
       <c r="AC51" s="49" t="n">
-        <v>28.4</v>
+        <v>28.5</v>
       </c>
       <c r="AD51" s="51" t="inlineStr">
         <is>
@@ -7899,7 +7899,7 @@
         <v>4.7</v>
       </c>
       <c r="Q52" s="50" t="n">
-        <v>3.53</v>
+        <v>3.52</v>
       </c>
       <c r="R52" s="50" t="n">
         <v>0.8</v>
@@ -7929,7 +7929,7 @@
         <v>91.3</v>
       </c>
       <c r="AA52" s="49" t="n">
-        <v>67.3</v>
+        <v>67.2</v>
       </c>
       <c r="AB52" s="49" t="n">
         <v>24.7</v>
@@ -8031,13 +8031,13 @@
         </is>
       </c>
       <c r="N53" s="49" t="n">
-        <v>33.7</v>
+        <v>33.8</v>
       </c>
       <c r="O53" s="49" t="n">
         <v>25.6</v>
       </c>
       <c r="P53" s="49" t="n">
-        <v>40.8</v>
+        <v>40.6</v>
       </c>
       <c r="Q53" s="50" t="n">
         <v>1.29</v>
@@ -8046,25 +8046,25 @@
         <v>1.44</v>
       </c>
       <c r="S53" s="49" t="n">
-        <v>51.4</v>
+        <v>51.2</v>
       </c>
       <c r="T53" s="49" t="n">
-        <v>48.6</v>
+        <v>48.8</v>
       </c>
       <c r="U53" s="49" t="n">
-        <v>55.3</v>
+        <v>55.2</v>
       </c>
       <c r="V53" s="49" t="n">
-        <v>44.7</v>
+        <v>44.8</v>
       </c>
       <c r="W53" s="49" t="n">
-        <v>75.7</v>
+        <v>75.5</v>
       </c>
       <c r="X53" s="49" t="n">
-        <v>59.2</v>
+        <v>59.4</v>
       </c>
       <c r="Y53" s="49" t="n">
-        <v>66.3</v>
+        <v>66.2</v>
       </c>
       <c r="Z53" s="49" t="n">
         <v>74.40000000000001</v>
@@ -8076,7 +8076,7 @@
         <v>42.4</v>
       </c>
       <c r="AC53" s="49" t="n">
-        <v>31</v>
+        <v>30.8</v>
       </c>
       <c r="AD53" s="51" t="inlineStr">
         <is>
@@ -8172,52 +8172,52 @@
         </is>
       </c>
       <c r="N54" s="49" t="n">
-        <v>55.3</v>
+        <v>55</v>
       </c>
       <c r="O54" s="49" t="n">
         <v>20.6</v>
       </c>
       <c r="P54" s="49" t="n">
-        <v>24.2</v>
+        <v>24.4</v>
       </c>
       <c r="Q54" s="50" t="n">
-        <v>2.16</v>
+        <v>2.15</v>
       </c>
       <c r="R54" s="50" t="n">
-        <v>1.38</v>
+        <v>1.39</v>
       </c>
       <c r="S54" s="49" t="n">
-        <v>68.59999999999999</v>
+        <v>68.7</v>
       </c>
       <c r="T54" s="49" t="n">
-        <v>31.4</v>
+        <v>31.3</v>
       </c>
       <c r="U54" s="49" t="n">
-        <v>66.2</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="V54" s="49" t="n">
-        <v>33.8</v>
+        <v>33.6</v>
       </c>
       <c r="W54" s="49" t="n">
-        <v>86.8</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="X54" s="49" t="n">
-        <v>75.8</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="Y54" s="49" t="n">
-        <v>44.7</v>
+        <v>45</v>
       </c>
       <c r="Z54" s="49" t="n">
         <v>79.40000000000001</v>
       </c>
       <c r="AA54" s="49" t="n">
-        <v>42</v>
+        <v>41.8</v>
       </c>
       <c r="AB54" s="49" t="n">
         <v>35.5</v>
       </c>
       <c r="AC54" s="49" t="n">
-        <v>22.5</v>
+        <v>22.7</v>
       </c>
       <c r="AD54" s="51" t="inlineStr">
         <is>
@@ -8316,49 +8316,49 @@
         <v>7.7</v>
       </c>
       <c r="O55" s="49" t="n">
-        <v>18.3</v>
+        <v>18.1</v>
       </c>
       <c r="P55" s="49" t="n">
-        <v>74</v>
+        <v>74.2</v>
       </c>
       <c r="Q55" s="50" t="n">
         <v>0.49</v>
       </c>
       <c r="R55" s="50" t="n">
-        <v>2.03</v>
+        <v>2.04</v>
       </c>
       <c r="S55" s="49" t="n">
-        <v>46</v>
+        <v>46.4</v>
       </c>
       <c r="T55" s="49" t="n">
-        <v>54</v>
+        <v>53.6</v>
       </c>
       <c r="U55" s="49" t="n">
-        <v>33.4</v>
+        <v>33.5</v>
       </c>
       <c r="V55" s="49" t="n">
-        <v>66.59999999999999</v>
+        <v>66.5</v>
       </c>
       <c r="W55" s="49" t="n">
-        <v>71.5</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="X55" s="49" t="n">
-        <v>26</v>
+        <v>25.8</v>
       </c>
       <c r="Y55" s="49" t="n">
         <v>92.3</v>
       </c>
       <c r="Z55" s="49" t="n">
-        <v>81.7</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="AA55" s="49" t="n">
         <v>8.6</v>
       </c>
       <c r="AB55" s="49" t="n">
-        <v>40.3</v>
+        <v>40.1</v>
       </c>
       <c r="AC55" s="49" t="n">
-        <v>51.1</v>
+        <v>51.4</v>
       </c>
       <c r="AD55" s="51" t="inlineStr">
         <is>
@@ -8432,7 +8432,7 @@
     <row r="3">
       <c r="A3" s="57" t="inlineStr">
         <is>
-          <t>Oluşturulma zamanı: 05.10.2026 02:00</t>
+          <t>Oluşturulma zamanı: 05.10.2026 02:56</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Güncel tahmin tablosu: 3-7 Ekim maçları (48 satır)
football-data.org rate limit nedeniyle bu çalıştırmada CL, DED, PPL,
BSA, ELC verisi eksik kaldı (429), bu yüzden 53 -> 48 satır.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBfpyxGus5xRHHn8xK9mQE
</commit_message>
<xml_diff>
--- a/maclar_ve_tahminler.xlsx
+++ b/maclar_ve_tahminler.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bilgi" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Maçlar ve Tahminler'!$A$2:$AI$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Maçlar ve Tahminler'!$A$2:$AI$50</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -349,10 +349,10 @@
     <xf numFmtId="0" fontId="4" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -722,7 +722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI55"/>
+  <dimension ref="A1:AI50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1075,52 +1075,52 @@
         </is>
       </c>
       <c r="N3" s="37" t="n">
-        <v>68.90000000000001</v>
+        <v>68.5</v>
       </c>
       <c r="O3" s="37" t="n">
-        <v>15.8</v>
+        <v>15.9</v>
       </c>
       <c r="P3" s="37" t="n">
-        <v>15.3</v>
+        <v>15.6</v>
       </c>
       <c r="Q3" s="38" t="n">
-        <v>2.85</v>
+        <v>2.83</v>
       </c>
       <c r="R3" s="38" t="n">
         <v>1.33</v>
       </c>
       <c r="S3" s="37" t="n">
-        <v>78.59999999999999</v>
+        <v>78.5</v>
       </c>
       <c r="T3" s="37" t="n">
-        <v>21.4</v>
+        <v>21.5</v>
       </c>
       <c r="U3" s="37" t="n">
-        <v>69.2</v>
+        <v>69.3</v>
       </c>
       <c r="V3" s="37" t="n">
-        <v>30.8</v>
+        <v>30.7</v>
       </c>
       <c r="W3" s="37" t="n">
-        <v>92.09999999999999</v>
+        <v>92</v>
       </c>
       <c r="X3" s="37" t="n">
-        <v>84.7</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="Y3" s="37" t="n">
-        <v>31.1</v>
+        <v>31.5</v>
       </c>
       <c r="Z3" s="37" t="n">
-        <v>84.2</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="AA3" s="37" t="n">
-        <v>53.3</v>
+        <v>53</v>
       </c>
       <c r="AB3" s="37" t="n">
-        <v>29.4</v>
+        <v>29.5</v>
       </c>
       <c r="AC3" s="37" t="n">
-        <v>17.3</v>
+        <v>17.5</v>
       </c>
       <c r="AD3" s="34" t="inlineStr">
         <is>
@@ -1212,19 +1212,19 @@
         </is>
       </c>
       <c r="N4" s="37" t="n">
-        <v>56.5</v>
+        <v>56.3</v>
       </c>
       <c r="O4" s="37" t="n">
-        <v>19.7</v>
+        <v>19.6</v>
       </c>
       <c r="P4" s="37" t="n">
-        <v>23.9</v>
+        <v>24.1</v>
       </c>
       <c r="Q4" s="38" t="n">
-        <v>2.32</v>
+        <v>2.31</v>
       </c>
       <c r="R4" s="38" t="n">
-        <v>1.47</v>
+        <v>1.48</v>
       </c>
       <c r="S4" s="37" t="n">
         <v>72.90000000000001</v>
@@ -1242,22 +1242,22 @@
         <v>89.09999999999999</v>
       </c>
       <c r="X4" s="37" t="n">
-        <v>76.09999999999999</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="Y4" s="37" t="n">
-        <v>43.5</v>
+        <v>43.7</v>
       </c>
       <c r="Z4" s="37" t="n">
-        <v>80.3</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="AA4" s="37" t="n">
-        <v>44</v>
+        <v>43.8</v>
       </c>
       <c r="AB4" s="37" t="n">
         <v>33.1</v>
       </c>
       <c r="AC4" s="37" t="n">
-        <v>22.9</v>
+        <v>23</v>
       </c>
       <c r="AD4" s="34" t="inlineStr">
         <is>
@@ -2034,25 +2034,25 @@
         </is>
       </c>
       <c r="N10" s="37" t="n">
-        <v>59.1</v>
+        <v>58.9</v>
       </c>
       <c r="O10" s="37" t="n">
-        <v>28.3</v>
+        <v>28.4</v>
       </c>
       <c r="P10" s="37" t="n">
-        <v>12.5</v>
+        <v>12.8</v>
       </c>
       <c r="Q10" s="38" t="n">
-        <v>1.36</v>
+        <v>1.35</v>
       </c>
       <c r="R10" s="38" t="n">
         <v>0.47</v>
       </c>
       <c r="S10" s="37" t="n">
-        <v>27.6</v>
+        <v>27.4</v>
       </c>
       <c r="T10" s="37" t="n">
-        <v>72.40000000000001</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="U10" s="37" t="n">
         <v>27.8</v>
@@ -2061,25 +2061,25 @@
         <v>72.2</v>
       </c>
       <c r="W10" s="37" t="n">
-        <v>54.6</v>
+        <v>54.4</v>
       </c>
       <c r="X10" s="37" t="n">
-        <v>87.5</v>
+        <v>87.2</v>
       </c>
       <c r="Y10" s="37" t="n">
-        <v>40.9</v>
+        <v>41.1</v>
       </c>
       <c r="Z10" s="37" t="n">
-        <v>71.7</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="AA10" s="37" t="n">
-        <v>39.3</v>
+        <v>39</v>
       </c>
       <c r="AB10" s="37" t="n">
-        <v>49.8</v>
+        <v>49.9</v>
       </c>
       <c r="AC10" s="37" t="n">
-        <v>10.9</v>
+        <v>11</v>
       </c>
       <c r="AD10" s="34" t="inlineStr">
         <is>
@@ -2582,49 +2582,49 @@
         </is>
       </c>
       <c r="N14" s="37" t="n">
-        <v>46.4</v>
+        <v>46.1</v>
       </c>
       <c r="O14" s="37" t="n">
-        <v>41.1</v>
+        <v>41.3</v>
       </c>
       <c r="P14" s="37" t="n">
-        <v>12.5</v>
+        <v>12.6</v>
       </c>
       <c r="Q14" s="38" t="n">
-        <v>0.83</v>
+        <v>0.82</v>
       </c>
       <c r="R14" s="38" t="n">
         <v>0.29</v>
       </c>
       <c r="S14" s="37" t="n">
-        <v>10.4</v>
+        <v>10.2</v>
       </c>
       <c r="T14" s="37" t="n">
-        <v>89.59999999999999</v>
+        <v>89.8</v>
       </c>
       <c r="U14" s="37" t="n">
-        <v>14.4</v>
+        <v>14.3</v>
       </c>
       <c r="V14" s="37" t="n">
-        <v>85.59999999999999</v>
+        <v>85.7</v>
       </c>
       <c r="W14" s="37" t="n">
-        <v>30.9</v>
+        <v>30.6</v>
       </c>
       <c r="X14" s="37" t="n">
-        <v>87.5</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="Y14" s="37" t="n">
-        <v>53.6</v>
+        <v>53.9</v>
       </c>
       <c r="Z14" s="37" t="n">
-        <v>58.9</v>
+        <v>58.7</v>
       </c>
       <c r="AA14" s="37" t="n">
-        <v>27.8</v>
+        <v>27.6</v>
       </c>
       <c r="AB14" s="37" t="n">
-        <v>63.4</v>
+        <v>63.6</v>
       </c>
       <c r="AC14" s="37" t="n">
         <v>8.800000000000001</v>
@@ -2719,52 +2719,52 @@
         </is>
       </c>
       <c r="N15" s="37" t="n">
-        <v>45.6</v>
+        <v>45.4</v>
       </c>
       <c r="O15" s="37" t="n">
-        <v>31.4</v>
+        <v>31.3</v>
       </c>
       <c r="P15" s="37" t="n">
-        <v>23</v>
+        <v>23.3</v>
       </c>
       <c r="Q15" s="38" t="n">
-        <v>1.14</v>
+        <v>1.13</v>
       </c>
       <c r="R15" s="38" t="n">
         <v>0.72</v>
       </c>
       <c r="S15" s="37" t="n">
-        <v>28.3</v>
+        <v>28.2</v>
       </c>
       <c r="T15" s="37" t="n">
-        <v>71.7</v>
+        <v>71.8</v>
       </c>
       <c r="U15" s="37" t="n">
-        <v>34.7</v>
+        <v>34.6</v>
       </c>
       <c r="V15" s="37" t="n">
-        <v>65.3</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="W15" s="37" t="n">
-        <v>55.3</v>
+        <v>55.1</v>
       </c>
       <c r="X15" s="37" t="n">
-        <v>77</v>
+        <v>76.7</v>
       </c>
       <c r="Y15" s="37" t="n">
-        <v>54.4</v>
+        <v>54.6</v>
       </c>
       <c r="Z15" s="37" t="n">
-        <v>68.59999999999999</v>
+        <v>68.7</v>
       </c>
       <c r="AA15" s="37" t="n">
-        <v>31.3</v>
+        <v>31.1</v>
       </c>
       <c r="AB15" s="37" t="n">
-        <v>50.9</v>
+        <v>51</v>
       </c>
       <c r="AC15" s="37" t="n">
-        <v>17.8</v>
+        <v>17.9</v>
       </c>
       <c r="AD15" s="34" t="inlineStr">
         <is>
@@ -2806,27 +2806,27 @@
       </c>
       <c r="C16" s="34" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D16" s="34" t="inlineStr">
         <is>
-          <t>Brezilya</t>
+          <t>Avrupa</t>
         </is>
       </c>
       <c r="E16" s="34" t="inlineStr">
         <is>
-          <t>Campeonato Brasileiro Série A</t>
+          <t>UEFA Uluslar Ligi</t>
         </is>
       </c>
       <c r="F16" s="35" t="inlineStr">
         <is>
-          <t>CA Mineiro</t>
+          <t>Azerbaijan</t>
         </is>
       </c>
       <c r="G16" s="35" t="inlineStr">
         <is>
-          <t>RB Bragantino</t>
+          <t>Lithuania</t>
         </is>
       </c>
       <c r="H16" s="34" t="inlineStr">
@@ -2834,11 +2834,15 @@
           <t>Bitti</t>
         </is>
       </c>
-      <c r="I16" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="J16" s="34" t="n">
-        <v>0</v>
+      <c r="I16" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J16" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K16" s="34" t="n">
         <v>1</v>
@@ -2846,62 +2850,62 @@
       <c r="L16" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="M16" s="36" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="M16" s="39" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
       <c r="N16" s="37" t="n">
-        <v>69.40000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="O16" s="37" t="n">
-        <v>17.3</v>
+        <v>51.5</v>
       </c>
       <c r="P16" s="37" t="n">
-        <v>13.2</v>
+        <v>38.6</v>
       </c>
       <c r="Q16" s="38" t="n">
-        <v>2.42</v>
+        <v>0.22</v>
       </c>
       <c r="R16" s="38" t="n">
-        <v>0.97</v>
+        <v>0.64</v>
       </c>
       <c r="S16" s="37" t="n">
-        <v>65.8</v>
+        <v>5.7</v>
       </c>
       <c r="T16" s="37" t="n">
-        <v>34.2</v>
+        <v>94.3</v>
       </c>
       <c r="U16" s="37" t="n">
-        <v>56.4</v>
+        <v>11</v>
       </c>
       <c r="V16" s="37" t="n">
-        <v>43.6</v>
+        <v>89</v>
       </c>
       <c r="W16" s="37" t="n">
-        <v>85.2</v>
+        <v>22.9</v>
       </c>
       <c r="X16" s="37" t="n">
-        <v>86.8</v>
+        <v>61.4</v>
       </c>
       <c r="Y16" s="37" t="n">
-        <v>30.6</v>
+        <v>90.2</v>
       </c>
       <c r="Z16" s="37" t="n">
-        <v>82.7</v>
+        <v>48.5</v>
       </c>
       <c r="AA16" s="37" t="n">
-        <v>50.7</v>
+        <v>7.3</v>
       </c>
       <c r="AB16" s="37" t="n">
-        <v>34.7</v>
+        <v>69.8</v>
       </c>
       <c r="AC16" s="37" t="n">
-        <v>14.6</v>
+        <v>22.9</v>
       </c>
       <c r="AD16" s="34" t="inlineStr">
         <is>
-          <t>2-0 (%10)</t>
+          <t>0-0 (%44)</t>
         </is>
       </c>
       <c r="AE16" s="34" t="n"/>
@@ -2939,7 +2943,7 @@
       </c>
       <c r="C17" s="34" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D17" s="34" t="inlineStr">
@@ -2954,12 +2958,12 @@
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Azerbaijan</t>
+          <t>Kosovo</t>
         </is>
       </c>
       <c r="G17" s="35" t="inlineStr">
         <is>
-          <t>Lithuania</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="H17" s="34" t="inlineStr">
@@ -2981,64 +2985,64 @@
         <v>1</v>
       </c>
       <c r="L17" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" s="39" t="inlineStr">
-        <is>
-          <t>X</t>
+        <v>1</v>
+      </c>
+      <c r="M17" s="40" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
       <c r="N17" s="37" t="n">
-        <v>9.800000000000001</v>
+        <v>10.3</v>
       </c>
       <c r="O17" s="37" t="n">
-        <v>51.5</v>
+        <v>21.7</v>
       </c>
       <c r="P17" s="37" t="n">
-        <v>38.6</v>
+        <v>68</v>
       </c>
       <c r="Q17" s="38" t="n">
-        <v>0.22</v>
+        <v>0.87</v>
       </c>
       <c r="R17" s="38" t="n">
-        <v>0.64</v>
+        <v>2.33</v>
       </c>
       <c r="S17" s="37" t="n">
-        <v>5.7</v>
+        <v>61.9</v>
       </c>
       <c r="T17" s="37" t="n">
-        <v>94.3</v>
+        <v>38.1</v>
       </c>
       <c r="U17" s="37" t="n">
-        <v>11</v>
+        <v>54.4</v>
       </c>
       <c r="V17" s="37" t="n">
-        <v>89</v>
+        <v>45.6</v>
       </c>
       <c r="W17" s="37" t="n">
-        <v>22.9</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="X17" s="37" t="n">
-        <v>61.4</v>
+        <v>32</v>
       </c>
       <c r="Y17" s="37" t="n">
-        <v>90.2</v>
+        <v>89.7</v>
       </c>
       <c r="Z17" s="37" t="n">
-        <v>48.5</v>
+        <v>78.3</v>
       </c>
       <c r="AA17" s="37" t="n">
-        <v>7.3</v>
+        <v>13.6</v>
       </c>
       <c r="AB17" s="37" t="n">
-        <v>69.8</v>
+        <v>34.5</v>
       </c>
       <c r="AC17" s="37" t="n">
-        <v>22.9</v>
+        <v>51.9</v>
       </c>
       <c r="AD17" s="34" t="inlineStr">
         <is>
-          <t>0-0 (%44)</t>
+          <t>0-2 (%11)</t>
         </is>
       </c>
       <c r="AE17" s="34" t="n"/>
@@ -3091,12 +3095,12 @@
       </c>
       <c r="F18" s="35" t="inlineStr">
         <is>
-          <t>Kosovo</t>
+          <t>Malta</t>
         </is>
       </c>
       <c r="G18" s="35" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Andorra</t>
         </is>
       </c>
       <c r="H18" s="34" t="inlineStr">
@@ -3118,64 +3122,64 @@
         <v>1</v>
       </c>
       <c r="L18" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="M18" s="40" t="inlineStr">
-        <is>
-          <t>2</t>
+        <v>0</v>
+      </c>
+      <c r="M18" s="36" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
       <c r="N18" s="37" t="n">
-        <v>10.3</v>
+        <v>58.3</v>
       </c>
       <c r="O18" s="37" t="n">
-        <v>21.7</v>
+        <v>32.6</v>
       </c>
       <c r="P18" s="37" t="n">
-        <v>68</v>
+        <v>9.1</v>
       </c>
       <c r="Q18" s="38" t="n">
-        <v>0.87</v>
+        <v>1.37</v>
       </c>
       <c r="R18" s="38" t="n">
-        <v>2.33</v>
+        <v>0.43</v>
       </c>
       <c r="S18" s="37" t="n">
-        <v>61.9</v>
+        <v>27.1</v>
       </c>
       <c r="T18" s="37" t="n">
-        <v>38.1</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="U18" s="37" t="n">
-        <v>54.4</v>
+        <v>28.6</v>
       </c>
       <c r="V18" s="37" t="n">
-        <v>45.6</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="W18" s="37" t="n">
-        <v>84.90000000000001</v>
+        <v>56.3</v>
       </c>
       <c r="X18" s="37" t="n">
-        <v>32</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="Y18" s="37" t="n">
-        <v>89.7</v>
+        <v>41.7</v>
       </c>
       <c r="Z18" s="37" t="n">
-        <v>78.3</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="AA18" s="37" t="n">
-        <v>13.6</v>
+        <v>40.1</v>
       </c>
       <c r="AB18" s="37" t="n">
-        <v>34.5</v>
+        <v>49.9</v>
       </c>
       <c r="AC18" s="37" t="n">
-        <v>51.9</v>
+        <v>10.1</v>
       </c>
       <c r="AD18" s="34" t="inlineStr">
         <is>
-          <t>0-2 (%11)</t>
+          <t>1-0 (%20)</t>
         </is>
       </c>
       <c r="AE18" s="34" t="n"/>
@@ -3213,27 +3217,27 @@
       </c>
       <c r="C19" s="34" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="D19" s="34" t="inlineStr">
         <is>
-          <t>Avrupa</t>
+          <t>Arjantin</t>
         </is>
       </c>
       <c r="E19" s="34" t="inlineStr">
         <is>
-          <t>UEFA Uluslar Ligi</t>
+          <t>Liga Profesional (Arjantin)</t>
         </is>
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Malta</t>
+          <t>Huracan</t>
         </is>
       </c>
       <c r="G19" s="35" t="inlineStr">
         <is>
-          <t>Andorra</t>
+          <t>Aldosivi</t>
         </is>
       </c>
       <c r="H19" s="34" t="inlineStr">
@@ -3263,56 +3267,56 @@
         </is>
       </c>
       <c r="N19" s="37" t="n">
-        <v>58.3</v>
+        <v>62.7</v>
       </c>
       <c r="O19" s="37" t="n">
-        <v>32.6</v>
+        <v>22.5</v>
       </c>
       <c r="P19" s="37" t="n">
-        <v>9.1</v>
+        <v>14.8</v>
       </c>
       <c r="Q19" s="38" t="n">
-        <v>1.37</v>
+        <v>1.82</v>
       </c>
       <c r="R19" s="38" t="n">
-        <v>0.43</v>
+        <v>0.75</v>
       </c>
       <c r="S19" s="37" t="n">
-        <v>27.1</v>
+        <v>47.4</v>
       </c>
       <c r="T19" s="37" t="n">
-        <v>72.90000000000001</v>
+        <v>52.6</v>
       </c>
       <c r="U19" s="37" t="n">
-        <v>28.6</v>
+        <v>44.3</v>
       </c>
       <c r="V19" s="37" t="n">
-        <v>71.40000000000001</v>
+        <v>55.7</v>
       </c>
       <c r="W19" s="37" t="n">
-        <v>56.3</v>
+        <v>72.8</v>
       </c>
       <c r="X19" s="37" t="n">
-        <v>90.90000000000001</v>
+        <v>85.2</v>
       </c>
       <c r="Y19" s="37" t="n">
-        <v>41.7</v>
+        <v>37.3</v>
       </c>
       <c r="Z19" s="37" t="n">
-        <v>67.40000000000001</v>
+        <v>77.5</v>
       </c>
       <c r="AA19" s="37" t="n">
-        <v>40.1</v>
+        <v>44.8</v>
       </c>
       <c r="AB19" s="37" t="n">
-        <v>49.9</v>
+        <v>40.8</v>
       </c>
       <c r="AC19" s="37" t="n">
-        <v>10.1</v>
+        <v>14.4</v>
       </c>
       <c r="AD19" s="34" t="inlineStr">
         <is>
-          <t>1-0 (%20)</t>
+          <t>1-0 (%14)</t>
         </is>
       </c>
       <c r="AE19" s="34" t="n"/>
@@ -3350,27 +3354,27 @@
       </c>
       <c r="C20" s="34" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="D20" s="34" t="inlineStr">
         <is>
-          <t>Arjantin</t>
+          <t>Avrupa</t>
         </is>
       </c>
       <c r="E20" s="34" t="inlineStr">
         <is>
-          <t>Liga Profesional (Arjantin)</t>
+          <t>UEFA Uluslar Ligi</t>
         </is>
       </c>
       <c r="F20" s="35" t="inlineStr">
         <is>
-          <t>Huracan</t>
+          <t>Greece</t>
         </is>
       </c>
       <c r="G20" s="35" t="inlineStr">
         <is>
-          <t>Aldosivi</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="H20" s="34" t="inlineStr">
@@ -3389,67 +3393,67 @@
         </is>
       </c>
       <c r="K20" s="34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L20" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="M20" s="36" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="M20" s="39" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
       <c r="N20" s="37" t="n">
-        <v>62.9</v>
+        <v>37.2</v>
       </c>
       <c r="O20" s="37" t="n">
-        <v>22.5</v>
+        <v>38.2</v>
       </c>
       <c r="P20" s="37" t="n">
-        <v>14.6</v>
+        <v>24.6</v>
       </c>
       <c r="Q20" s="38" t="n">
-        <v>1.83</v>
+        <v>1.06</v>
       </c>
       <c r="R20" s="38" t="n">
-        <v>0.75</v>
+        <v>0.83</v>
       </c>
       <c r="S20" s="37" t="n">
-        <v>47.6</v>
+        <v>29.5</v>
       </c>
       <c r="T20" s="37" t="n">
-        <v>52.4</v>
+        <v>70.5</v>
       </c>
       <c r="U20" s="37" t="n">
-        <v>44.4</v>
+        <v>40.2</v>
       </c>
       <c r="V20" s="37" t="n">
-        <v>55.6</v>
+        <v>59.8</v>
       </c>
       <c r="W20" s="37" t="n">
-        <v>73</v>
+        <v>59.8</v>
       </c>
       <c r="X20" s="37" t="n">
-        <v>85.40000000000001</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="Y20" s="37" t="n">
-        <v>37.1</v>
+        <v>62.8</v>
       </c>
       <c r="Z20" s="37" t="n">
-        <v>77.5</v>
+        <v>61.8</v>
       </c>
       <c r="AA20" s="37" t="n">
-        <v>45.1</v>
+        <v>28.4</v>
       </c>
       <c r="AB20" s="37" t="n">
-        <v>40.7</v>
+        <v>50.6</v>
       </c>
       <c r="AC20" s="37" t="n">
-        <v>14.3</v>
+        <v>21</v>
       </c>
       <c r="AD20" s="34" t="inlineStr">
         <is>
-          <t>1-0 (%14)</t>
+          <t>0-0 (%18)</t>
         </is>
       </c>
       <c r="AE20" s="34" t="n"/>
@@ -3502,12 +3506,12 @@
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Greece</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="G21" s="35" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Israel</t>
         </is>
       </c>
       <c r="H21" s="34" t="inlineStr">
@@ -3526,67 +3530,67 @@
         </is>
       </c>
       <c r="K21" s="34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" s="39" t="inlineStr">
-        <is>
-          <t>X</t>
+        <v>1</v>
+      </c>
+      <c r="M21" s="36" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
       <c r="N21" s="37" t="n">
-        <v>37.2</v>
+        <v>91.7</v>
       </c>
       <c r="O21" s="37" t="n">
-        <v>38.2</v>
+        <v>7.6</v>
       </c>
       <c r="P21" s="37" t="n">
-        <v>24.6</v>
+        <v>0.7</v>
       </c>
       <c r="Q21" s="38" t="n">
-        <v>1.06</v>
+        <v>3.23</v>
       </c>
       <c r="R21" s="38" t="n">
-        <v>0.83</v>
+        <v>0.26</v>
       </c>
       <c r="S21" s="37" t="n">
-        <v>29.5</v>
+        <v>67.8</v>
       </c>
       <c r="T21" s="37" t="n">
-        <v>70.5</v>
+        <v>32.2</v>
       </c>
       <c r="U21" s="37" t="n">
-        <v>40.2</v>
+        <v>23</v>
       </c>
       <c r="V21" s="37" t="n">
-        <v>59.8</v>
+        <v>77</v>
       </c>
       <c r="W21" s="37" t="n">
-        <v>59.8</v>
+        <v>87</v>
       </c>
       <c r="X21" s="37" t="n">
-        <v>75.40000000000001</v>
+        <v>99.3</v>
       </c>
       <c r="Y21" s="37" t="n">
-        <v>62.8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="Z21" s="37" t="n">
-        <v>61.8</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="AA21" s="37" t="n">
-        <v>28.4</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="AB21" s="37" t="n">
-        <v>50.6</v>
+        <v>24.5</v>
       </c>
       <c r="AC21" s="37" t="n">
-        <v>21</v>
+        <v>2.9</v>
       </c>
       <c r="AD21" s="34" t="inlineStr">
         <is>
-          <t>0-0 (%18)</t>
+          <t>3-0 (%17)</t>
         </is>
       </c>
       <c r="AE21" s="34" t="n"/>
@@ -3639,12 +3643,12 @@
       </c>
       <c r="F22" s="35" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="G22" s="35" t="inlineStr">
         <is>
-          <t>Israel</t>
+          <t>Serbia</t>
         </is>
       </c>
       <c r="H22" s="34" t="inlineStr">
@@ -3663,7 +3667,7 @@
         </is>
       </c>
       <c r="K22" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L22" s="34" t="n">
         <v>1</v>
@@ -3674,56 +3678,56 @@
         </is>
       </c>
       <c r="N22" s="37" t="n">
-        <v>91.7</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="O22" s="37" t="n">
-        <v>7.6</v>
+        <v>13.2</v>
       </c>
       <c r="P22" s="37" t="n">
-        <v>0.7</v>
+        <v>4.9</v>
       </c>
       <c r="Q22" s="38" t="n">
-        <v>3.23</v>
+        <v>3.15</v>
       </c>
       <c r="R22" s="38" t="n">
-        <v>0.26</v>
+        <v>0.79</v>
       </c>
       <c r="S22" s="37" t="n">
-        <v>67.8</v>
+        <v>75.2</v>
       </c>
       <c r="T22" s="37" t="n">
-        <v>32.2</v>
+        <v>24.8</v>
       </c>
       <c r="U22" s="37" t="n">
-        <v>23</v>
+        <v>53.5</v>
       </c>
       <c r="V22" s="37" t="n">
-        <v>77</v>
+        <v>46.5</v>
       </c>
       <c r="W22" s="37" t="n">
-        <v>87</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="X22" s="37" t="n">
-        <v>99.3</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="Y22" s="37" t="n">
-        <v>8.300000000000001</v>
+        <v>18.1</v>
       </c>
       <c r="Z22" s="37" t="n">
-        <v>92.40000000000001</v>
+        <v>86.8</v>
       </c>
       <c r="AA22" s="37" t="n">
-        <v>72.59999999999999</v>
+        <v>64.2</v>
       </c>
       <c r="AB22" s="37" t="n">
-        <v>24.5</v>
+        <v>26.7</v>
       </c>
       <c r="AC22" s="37" t="n">
-        <v>2.9</v>
+        <v>9.1</v>
       </c>
       <c r="AD22" s="34" t="inlineStr">
         <is>
-          <t>3-0 (%17)</t>
+          <t>3-0 (%10)</t>
         </is>
       </c>
       <c r="AE22" s="34" t="n"/>
@@ -3776,12 +3780,12 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="G23" s="35" t="inlineStr">
         <is>
-          <t>Serbia</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="H23" s="34" t="inlineStr">
@@ -3811,56 +3815,56 @@
         </is>
       </c>
       <c r="N23" s="37" t="n">
-        <v>81.90000000000001</v>
+        <v>83.7</v>
       </c>
       <c r="O23" s="37" t="n">
-        <v>13.2</v>
+        <v>9.5</v>
       </c>
       <c r="P23" s="37" t="n">
-        <v>4.9</v>
+        <v>6.8</v>
       </c>
       <c r="Q23" s="38" t="n">
-        <v>3.15</v>
+        <v>4.39</v>
       </c>
       <c r="R23" s="38" t="n">
-        <v>0.79</v>
+        <v>1.49</v>
       </c>
       <c r="S23" s="37" t="n">
-        <v>75.2</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="T23" s="37" t="n">
-        <v>24.8</v>
+        <v>6.9</v>
       </c>
       <c r="U23" s="37" t="n">
-        <v>53.5</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="V23" s="37" t="n">
-        <v>46.5</v>
+        <v>23.1</v>
       </c>
       <c r="W23" s="37" t="n">
-        <v>91.59999999999999</v>
+        <v>98.5</v>
       </c>
       <c r="X23" s="37" t="n">
-        <v>95.09999999999999</v>
+        <v>93.2</v>
       </c>
       <c r="Y23" s="37" t="n">
-        <v>18.1</v>
+        <v>16.3</v>
       </c>
       <c r="Z23" s="37" t="n">
-        <v>86.8</v>
+        <v>90.5</v>
       </c>
       <c r="AA23" s="37" t="n">
-        <v>64.2</v>
+        <v>68.2</v>
       </c>
       <c r="AB23" s="37" t="n">
-        <v>26.7</v>
+        <v>20.1</v>
       </c>
       <c r="AC23" s="37" t="n">
-        <v>9.1</v>
+        <v>11.7</v>
       </c>
       <c r="AD23" s="34" t="inlineStr">
         <is>
-          <t>3-0 (%10)</t>
+          <t>4-1 (%7)</t>
         </is>
       </c>
       <c r="AE23" s="34" t="n"/>
@@ -3913,12 +3917,12 @@
       </c>
       <c r="F24" s="35" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Wales</t>
         </is>
       </c>
       <c r="G24" s="35" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="H24" s="34" t="inlineStr">
@@ -3937,67 +3941,67 @@
         </is>
       </c>
       <c r="K24" s="34" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L24" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="M24" s="36" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="M24" s="40" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
       <c r="N24" s="37" t="n">
-        <v>83.7</v>
+        <v>24.7</v>
       </c>
       <c r="O24" s="37" t="n">
-        <v>9.5</v>
+        <v>24</v>
       </c>
       <c r="P24" s="37" t="n">
-        <v>6.8</v>
+        <v>51.3</v>
       </c>
       <c r="Q24" s="38" t="n">
-        <v>4.39</v>
+        <v>1.57</v>
       </c>
       <c r="R24" s="38" t="n">
-        <v>1.49</v>
+        <v>2.25</v>
       </c>
       <c r="S24" s="37" t="n">
-        <v>93.09999999999999</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="T24" s="37" t="n">
-        <v>6.9</v>
+        <v>26.6</v>
       </c>
       <c r="U24" s="37" t="n">
-        <v>76.90000000000001</v>
+        <v>72.7</v>
       </c>
       <c r="V24" s="37" t="n">
-        <v>23.1</v>
+        <v>27.3</v>
       </c>
       <c r="W24" s="37" t="n">
-        <v>98.5</v>
+        <v>91.3</v>
       </c>
       <c r="X24" s="37" t="n">
-        <v>93.2</v>
+        <v>48.7</v>
       </c>
       <c r="Y24" s="37" t="n">
-        <v>16.3</v>
+        <v>75.3</v>
       </c>
       <c r="Z24" s="37" t="n">
-        <v>90.5</v>
+        <v>76</v>
       </c>
       <c r="AA24" s="37" t="n">
-        <v>68.2</v>
+        <v>24.8</v>
       </c>
       <c r="AB24" s="37" t="n">
-        <v>20.1</v>
+        <v>33.2</v>
       </c>
       <c r="AC24" s="37" t="n">
-        <v>11.7</v>
+        <v>41.9</v>
       </c>
       <c r="AD24" s="34" t="inlineStr">
         <is>
-          <t>4-1 (%7)</t>
+          <t>1-1 (%10)</t>
         </is>
       </c>
       <c r="AE24" s="34" t="n"/>
@@ -4035,27 +4039,27 @@
       </c>
       <c r="C25" s="34" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D25" s="34" t="inlineStr">
         <is>
-          <t>Avrupa</t>
+          <t>Arjantin</t>
         </is>
       </c>
       <c r="E25" s="34" t="inlineStr">
         <is>
-          <t>UEFA Uluslar Ligi</t>
+          <t>Liga Profesional (Arjantin)</t>
         </is>
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Wales</t>
+          <t>Talleres Cordoba</t>
         </is>
       </c>
       <c r="G25" s="35" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Belgrano</t>
         </is>
       </c>
       <c r="H25" s="34" t="inlineStr">
@@ -4085,56 +4089,56 @@
         </is>
       </c>
       <c r="N25" s="37" t="n">
-        <v>24.7</v>
+        <v>20</v>
       </c>
       <c r="O25" s="37" t="n">
-        <v>24</v>
+        <v>25.1</v>
       </c>
       <c r="P25" s="37" t="n">
-        <v>51.3</v>
+        <v>54.9</v>
       </c>
       <c r="Q25" s="38" t="n">
-        <v>1.57</v>
+        <v>0.87</v>
       </c>
       <c r="R25" s="38" t="n">
-        <v>2.25</v>
+        <v>1.62</v>
       </c>
       <c r="S25" s="37" t="n">
-        <v>73.40000000000001</v>
+        <v>45.2</v>
       </c>
       <c r="T25" s="37" t="n">
-        <v>26.6</v>
+        <v>54.8</v>
       </c>
       <c r="U25" s="37" t="n">
-        <v>72.7</v>
+        <v>46.7</v>
       </c>
       <c r="V25" s="37" t="n">
-        <v>27.3</v>
+        <v>53.3</v>
       </c>
       <c r="W25" s="37" t="n">
-        <v>91.3</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="X25" s="37" t="n">
-        <v>48.7</v>
+        <v>45.1</v>
       </c>
       <c r="Y25" s="37" t="n">
-        <v>75.3</v>
+        <v>80</v>
       </c>
       <c r="Z25" s="37" t="n">
-        <v>76</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="AA25" s="37" t="n">
-        <v>24.8</v>
+        <v>17.8</v>
       </c>
       <c r="AB25" s="37" t="n">
-        <v>33.2</v>
+        <v>42.7</v>
       </c>
       <c r="AC25" s="37" t="n">
-        <v>41.9</v>
+        <v>39.5</v>
       </c>
       <c r="AD25" s="34" t="inlineStr">
         <is>
-          <t>1-1 (%10)</t>
+          <t>0-1 (%13)</t>
         </is>
       </c>
       <c r="AE25" s="34" t="n"/>
@@ -4160,423 +4164,414 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="41" t="inlineStr">
+      <c r="A26" s="34" t="inlineStr">
         <is>
           <t>05.10.2026</t>
         </is>
       </c>
-      <c r="B26" s="41" t="inlineStr">
+      <c r="B26" s="34" t="inlineStr">
         <is>
           <t>Pazartesi</t>
         </is>
       </c>
-      <c r="C26" s="41" t="inlineStr">
+      <c r="C26" s="34" t="inlineStr">
         <is>
           <t>01:15</t>
         </is>
       </c>
-      <c r="D26" s="41" t="inlineStr">
+      <c r="D26" s="34" t="inlineStr">
         <is>
           <t>Arjantin</t>
         </is>
       </c>
-      <c r="E26" s="41" t="inlineStr">
+      <c r="E26" s="34" t="inlineStr">
         <is>
           <t>Liga Profesional (Arjantin)</t>
         </is>
       </c>
-      <c r="F26" s="42" t="inlineStr">
+      <c r="F26" s="35" t="inlineStr">
         <is>
           <t>Argentinos Jrs</t>
         </is>
       </c>
-      <c r="G26" s="42" t="inlineStr">
+      <c r="G26" s="35" t="inlineStr">
         <is>
           <t>Tigre</t>
         </is>
       </c>
-      <c r="H26" s="41" t="inlineStr">
-        <is>
-          <t>Canlı</t>
-        </is>
-      </c>
-      <c r="I26" s="41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J26" s="41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K26" s="41" t="n">
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>Bitti</t>
+        </is>
+      </c>
+      <c r="I26" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J26" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K26" s="34" t="n">
         <v>2</v>
       </c>
-      <c r="L26" s="41" t="n">
+      <c r="L26" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="M26" s="43" t="inlineStr">
+      <c r="M26" s="36" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="N26" s="44" t="n">
-        <v>53</v>
-      </c>
-      <c r="O26" s="44" t="n">
-        <v>29.5</v>
-      </c>
-      <c r="P26" s="44" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="Q26" s="45" t="n">
+      <c r="N26" s="37" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="O26" s="37" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="P26" s="37" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="Q26" s="38" t="n">
         <v>1.28</v>
       </c>
-      <c r="R26" s="45" t="n">
+      <c r="R26" s="38" t="n">
         <v>0.61</v>
       </c>
-      <c r="S26" s="44" t="n">
+      <c r="S26" s="37" t="n">
         <v>29.4</v>
       </c>
-      <c r="T26" s="44" t="n">
+      <c r="T26" s="37" t="n">
         <v>70.59999999999999</v>
       </c>
-      <c r="U26" s="44" t="n">
+      <c r="U26" s="37" t="n">
         <v>33</v>
       </c>
-      <c r="V26" s="44" t="n">
+      <c r="V26" s="37" t="n">
         <v>67</v>
       </c>
-      <c r="W26" s="44" t="n">
-        <v>56.5</v>
-      </c>
-      <c r="X26" s="44" t="n">
-        <v>82.5</v>
-      </c>
-      <c r="Y26" s="44" t="n">
-        <v>47</v>
-      </c>
-      <c r="Z26" s="44" t="n">
-        <v>70.5</v>
-      </c>
-      <c r="AA26" s="44" t="n">
-        <v>35.9</v>
-      </c>
-      <c r="AB26" s="44" t="n">
+      <c r="W26" s="37" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="X26" s="37" t="n">
+        <v>82.3</v>
+      </c>
+      <c r="Y26" s="37" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="Z26" s="37" t="n">
+        <v>70.59999999999999</v>
+      </c>
+      <c r="AA26" s="37" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="AB26" s="37" t="n">
         <v>49.7</v>
       </c>
-      <c r="AC26" s="44" t="n">
-        <v>14.4</v>
-      </c>
-      <c r="AD26" s="41" t="inlineStr">
+      <c r="AC26" s="37" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="AD26" s="34" t="inlineStr">
         <is>
           <t>1-0 (%19)</t>
         </is>
       </c>
-      <c r="AE26" s="41" t="n"/>
-      <c r="AF26" s="41" t="inlineStr">
-        <is>
-          <t>Gariano A.</t>
-        </is>
-      </c>
-      <c r="AG26" s="41" t="inlineStr">
-        <is>
-          <t>Estadio Diego Armando Maradona (Buenos Aires)</t>
-        </is>
-      </c>
-      <c r="AH26" s="41" t="inlineStr">
-        <is>
-          <t>17°C, Açık, 8 km/sa</t>
-        </is>
-      </c>
-      <c r="AI26" s="41" t="inlineStr">
-        <is>
-          <t>EV: (Kesin) Siri Payer, Paredes, Mendoza, Alvarez, Prieto, Gutierrez, Lopez, Gimenez, Oroz, Veron, Molina
-DEP: (Kesin) Zenobio, Moreno, Laso, Barrionuevo, Alvarez, Saralegui, Gonzalez, Leyes, Lopez, Russo, Domina</t>
+      <c r="AE26" s="34" t="n"/>
+      <c r="AF26" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG26" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AH26" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI26" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="46" t="inlineStr">
+      <c r="A27" s="34" t="inlineStr">
         <is>
           <t>05.10.2026</t>
         </is>
       </c>
-      <c r="B27" s="46" t="inlineStr">
+      <c r="B27" s="34" t="inlineStr">
         <is>
           <t>Pazartesi</t>
         </is>
       </c>
-      <c r="C27" s="46" t="inlineStr">
+      <c r="C27" s="34" t="inlineStr">
         <is>
           <t>03:30</t>
         </is>
       </c>
-      <c r="D27" s="46" t="inlineStr">
+      <c r="D27" s="34" t="inlineStr">
         <is>
           <t>Arjantin</t>
         </is>
       </c>
-      <c r="E27" s="46" t="inlineStr">
+      <c r="E27" s="34" t="inlineStr">
         <is>
           <t>Liga Profesional (Arjantin)</t>
         </is>
       </c>
-      <c r="F27" s="47" t="inlineStr">
+      <c r="F27" s="35" t="inlineStr">
         <is>
           <t>Estudiantes Rio Cuarto</t>
         </is>
       </c>
-      <c r="G27" s="47" t="inlineStr">
+      <c r="G27" s="35" t="inlineStr">
         <is>
           <t>Racing Club</t>
         </is>
       </c>
-      <c r="H27" s="46" t="inlineStr">
-        <is>
-          <t>Planlandı</t>
-        </is>
-      </c>
-      <c r="I27" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J27" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K27" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L27" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M27" s="48" t="inlineStr">
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>Bitti</t>
+        </is>
+      </c>
+      <c r="I27" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J27" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K27" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="L27" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="M27" s="40" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="N27" s="49" t="n">
+      <c r="N27" s="37" t="n">
         <v>28.9</v>
       </c>
-      <c r="O27" s="49" t="n">
-        <v>30.7</v>
-      </c>
-      <c r="P27" s="49" t="n">
-        <v>40.4</v>
-      </c>
-      <c r="Q27" s="50" t="n">
+      <c r="O27" s="37" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="P27" s="37" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="Q27" s="38" t="n">
         <v>0.9</v>
       </c>
-      <c r="R27" s="50" t="n">
+      <c r="R27" s="38" t="n">
         <v>1.12</v>
       </c>
-      <c r="S27" s="49" t="n">
+      <c r="S27" s="37" t="n">
         <v>32.8</v>
       </c>
-      <c r="T27" s="49" t="n">
+      <c r="T27" s="37" t="n">
         <v>67.2</v>
       </c>
-      <c r="U27" s="49" t="n">
+      <c r="U27" s="37" t="n">
         <v>40</v>
       </c>
-      <c r="V27" s="49" t="n">
+      <c r="V27" s="37" t="n">
         <v>60</v>
       </c>
-      <c r="W27" s="49" t="n">
-        <v>60</v>
-      </c>
-      <c r="X27" s="49" t="n">
-        <v>59.6</v>
-      </c>
-      <c r="Y27" s="49" t="n">
+      <c r="W27" s="37" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="X27" s="37" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="Y27" s="37" t="n">
         <v>71.09999999999999</v>
       </c>
-      <c r="Z27" s="49" t="n">
-        <v>69.3</v>
-      </c>
-      <c r="AA27" s="49" t="n">
-        <v>22.1</v>
-      </c>
-      <c r="AB27" s="49" t="n">
+      <c r="Z27" s="37" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="AA27" s="37" t="n">
+        <v>22</v>
+      </c>
+      <c r="AB27" s="37" t="n">
         <v>49</v>
       </c>
-      <c r="AC27" s="49" t="n">
-        <v>28.9</v>
-      </c>
-      <c r="AD27" s="51" t="inlineStr">
+      <c r="AC27" s="37" t="n">
+        <v>29</v>
+      </c>
+      <c r="AD27" s="34" t="inlineStr">
         <is>
           <t>0-1 (%15)</t>
         </is>
       </c>
-      <c r="AE27" s="46" t="n"/>
-      <c r="AF27" s="46" t="inlineStr">
-        <is>
-          <t>Viola F.</t>
-        </is>
-      </c>
-      <c r="AG27" s="46" t="inlineStr">
-        <is>
-          <t>Estadio Ciudad de Río Cuarto Antonio Candini (Cordoba)</t>
-        </is>
-      </c>
-      <c r="AH27" s="46" t="inlineStr">
-        <is>
-          <t>17°C, Bulutlu, 7 km/sa</t>
-        </is>
-      </c>
-      <c r="AI27" s="46" t="inlineStr">
-        <is>
-          <t>EV: (Tahmini) Bruera, Antonini, Maffini, Valenti, Cabrera, Gonzalez, Gonzalez, Alanis, Rodriguez, Valiente, Hesar
-DEP: (Tahmini) Cambeses, Cannavo, Martinez, Perez, Escudero, Rodriguez, Ortegoza, Perez, Lodico, Diaz, Adrian Martinez</t>
+      <c r="AE27" s="34" t="n"/>
+      <c r="AF27" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG27" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AH27" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI27" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="52" t="inlineStr">
+      <c r="A28" s="41" t="inlineStr">
         <is>
           <t>05.10.2026</t>
         </is>
       </c>
-      <c r="B28" s="52" t="inlineStr">
+      <c r="B28" s="41" t="inlineStr">
         <is>
           <t>Pazartesi</t>
         </is>
       </c>
-      <c r="C28" s="52" t="inlineStr">
+      <c r="C28" s="41" t="inlineStr">
         <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="D28" s="52" t="inlineStr">
+      <c r="D28" s="41" t="inlineStr">
         <is>
           <t>Avrupa</t>
         </is>
       </c>
-      <c r="E28" s="52" t="inlineStr">
+      <c r="E28" s="41" t="inlineStr">
         <is>
           <t>UEFA Uluslar Ligi</t>
         </is>
       </c>
-      <c r="F28" s="53" t="inlineStr">
+      <c r="F28" s="42" t="inlineStr">
         <is>
           <t>Cyprus</t>
         </is>
       </c>
-      <c r="G28" s="53" t="inlineStr">
+      <c r="G28" s="42" t="inlineStr">
         <is>
           <t>Latvia</t>
         </is>
       </c>
-      <c r="H28" s="52" t="inlineStr">
-        <is>
-          <t>Planlandı</t>
-        </is>
-      </c>
-      <c r="I28" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J28" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K28" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L28" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M28" s="54" t="inlineStr">
+      <c r="H28" s="41" t="inlineStr">
+        <is>
+          <t>Devre Arası</t>
+        </is>
+      </c>
+      <c r="I28" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J28" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K28" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="43" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="N28" s="49" t="n">
+      <c r="N28" s="44" t="n">
         <v>65.2</v>
       </c>
-      <c r="O28" s="49" t="n">
+      <c r="O28" s="44" t="n">
         <v>30.8</v>
       </c>
-      <c r="P28" s="49" t="n">
+      <c r="P28" s="44" t="n">
         <v>4</v>
       </c>
-      <c r="Q28" s="50" t="n">
+      <c r="Q28" s="45" t="n">
         <v>1.32</v>
       </c>
-      <c r="R28" s="50" t="n">
+      <c r="R28" s="45" t="n">
         <v>0.2</v>
       </c>
-      <c r="S28" s="49" t="n">
+      <c r="S28" s="44" t="n">
         <v>19.6</v>
       </c>
-      <c r="T28" s="49" t="n">
+      <c r="T28" s="44" t="n">
         <v>80.40000000000001</v>
       </c>
-      <c r="U28" s="49" t="n">
+      <c r="U28" s="44" t="n">
         <v>14.6</v>
       </c>
-      <c r="V28" s="49" t="n">
+      <c r="V28" s="44" t="n">
         <v>85.40000000000001</v>
       </c>
-      <c r="W28" s="49" t="n">
+      <c r="W28" s="44" t="n">
         <v>46.3</v>
       </c>
-      <c r="X28" s="49" t="n">
+      <c r="X28" s="44" t="n">
         <v>96</v>
       </c>
-      <c r="Y28" s="49" t="n">
+      <c r="Y28" s="44" t="n">
         <v>34.8</v>
       </c>
-      <c r="Z28" s="49" t="n">
+      <c r="Z28" s="44" t="n">
         <v>69.2</v>
       </c>
-      <c r="AA28" s="49" t="n">
+      <c r="AA28" s="44" t="n">
         <v>42</v>
       </c>
-      <c r="AB28" s="49" t="n">
+      <c r="AB28" s="44" t="n">
         <v>53.2</v>
       </c>
-      <c r="AC28" s="49" t="n">
+      <c r="AC28" s="44" t="n">
         <v>4.8</v>
       </c>
-      <c r="AD28" s="51" t="inlineStr">
+      <c r="AD28" s="41" t="inlineStr">
         <is>
           <t>1-0 (%27)</t>
         </is>
       </c>
-      <c r="AE28" s="52" t="n"/>
-      <c r="AF28" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG28" s="52" t="inlineStr">
+      <c r="AE28" s="41" t="n"/>
+      <c r="AF28" s="41" t="inlineStr">
+        <is>
+          <t>Kruashvili G.</t>
+        </is>
+      </c>
+      <c r="AG28" s="41" t="inlineStr">
         <is>
           <t>GSP Stadium (Nicosia)</t>
         </is>
       </c>
-      <c r="AH28" s="52" t="inlineStr">
-        <is>
-          <t>22°C, Bulutlu, 8 km/sa</t>
-        </is>
-      </c>
-      <c r="AI28" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="AH28" s="41" t="inlineStr">
+        <is>
+          <t>22°C, Bulutlu, 12 km/sa</t>
+        </is>
+      </c>
+      <c r="AI28" s="41" t="inlineStr">
+        <is>
+          <t>EV: (Kesin) Fabiano, Konomis, Kyprianou, Panagiotou, Malekkidis, Artymatas, Kastanos, Edwards, Loizou, Kakoullis, Pittas
+DEP: (Kesin) Matrevics, Jurkovskis, Melniks, Vientiess, Balodis, Ciganiks, Daskevics, Vapne, Zelenkovs, Strods, Gutkovskis</t>
         </is>
       </c>
     </row>
@@ -4712,12 +4707,13 @@
       </c>
       <c r="AH29" s="46" t="inlineStr">
         <is>
-          <t>18°C, Bulutlu, 2 km/sa</t>
+          <t>17°C, Bulutlu, 1 km/sa</t>
         </is>
       </c>
       <c r="AI29" s="46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Tahmini) Hamzic, Memic, Katic, Muharemovic, Kolasinac, Bajraktarevic, Basic, Gigovic, Alajbegovic, Demirovic, Tabakovic
+DEP: (Tahmini) Bulka, Cash, Bednarek, Kiwior, Frankowski, Nowak, Zielinski, Swiderski, Szymanski, Zalewski, Zukowski</t>
         </is>
       </c>
     </row>
@@ -4782,65 +4778,69 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M30" s="55" t="inlineStr">
+      <c r="M30" s="54" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
       <c r="N30" s="49" t="n">
-        <v>16.5</v>
+        <v>15.3</v>
       </c>
       <c r="O30" s="49" t="n">
-        <v>56.5</v>
+        <v>60.2</v>
       </c>
       <c r="P30" s="49" t="n">
-        <v>26.9</v>
+        <v>24.5</v>
       </c>
       <c r="Q30" s="50" t="n">
-        <v>0.31</v>
+        <v>0.27</v>
       </c>
       <c r="R30" s="50" t="n">
-        <v>0.46</v>
+        <v>0.39</v>
       </c>
       <c r="S30" s="49" t="n">
-        <v>4.3</v>
+        <v>2.9</v>
       </c>
       <c r="T30" s="49" t="n">
-        <v>95.7</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="U30" s="49" t="n">
-        <v>11.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="V30" s="49" t="n">
-        <v>88.5</v>
+        <v>91.2</v>
       </c>
       <c r="W30" s="49" t="n">
-        <v>19.6</v>
+        <v>15.3</v>
       </c>
       <c r="X30" s="49" t="n">
-        <v>73.09999999999999</v>
+        <v>75.5</v>
       </c>
       <c r="Y30" s="49" t="n">
-        <v>83.5</v>
+        <v>84.7</v>
       </c>
       <c r="Z30" s="49" t="n">
-        <v>43.5</v>
+        <v>39.8</v>
       </c>
       <c r="AA30" s="49" t="n">
-        <v>10.8</v>
+        <v>9.6</v>
       </c>
       <c r="AB30" s="49" t="n">
-        <v>72.8</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="AC30" s="49" t="n">
-        <v>16.3</v>
+        <v>14.3</v>
       </c>
       <c r="AD30" s="51" t="inlineStr">
         <is>
-          <t>0-0 (%48)</t>
-        </is>
-      </c>
-      <c r="AE30" s="52" t="n"/>
+          <t>0-0 (%53)</t>
+        </is>
+      </c>
+      <c r="AE30" s="52" t="inlineStr">
+        <is>
+          <t>Ev kilit oyuncu eksik (Olise M.) -&gt; hücum -%15 | Dep kilit oyuncu eksik (De Bruyne K.) -&gt; hücum -%15</t>
+        </is>
+      </c>
       <c r="AF30" s="52" t="inlineStr">
         <is>
           <t>-</t>
@@ -4858,7 +4858,8 @@
       </c>
       <c r="AI30" s="52" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Tahmini) Restes, Kounde, Yoro, Lacroix, Diouf, Akliouche, Camavinga, Kone, Dembele, Barcola, Lepaul
+DEP: (Tahmini) Lammens, Castagne, Ngoy, Mechele, De Cuyper, Lavia, Raskin, Moreira, Vanaken, Godts, De Ketelaere</t>
         </is>
       </c>
     </row>
@@ -4923,65 +4924,69 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M31" s="54" t="inlineStr">
+      <c r="M31" s="55" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="N31" s="49" t="n">
-        <v>95.09999999999999</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="O31" s="49" t="n">
-        <v>4.4</v>
+        <v>4</v>
       </c>
       <c r="P31" s="49" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="Q31" s="50" t="n">
         <v>4.19</v>
       </c>
       <c r="R31" s="50" t="n">
-        <v>0.38</v>
+        <v>0.32</v>
       </c>
       <c r="S31" s="49" t="n">
-        <v>83.2</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="T31" s="49" t="n">
-        <v>16.8</v>
+        <v>17.4</v>
       </c>
       <c r="U31" s="49" t="n">
-        <v>31.7</v>
+        <v>27.7</v>
       </c>
       <c r="V31" s="49" t="n">
-        <v>68.3</v>
+        <v>72.3</v>
       </c>
       <c r="W31" s="49" t="n">
-        <v>94.59999999999999</v>
+        <v>94.2</v>
       </c>
       <c r="X31" s="49" t="n">
-        <v>99.40000000000001</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="Y31" s="49" t="n">
-        <v>4.9</v>
+        <v>4.4</v>
       </c>
       <c r="Z31" s="49" t="n">
-        <v>95.59999999999999</v>
+        <v>96</v>
       </c>
       <c r="AA31" s="49" t="n">
-        <v>79.90000000000001</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="AB31" s="49" t="n">
-        <v>17.3</v>
+        <v>17</v>
       </c>
       <c r="AC31" s="49" t="n">
-        <v>2.8</v>
+        <v>2.4</v>
       </c>
       <c r="AD31" s="51" t="inlineStr">
         <is>
-          <t>4-0 (%13)</t>
-        </is>
-      </c>
-      <c r="AE31" s="46" t="n"/>
+          <t>4-0 (%14)</t>
+        </is>
+      </c>
+      <c r="AE31" s="46" t="inlineStr">
+        <is>
+          <t>Dep kilit oyuncu eksik (Yilmaz B.) -&gt; hücum -%15</t>
+        </is>
+      </c>
       <c r="AF31" s="46" t="inlineStr">
         <is>
           <t>-</t>
@@ -4999,7 +5004,8 @@
       </c>
       <c r="AI31" s="46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Tahmini) Donnarumma, Kayode, Scalvini, Bastoni, Calafiori, Barella, Tonali, Fagioli, Vergara, Esposito, Esposito
+DEP: (Tahmini) Cakir, Celik, Demiral, Bardakci, Kadioglu, Aydin, Elmaz, Yuksek, Akturkoglu, Gul, Akgun</t>
         </is>
       </c>
     </row>
@@ -5064,7 +5070,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M32" s="54" t="inlineStr">
+      <c r="M32" s="55" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5135,12 +5141,13 @@
       </c>
       <c r="AH32" s="52" t="inlineStr">
         <is>
-          <t>16°C, Az bulutlu, 5 km/sa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AI32" s="52" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: -
+DEP: -</t>
         </is>
       </c>
     </row>
@@ -5205,7 +5212,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M33" s="54" t="inlineStr">
+      <c r="M33" s="55" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5276,12 +5283,13 @@
       </c>
       <c r="AH33" s="46" t="inlineStr">
         <is>
-          <t>14°C, Bulutlu, 3 km/sa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AI33" s="46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Tahmini) Charles, Spencer, Atcheson, McConville, Brown, Devlin, Morrison, Hume, Charles, Price, Donley
+DEP: (Tahmini) Mamardashvili, Kakabadze, Goglichidze, Dvali, Lochoshvili, Tsitaishvili, Yegoian, Mekvabishvili, Chakvetadze, Mikautadze, Kvaratskhelia</t>
         </is>
       </c>
     </row>
@@ -5407,7 +5415,7 @@
       <c r="AE34" s="52" t="n"/>
       <c r="AF34" s="52" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Masiyev E.</t>
         </is>
       </c>
       <c r="AG34" s="52" t="inlineStr">
@@ -5417,12 +5425,13 @@
       </c>
       <c r="AH34" s="52" t="inlineStr">
         <is>
-          <t>18°C, Parçalı bulutlu, 2 km/sa</t>
+          <t>18°C, Az bulutlu, 1 km/sa</t>
         </is>
       </c>
       <c r="AI34" s="52" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Tahmini) Hindrich, Ratiu, Coubis, Ilie, Bancu, Marin, Baluta, Mihaila, Hagi, Man, Birligea
+DEP: (Tahmini) Johansson, Skoglund, Lindelof, Smith, Gudmundsson, Bernhardsson, Larsson, Karlstrom, Nanasi, Zeneli, Gyokeres</t>
         </is>
       </c>
     </row>
@@ -5487,7 +5496,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M35" s="55" t="inlineStr">
+      <c r="M35" s="54" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -5558,12 +5567,13 @@
       </c>
       <c r="AH35" s="46" t="inlineStr">
         <is>
-          <t>17°C, Açık, 4 km/sa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AI35" s="46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Tahmini) Riznyk, Bondar, Zabarnyi, Sarapiy, Mykhaylichenko, Tsygankov, Ocheretko, Brazhko, Sudakov, Yarmolenko, Yaremchuk
+DEP: (Tahmini) Toth, Osvath, Orban, Csinger, Markgraf, Schafer, Toth, Lukacs, Szoboszlai, Nagy, Toth</t>
         </is>
       </c>
     </row>
@@ -5628,7 +5638,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M36" s="55" t="inlineStr">
+      <c r="M36" s="54" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -5704,7 +5714,8 @@
       </c>
       <c r="AI36" s="52" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: -
+DEP: -</t>
         </is>
       </c>
     </row>
@@ -5769,19 +5780,19 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M37" s="54" t="inlineStr">
+      <c r="M37" s="55" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="N37" s="49" t="n">
-        <v>50</v>
+        <v>49.9</v>
       </c>
       <c r="O37" s="49" t="n">
         <v>32.8</v>
       </c>
       <c r="P37" s="49" t="n">
-        <v>17.2</v>
+        <v>17.3</v>
       </c>
       <c r="Q37" s="50" t="n">
         <v>1.11</v>
@@ -5790,37 +5801,37 @@
         <v>0.52</v>
       </c>
       <c r="S37" s="49" t="n">
-        <v>22.5</v>
+        <v>22.4</v>
       </c>
       <c r="T37" s="49" t="n">
-        <v>77.5</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="U37" s="49" t="n">
-        <v>27.4</v>
+        <v>27.3</v>
       </c>
       <c r="V37" s="49" t="n">
-        <v>72.59999999999999</v>
+        <v>72.7</v>
       </c>
       <c r="W37" s="49" t="n">
-        <v>48.7</v>
+        <v>48.5</v>
       </c>
       <c r="X37" s="49" t="n">
-        <v>82.8</v>
+        <v>82.7</v>
       </c>
       <c r="Y37" s="49" t="n">
-        <v>50</v>
+        <v>50.1</v>
       </c>
       <c r="Z37" s="49" t="n">
         <v>67.2</v>
       </c>
       <c r="AA37" s="49" t="n">
-        <v>32.8</v>
+        <v>32.7</v>
       </c>
       <c r="AB37" s="49" t="n">
-        <v>53.7</v>
+        <v>53.8</v>
       </c>
       <c r="AC37" s="49" t="n">
-        <v>13.4</v>
+        <v>13.5</v>
       </c>
       <c r="AD37" s="51" t="inlineStr">
         <is>
@@ -5830,22 +5841,23 @@
       <c r="AE37" s="46" t="n"/>
       <c r="AF37" s="46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Merlos A.</t>
         </is>
       </c>
       <c r="AG37" s="46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Estadio Guillermo Laza (Buenos Aires)</t>
         </is>
       </c>
       <c r="AH37" s="46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>20°C, Bulutlu, 14 km/sa</t>
         </is>
       </c>
       <c r="AI37" s="46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Tahmini) Arce, Bracamonte, Gariglio, Paz, Ramirez, Sansotre, Goitia, Celiz, Monje, Diaz, Gonzalez
+DEP: (Tahmini) Aguerre, Moyano, Maciel, Casermeiro, Martinez, Vera, Gonzalez, Barrera, Iacobellis, Caceres, Naya</t>
         </is>
       </c>
     </row>
@@ -5910,19 +5922,19 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M38" s="54" t="inlineStr">
+      <c r="M38" s="55" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="N38" s="49" t="n">
-        <v>41.6</v>
+        <v>41.5</v>
       </c>
       <c r="O38" s="49" t="n">
-        <v>28.1</v>
+        <v>28</v>
       </c>
       <c r="P38" s="49" t="n">
-        <v>30.2</v>
+        <v>30.5</v>
       </c>
       <c r="Q38" s="50" t="n">
         <v>1.28</v>
@@ -5931,10 +5943,10 @@
         <v>1.05</v>
       </c>
       <c r="S38" s="49" t="n">
-        <v>41.1</v>
+        <v>41.2</v>
       </c>
       <c r="T38" s="49" t="n">
-        <v>58.9</v>
+        <v>58.8</v>
       </c>
       <c r="U38" s="49" t="n">
         <v>47</v>
@@ -5943,25 +5955,25 @@
         <v>53</v>
       </c>
       <c r="W38" s="49" t="n">
-        <v>67.7</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="X38" s="49" t="n">
-        <v>69.8</v>
+        <v>69.5</v>
       </c>
       <c r="Y38" s="49" t="n">
-        <v>58.4</v>
+        <v>58.5</v>
       </c>
       <c r="Z38" s="49" t="n">
-        <v>71.90000000000001</v>
+        <v>72</v>
       </c>
       <c r="AA38" s="49" t="n">
-        <v>30.8</v>
+        <v>30.7</v>
       </c>
       <c r="AB38" s="49" t="n">
         <v>45.3</v>
       </c>
       <c r="AC38" s="49" t="n">
-        <v>23.9</v>
+        <v>24</v>
       </c>
       <c r="AD38" s="51" t="inlineStr">
         <is>
@@ -6051,58 +6063,58 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M39" s="54" t="inlineStr">
+      <c r="M39" s="55" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="N39" s="49" t="n">
-        <v>80.90000000000001</v>
+        <v>80.7</v>
       </c>
       <c r="O39" s="49" t="n">
-        <v>12.8</v>
+        <v>12.9</v>
       </c>
       <c r="P39" s="49" t="n">
-        <v>6.2</v>
+        <v>6.4</v>
       </c>
       <c r="Q39" s="50" t="n">
-        <v>2.72</v>
+        <v>2.7</v>
       </c>
       <c r="R39" s="50" t="n">
         <v>0.64</v>
       </c>
       <c r="S39" s="49" t="n">
-        <v>65.09999999999999</v>
+        <v>64.7</v>
       </c>
       <c r="T39" s="49" t="n">
-        <v>34.9</v>
+        <v>35.3</v>
       </c>
       <c r="U39" s="49" t="n">
-        <v>44.1</v>
+        <v>44</v>
       </c>
       <c r="V39" s="49" t="n">
-        <v>55.9</v>
+        <v>56</v>
       </c>
       <c r="W39" s="49" t="n">
-        <v>84.8</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="X39" s="49" t="n">
-        <v>93.8</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="Y39" s="49" t="n">
-        <v>19.1</v>
+        <v>19.3</v>
       </c>
       <c r="Z39" s="49" t="n">
-        <v>87.2</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="AA39" s="49" t="n">
-        <v>60.8</v>
+        <v>60.5</v>
       </c>
       <c r="AB39" s="49" t="n">
-        <v>30.6</v>
+        <v>30.8</v>
       </c>
       <c r="AC39" s="49" t="n">
-        <v>8.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="AD39" s="51" t="inlineStr">
         <is>
@@ -6198,52 +6210,52 @@
         </is>
       </c>
       <c r="N40" s="49" t="n">
-        <v>33.3</v>
+        <v>33</v>
       </c>
       <c r="O40" s="49" t="n">
-        <v>25.6</v>
+        <v>25.5</v>
       </c>
       <c r="P40" s="49" t="n">
-        <v>41.1</v>
+        <v>41.5</v>
       </c>
       <c r="Q40" s="50" t="n">
-        <v>1.29</v>
+        <v>1.28</v>
       </c>
       <c r="R40" s="50" t="n">
-        <v>1.46</v>
+        <v>1.47</v>
       </c>
       <c r="S40" s="49" t="n">
-        <v>52</v>
+        <v>51.9</v>
       </c>
       <c r="T40" s="49" t="n">
-        <v>48</v>
+        <v>48.1</v>
       </c>
       <c r="U40" s="49" t="n">
-        <v>55.9</v>
+        <v>55.7</v>
       </c>
       <c r="V40" s="49" t="n">
-        <v>44.1</v>
+        <v>44.3</v>
       </c>
       <c r="W40" s="49" t="n">
-        <v>76.2</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="X40" s="49" t="n">
-        <v>58.9</v>
+        <v>58.5</v>
       </c>
       <c r="Y40" s="49" t="n">
-        <v>66.7</v>
+        <v>67</v>
       </c>
       <c r="Z40" s="49" t="n">
-        <v>74.40000000000001</v>
+        <v>74.5</v>
       </c>
       <c r="AA40" s="49" t="n">
-        <v>27</v>
+        <v>26.8</v>
       </c>
       <c r="AB40" s="49" t="n">
-        <v>41.1</v>
+        <v>41.2</v>
       </c>
       <c r="AC40" s="49" t="n">
-        <v>31.9</v>
+        <v>32</v>
       </c>
       <c r="AD40" s="51" t="inlineStr">
         <is>
@@ -6474,7 +6486,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M42" s="54" t="inlineStr">
+      <c r="M42" s="55" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -6897,7 +6909,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M45" s="54" t="inlineStr">
+      <c r="M45" s="55" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -7038,7 +7050,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M46" s="55" t="inlineStr">
+      <c r="M46" s="54" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -7179,7 +7191,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M47" s="54" t="inlineStr">
+      <c r="M47" s="55" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -7461,7 +7473,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M49" s="55" t="inlineStr">
+      <c r="M49" s="54" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -7602,7 +7614,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M50" s="54" t="inlineStr">
+      <c r="M50" s="55" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -7682,713 +7694,8 @@
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="46" t="inlineStr">
-        <is>
-          <t>08.10.2026</t>
-        </is>
-      </c>
-      <c r="B51" s="46" t="inlineStr">
-        <is>
-          <t>Perşembe</t>
-        </is>
-      </c>
-      <c r="C51" s="46" t="inlineStr">
-        <is>
-          <t>01:30</t>
-        </is>
-      </c>
-      <c r="D51" s="46" t="inlineStr">
-        <is>
-          <t>Brezilya</t>
-        </is>
-      </c>
-      <c r="E51" s="46" t="inlineStr">
-        <is>
-          <t>Campeonato Brasileiro Série A</t>
-        </is>
-      </c>
-      <c r="F51" s="47" t="inlineStr">
-        <is>
-          <t>RB Bragantino</t>
-        </is>
-      </c>
-      <c r="G51" s="47" t="inlineStr">
-        <is>
-          <t>Mirassol FC</t>
-        </is>
-      </c>
-      <c r="H51" s="46" t="inlineStr">
-        <is>
-          <t>Planlandı</t>
-        </is>
-      </c>
-      <c r="I51" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J51" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K51" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L51" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M51" s="48" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="N51" s="49" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="O51" s="49" t="n">
-        <v>26.6</v>
-      </c>
-      <c r="P51" s="49" t="n">
-        <v>37.6</v>
-      </c>
-      <c r="Q51" s="50" t="n">
-        <v>1.26</v>
-      </c>
-      <c r="R51" s="50" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="S51" s="49" t="n">
-        <v>47.1</v>
-      </c>
-      <c r="T51" s="49" t="n">
-        <v>52.9</v>
-      </c>
-      <c r="U51" s="49" t="n">
-        <v>52.1</v>
-      </c>
-      <c r="V51" s="49" t="n">
-        <v>47.9</v>
-      </c>
-      <c r="W51" s="49" t="n">
-        <v>72.5</v>
-      </c>
-      <c r="X51" s="49" t="n">
-        <v>62.4</v>
-      </c>
-      <c r="Y51" s="49" t="n">
-        <v>64.2</v>
-      </c>
-      <c r="Z51" s="49" t="n">
-        <v>73.40000000000001</v>
-      </c>
-      <c r="AA51" s="49" t="n">
-        <v>27.4</v>
-      </c>
-      <c r="AB51" s="49" t="n">
-        <v>44</v>
-      </c>
-      <c r="AC51" s="49" t="n">
-        <v>28.5</v>
-      </c>
-      <c r="AD51" s="51" t="inlineStr">
-        <is>
-          <t>1-1 (%13)</t>
-        </is>
-      </c>
-      <c r="AE51" s="46" t="n"/>
-      <c r="AF51" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG51" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AH51" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AI51" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="52" t="inlineStr">
-        <is>
-          <t>08.10.2026</t>
-        </is>
-      </c>
-      <c r="B52" s="52" t="inlineStr">
-        <is>
-          <t>Perşembe</t>
-        </is>
-      </c>
-      <c r="C52" s="52" t="inlineStr">
-        <is>
-          <t>01:30</t>
-        </is>
-      </c>
-      <c r="D52" s="52" t="inlineStr">
-        <is>
-          <t>Brezilya</t>
-        </is>
-      </c>
-      <c r="E52" s="52" t="inlineStr">
-        <is>
-          <t>Campeonato Brasileiro Série A</t>
-        </is>
-      </c>
-      <c r="F52" s="53" t="inlineStr">
-        <is>
-          <t>SC Internacional</t>
-        </is>
-      </c>
-      <c r="G52" s="53" t="inlineStr">
-        <is>
-          <t>SC Corinthians Paulista</t>
-        </is>
-      </c>
-      <c r="H52" s="52" t="inlineStr">
-        <is>
-          <t>Planlandı</t>
-        </is>
-      </c>
-      <c r="I52" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J52" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K52" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L52" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M52" s="54" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N52" s="49" t="n">
-        <v>86.59999999999999</v>
-      </c>
-      <c r="O52" s="49" t="n">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="P52" s="49" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="Q52" s="50" t="n">
-        <v>3.52</v>
-      </c>
-      <c r="R52" s="50" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="S52" s="49" t="n">
-        <v>80.5</v>
-      </c>
-      <c r="T52" s="49" t="n">
-        <v>19.5</v>
-      </c>
-      <c r="U52" s="49" t="n">
-        <v>53.4</v>
-      </c>
-      <c r="V52" s="49" t="n">
-        <v>46.6</v>
-      </c>
-      <c r="W52" s="49" t="n">
-        <v>92.90000000000001</v>
-      </c>
-      <c r="X52" s="49" t="n">
-        <v>95.3</v>
-      </c>
-      <c r="Y52" s="49" t="n">
-        <v>13.4</v>
-      </c>
-      <c r="Z52" s="49" t="n">
-        <v>91.3</v>
-      </c>
-      <c r="AA52" s="49" t="n">
-        <v>67.2</v>
-      </c>
-      <c r="AB52" s="49" t="n">
-        <v>24.7</v>
-      </c>
-      <c r="AC52" s="49" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="AD52" s="51" t="inlineStr">
-        <is>
-          <t>3-0 (%10)</t>
-        </is>
-      </c>
-      <c r="AE52" s="52" t="n"/>
-      <c r="AF52" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG52" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AH52" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AI52" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="46" t="inlineStr">
-        <is>
-          <t>08.10.2026</t>
-        </is>
-      </c>
-      <c r="B53" s="46" t="inlineStr">
-        <is>
-          <t>Perşembe</t>
-        </is>
-      </c>
-      <c r="C53" s="46" t="inlineStr">
-        <is>
-          <t>01:30</t>
-        </is>
-      </c>
-      <c r="D53" s="46" t="inlineStr">
-        <is>
-          <t>Brezilya</t>
-        </is>
-      </c>
-      <c r="E53" s="46" t="inlineStr">
-        <is>
-          <t>Campeonato Brasileiro Série A</t>
-        </is>
-      </c>
-      <c r="F53" s="47" t="inlineStr">
-        <is>
-          <t>Clube do Remo</t>
-        </is>
-      </c>
-      <c r="G53" s="47" t="inlineStr">
-        <is>
-          <t>Grêmio FBPA</t>
-        </is>
-      </c>
-      <c r="H53" s="46" t="inlineStr">
-        <is>
-          <t>Planlandı</t>
-        </is>
-      </c>
-      <c r="I53" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J53" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K53" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L53" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M53" s="48" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="N53" s="49" t="n">
-        <v>33.8</v>
-      </c>
-      <c r="O53" s="49" t="n">
-        <v>25.6</v>
-      </c>
-      <c r="P53" s="49" t="n">
-        <v>40.6</v>
-      </c>
-      <c r="Q53" s="50" t="n">
-        <v>1.29</v>
-      </c>
-      <c r="R53" s="50" t="n">
-        <v>1.44</v>
-      </c>
-      <c r="S53" s="49" t="n">
-        <v>51.2</v>
-      </c>
-      <c r="T53" s="49" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="U53" s="49" t="n">
-        <v>55.2</v>
-      </c>
-      <c r="V53" s="49" t="n">
-        <v>44.8</v>
-      </c>
-      <c r="W53" s="49" t="n">
-        <v>75.5</v>
-      </c>
-      <c r="X53" s="49" t="n">
-        <v>59.4</v>
-      </c>
-      <c r="Y53" s="49" t="n">
-        <v>66.2</v>
-      </c>
-      <c r="Z53" s="49" t="n">
-        <v>74.40000000000001</v>
-      </c>
-      <c r="AA53" s="49" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="AB53" s="49" t="n">
-        <v>42.4</v>
-      </c>
-      <c r="AC53" s="49" t="n">
-        <v>30.8</v>
-      </c>
-      <c r="AD53" s="51" t="inlineStr">
-        <is>
-          <t>1-1 (%12)</t>
-        </is>
-      </c>
-      <c r="AE53" s="46" t="n"/>
-      <c r="AF53" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG53" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AH53" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AI53" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="52" t="inlineStr">
-        <is>
-          <t>08.10.2026</t>
-        </is>
-      </c>
-      <c r="B54" s="52" t="inlineStr">
-        <is>
-          <t>Perşembe</t>
-        </is>
-      </c>
-      <c r="C54" s="52" t="inlineStr">
-        <is>
-          <t>02:00</t>
-        </is>
-      </c>
-      <c r="D54" s="52" t="inlineStr">
-        <is>
-          <t>Brezilya</t>
-        </is>
-      </c>
-      <c r="E54" s="52" t="inlineStr">
-        <is>
-          <t>Campeonato Brasileiro Série A</t>
-        </is>
-      </c>
-      <c r="F54" s="53" t="inlineStr">
-        <is>
-          <t>EC Vitória</t>
-        </is>
-      </c>
-      <c r="G54" s="53" t="inlineStr">
-        <is>
-          <t>Chapecoense AF</t>
-        </is>
-      </c>
-      <c r="H54" s="52" t="inlineStr">
-        <is>
-          <t>Planlandı</t>
-        </is>
-      </c>
-      <c r="I54" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J54" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K54" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L54" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M54" s="54" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N54" s="49" t="n">
-        <v>55</v>
-      </c>
-      <c r="O54" s="49" t="n">
-        <v>20.6</v>
-      </c>
-      <c r="P54" s="49" t="n">
-        <v>24.4</v>
-      </c>
-      <c r="Q54" s="50" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="R54" s="50" t="n">
-        <v>1.39</v>
-      </c>
-      <c r="S54" s="49" t="n">
-        <v>68.7</v>
-      </c>
-      <c r="T54" s="49" t="n">
-        <v>31.3</v>
-      </c>
-      <c r="U54" s="49" t="n">
-        <v>66.40000000000001</v>
-      </c>
-      <c r="V54" s="49" t="n">
-        <v>33.6</v>
-      </c>
-      <c r="W54" s="49" t="n">
-        <v>86.90000000000001</v>
-      </c>
-      <c r="X54" s="49" t="n">
-        <v>75.59999999999999</v>
-      </c>
-      <c r="Y54" s="49" t="n">
-        <v>45</v>
-      </c>
-      <c r="Z54" s="49" t="n">
-        <v>79.40000000000001</v>
-      </c>
-      <c r="AA54" s="49" t="n">
-        <v>41.8</v>
-      </c>
-      <c r="AB54" s="49" t="n">
-        <v>35.5</v>
-      </c>
-      <c r="AC54" s="49" t="n">
-        <v>22.7</v>
-      </c>
-      <c r="AD54" s="51" t="inlineStr">
-        <is>
-          <t>2-1 (%9)</t>
-        </is>
-      </c>
-      <c r="AE54" s="52" t="n"/>
-      <c r="AF54" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG54" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AH54" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AI54" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="46" t="inlineStr">
-        <is>
-          <t>08.10.2026</t>
-        </is>
-      </c>
-      <c r="B55" s="46" t="inlineStr">
-        <is>
-          <t>Perşembe</t>
-        </is>
-      </c>
-      <c r="C55" s="46" t="inlineStr">
-        <is>
-          <t>02:30</t>
-        </is>
-      </c>
-      <c r="D55" s="46" t="inlineStr">
-        <is>
-          <t>Brezilya</t>
-        </is>
-      </c>
-      <c r="E55" s="46" t="inlineStr">
-        <is>
-          <t>Campeonato Brasileiro Série A</t>
-        </is>
-      </c>
-      <c r="F55" s="47" t="inlineStr">
-        <is>
-          <t>Botafogo FR</t>
-        </is>
-      </c>
-      <c r="G55" s="47" t="inlineStr">
-        <is>
-          <t>CR Vasco da Gama</t>
-        </is>
-      </c>
-      <c r="H55" s="46" t="inlineStr">
-        <is>
-          <t>Planlandı</t>
-        </is>
-      </c>
-      <c r="I55" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J55" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K55" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L55" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M55" s="48" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="N55" s="49" t="n">
-        <v>7.7</v>
-      </c>
-      <c r="O55" s="49" t="n">
-        <v>18.1</v>
-      </c>
-      <c r="P55" s="49" t="n">
-        <v>74.2</v>
-      </c>
-      <c r="Q55" s="50" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="R55" s="50" t="n">
-        <v>2.04</v>
-      </c>
-      <c r="S55" s="49" t="n">
-        <v>46.4</v>
-      </c>
-      <c r="T55" s="49" t="n">
-        <v>53.6</v>
-      </c>
-      <c r="U55" s="49" t="n">
-        <v>33.5</v>
-      </c>
-      <c r="V55" s="49" t="n">
-        <v>66.5</v>
-      </c>
-      <c r="W55" s="49" t="n">
-        <v>71.90000000000001</v>
-      </c>
-      <c r="X55" s="49" t="n">
-        <v>25.8</v>
-      </c>
-      <c r="Y55" s="49" t="n">
-        <v>92.3</v>
-      </c>
-      <c r="Z55" s="49" t="n">
-        <v>81.90000000000001</v>
-      </c>
-      <c r="AA55" s="49" t="n">
-        <v>8.6</v>
-      </c>
-      <c r="AB55" s="49" t="n">
-        <v>40.1</v>
-      </c>
-      <c r="AC55" s="49" t="n">
-        <v>51.4</v>
-      </c>
-      <c r="AD55" s="51" t="inlineStr">
-        <is>
-          <t>0-2 (%17)</t>
-        </is>
-      </c>
-      <c r="AE55" s="46" t="n"/>
-      <c r="AF55" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG55" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AH55" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AI55" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:AI55"/>
+  <autoFilter ref="A2:AI50"/>
   <mergeCells count="12">
     <mergeCell ref="X1:Z1"/>
     <mergeCell ref="AA1:AC1"/>
@@ -8432,7 +7739,7 @@
     <row r="3">
       <c r="A3" s="57" t="inlineStr">
         <is>
-          <t>Oluşturulma zamanı: 05.10.2026 02:56</t>
+          <t>Oluşturulma zamanı: 05.10.2026 20:04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Güncel tahmin tablosu: 3-8 Ekim maçları (54 satır, Elo harmanlamalı)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBfpyxGus5xRHHn8xK9mQE
</commit_message>
<xml_diff>
--- a/maclar_ve_tahminler.xlsx
+++ b/maclar_ve_tahminler.xlsx
@@ -5678,7 +5678,7 @@
       </c>
       <c r="AH36" s="41" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18°C, Parçalı bulutlu, 3 km/sa</t>
         </is>
       </c>
       <c r="AI36" s="41" t="inlineStr">
@@ -8555,7 +8555,7 @@
     <row r="3">
       <c r="A3" s="52" t="inlineStr">
         <is>
-          <t>Oluşturulma zamanı: 05.10.2026 21:12</t>
+          <t>Oluşturulma zamanı: 05.10.2026 21:34</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Güncelle: otomatik GitHub Actions güncellemesi (2026-10-14 10:38 UTC)
</commit_message>
<xml_diff>
--- a/maclar_ve_tahminler.xlsx
+++ b/maclar_ve_tahminler.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Maçlar ve Tahminler'!$A$2:$AI$81</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Öne Çıkanlar'!$A$1:$I$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Öne Çıkanlar'!$A$1:$I$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2698,59 +2698,63 @@
         </is>
       </c>
       <c r="N15" s="42" t="n">
-        <v>69.2</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="O15" s="42" t="n">
-        <v>17.1</v>
+        <v>19.6</v>
       </c>
       <c r="P15" s="42" t="n">
-        <v>13.8</v>
+        <v>16.1</v>
       </c>
       <c r="Q15" s="43" t="n">
-        <v>3.02</v>
+        <v>2.57</v>
       </c>
       <c r="R15" s="43" t="n">
         <v>1.04</v>
       </c>
       <c r="S15" s="42" t="n">
-        <v>64.90000000000001</v>
+        <v>60.9</v>
       </c>
       <c r="T15" s="42" t="n">
-        <v>35.1</v>
+        <v>39.1</v>
       </c>
       <c r="U15" s="42" t="n">
-        <v>59.2</v>
+        <v>58.4</v>
       </c>
       <c r="V15" s="42" t="n">
-        <v>40.8</v>
+        <v>41.6</v>
       </c>
       <c r="W15" s="42" t="n">
-        <v>91.7</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="X15" s="42" t="n">
-        <v>86.2</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="Y15" s="42" t="n">
-        <v>30.8</v>
+        <v>35.6</v>
       </c>
       <c r="Z15" s="42" t="n">
-        <v>82.90000000000001</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="AA15" s="42" t="n">
-        <v>59.2</v>
+        <v>53.1</v>
       </c>
       <c r="AB15" s="42" t="n">
-        <v>28.1</v>
+        <v>31.9</v>
       </c>
       <c r="AC15" s="42" t="n">
-        <v>12.7</v>
+        <v>15</v>
       </c>
       <c r="AD15" s="44" t="inlineStr">
         <is>
-          <t>3-1 (%8)</t>
-        </is>
-      </c>
-      <c r="AE15" s="39" t="n"/>
+          <t>2-1 (%9)</t>
+        </is>
+      </c>
+      <c r="AE15" s="39" t="inlineStr">
+        <is>
+          <t>Ev kilit oyuncu eksik (Yaldir P.) -&gt; hücum -%15</t>
+        </is>
+      </c>
       <c r="AF15" s="39" t="inlineStr">
         <is>
           <t>Guldibi O.</t>
@@ -2763,12 +2767,13 @@
       </c>
       <c r="AH15" s="39" t="inlineStr">
         <is>
-          <t>26°C, Bulutlu, 14 km/sa</t>
+          <t>26°C, Bulutlu, 12 km/sa</t>
         </is>
       </c>
       <c r="AI15" s="39" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Kesin) Tetik, Altiparmak, Artan, Benny, Biron, Cagiran, Gurbulak, Jo, Matheus Doria, Mert, Subasi
+DEP: (Kesin) Tutar, Cham, Duymaz, Fall, Mendy, Nizam, Ologo Inainfe, Sahin, Sonmez, Tuncer, Uzunhan</t>
         </is>
       </c>
     </row>
@@ -2904,7 +2909,7 @@
       </c>
       <c r="AH16" s="45" t="inlineStr">
         <is>
-          <t>18°C, Sağanak, 27 km/sa</t>
+          <t>18°C, Gök gürültülü sağanak, 20 km/sa</t>
         </is>
       </c>
       <c r="AI16" s="45" t="inlineStr">
@@ -3045,7 +3050,7 @@
       </c>
       <c r="AH17" s="39" t="inlineStr">
         <is>
-          <t>16°C, Bulutlu, 7 km/sa</t>
+          <t>16°C, Bulutlu, 8 km/sa</t>
         </is>
       </c>
       <c r="AI17" s="39" t="inlineStr">
@@ -3186,7 +3191,7 @@
       </c>
       <c r="AH18" s="45" t="inlineStr">
         <is>
-          <t>18°C, Bulutlu, 13 km/sa</t>
+          <t>17°C, Bulutlu, 12 km/sa</t>
         </is>
       </c>
       <c r="AI18" s="45" t="inlineStr">
@@ -3327,7 +3332,7 @@
       </c>
       <c r="AH19" s="39" t="inlineStr">
         <is>
-          <t>17°C, Gök gürültülü sağanak, 9 km/sa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AI19" s="39" t="inlineStr">
@@ -3468,7 +3473,7 @@
       </c>
       <c r="AH20" s="45" t="inlineStr">
         <is>
-          <t>13°C, Hafif yağmur, 6 km/sa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AI20" s="45" t="inlineStr">
@@ -11863,56 +11868,56 @@
         </is>
       </c>
       <c r="N80" s="42" t="n">
-        <v>59.5</v>
+        <v>58.4</v>
       </c>
       <c r="O80" s="42" t="n">
-        <v>20.5</v>
+        <v>21.7</v>
       </c>
       <c r="P80" s="42" t="n">
-        <v>20</v>
+        <v>19.8</v>
       </c>
       <c r="Q80" s="43" t="n">
-        <v>2.75</v>
+        <v>2.35</v>
       </c>
       <c r="R80" s="43" t="n">
-        <v>1.36</v>
+        <v>1.12</v>
       </c>
       <c r="S80" s="42" t="n">
-        <v>65.3</v>
+        <v>59.8</v>
       </c>
       <c r="T80" s="42" t="n">
-        <v>34.7</v>
+        <v>40.2</v>
       </c>
       <c r="U80" s="42" t="n">
-        <v>63.3</v>
+        <v>59</v>
       </c>
       <c r="V80" s="42" t="n">
-        <v>36.7</v>
+        <v>41</v>
       </c>
       <c r="W80" s="42" t="n">
-        <v>92.09999999999999</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="X80" s="42" t="n">
-        <v>80</v>
+        <v>80.2</v>
       </c>
       <c r="Y80" s="42" t="n">
-        <v>40.5</v>
+        <v>41.6</v>
       </c>
       <c r="Z80" s="42" t="n">
-        <v>79.5</v>
+        <v>78.3</v>
       </c>
       <c r="AA80" s="42" t="n">
-        <v>49.7</v>
+        <v>47.8</v>
       </c>
       <c r="AB80" s="42" t="n">
-        <v>32.1</v>
+        <v>35</v>
       </c>
       <c r="AC80" s="42" t="n">
-        <v>18.2</v>
+        <v>17.3</v>
       </c>
       <c r="AD80" s="44" t="inlineStr">
         <is>
-          <t>2-1 (%8)</t>
+          <t>2-1 (%10)</t>
         </is>
       </c>
       <c r="AE80" s="45" t="n"/>
@@ -12104,7 +12109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12458,27 +12463,27 @@
       </c>
       <c r="B9" s="44" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C9" s="44" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Avrupa</t>
         </is>
       </c>
       <c r="D9" s="44" t="inlineStr">
         <is>
-          <t>TFF 1. Lig</t>
+          <t>UEFA Champions League</t>
         </is>
       </c>
       <c r="E9" s="50" t="inlineStr">
         <is>
-          <t>Batman Petrolspor</t>
+          <t>AS Roma</t>
         </is>
       </c>
       <c r="F9" s="50" t="inlineStr">
         <is>
-          <t>Istanbulspor AS</t>
+          <t>Real Madrid CF</t>
         </is>
       </c>
       <c r="G9" s="44" t="inlineStr">
@@ -12492,52 +12497,52 @@
         </is>
       </c>
       <c r="I9" s="51" t="n">
-        <v>91.7</v>
+        <v>90.3</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="44" t="inlineStr">
+      <c r="A10" s="52" t="inlineStr">
         <is>
           <t>14.10.2026</t>
         </is>
       </c>
-      <c r="B10" s="44" t="inlineStr">
+      <c r="B10" s="52" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C10" s="44" t="inlineStr">
+      <c r="C10" s="52" t="inlineStr">
         <is>
           <t>Avrupa</t>
         </is>
       </c>
-      <c r="D10" s="44" t="inlineStr">
+      <c r="D10" s="52" t="inlineStr">
         <is>
           <t>UEFA Champions League</t>
         </is>
       </c>
-      <c r="E10" s="50" t="inlineStr">
-        <is>
-          <t>AS Roma</t>
-        </is>
-      </c>
-      <c r="F10" s="50" t="inlineStr">
-        <is>
-          <t>Real Madrid CF</t>
-        </is>
-      </c>
-      <c r="G10" s="44" t="inlineStr">
-        <is>
-          <t>1.5 Üst</t>
-        </is>
-      </c>
-      <c r="H10" s="44" t="inlineStr">
-        <is>
-          <t>Üst</t>
-        </is>
-      </c>
-      <c r="I10" s="51" t="n">
-        <v>90.3</v>
+      <c r="E10" s="53" t="inlineStr">
+        <is>
+          <t>Real Betis Balompié</t>
+        </is>
+      </c>
+      <c r="F10" s="53" t="inlineStr">
+        <is>
+          <t>FC Porto</t>
+        </is>
+      </c>
+      <c r="G10" s="52" t="inlineStr">
+        <is>
+          <t>Çifte Şans</t>
+        </is>
+      </c>
+      <c r="H10" s="52" t="inlineStr">
+        <is>
+          <t>1X</t>
+        </is>
+      </c>
+      <c r="I10" s="54" t="n">
+        <v>86.90000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -12548,27 +12553,27 @@
       </c>
       <c r="B11" s="52" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C11" s="52" t="inlineStr">
         <is>
-          <t>Avrupa</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="D11" s="52" t="inlineStr">
         <is>
-          <t>UEFA Champions League</t>
+          <t>TFF 1. Lig</t>
         </is>
       </c>
       <c r="E11" s="53" t="inlineStr">
         <is>
-          <t>Real Betis Balompié</t>
+          <t>Umraniyespor</t>
         </is>
       </c>
       <c r="F11" s="53" t="inlineStr">
         <is>
-          <t>FC Porto</t>
+          <t>Boluspor</t>
         </is>
       </c>
       <c r="G11" s="52" t="inlineStr">
@@ -12582,7 +12587,7 @@
         </is>
       </c>
       <c r="I11" s="54" t="n">
-        <v>86.90000000000001</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12">
@@ -12593,27 +12598,27 @@
       </c>
       <c r="B12" s="52" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C12" s="52" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Avrupa</t>
         </is>
       </c>
       <c r="D12" s="52" t="inlineStr">
         <is>
-          <t>TFF 1. Lig</t>
+          <t>UEFA Champions League</t>
         </is>
       </c>
       <c r="E12" s="53" t="inlineStr">
         <is>
-          <t>Batman Petrolspor</t>
+          <t>Aston Villa FC</t>
         </is>
       </c>
       <c r="F12" s="53" t="inlineStr">
         <is>
-          <t>Istanbulspor AS</t>
+          <t>Fenerbahçe SK</t>
         </is>
       </c>
       <c r="G12" s="52" t="inlineStr">
@@ -12627,7 +12632,7 @@
         </is>
       </c>
       <c r="I12" s="54" t="n">
-        <v>86.2</v>
+        <v>84.40000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -12638,7 +12643,7 @@
       </c>
       <c r="B13" s="52" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="C13" s="52" t="inlineStr">
@@ -12653,12 +12658,12 @@
       </c>
       <c r="E13" s="53" t="inlineStr">
         <is>
-          <t>Umraniyespor</t>
+          <t>Batman Petrolspor</t>
         </is>
       </c>
       <c r="F13" s="53" t="inlineStr">
         <is>
-          <t>Boluspor</t>
+          <t>Istanbulspor AS</t>
         </is>
       </c>
       <c r="G13" s="52" t="inlineStr">
@@ -12672,7 +12677,7 @@
         </is>
       </c>
       <c r="I13" s="54" t="n">
-        <v>86</v>
+        <v>83.90000000000001</v>
       </c>
     </row>
     <row r="14">
@@ -12698,12 +12703,12 @@
       </c>
       <c r="E14" s="53" t="inlineStr">
         <is>
-          <t>Aston Villa FC</t>
+          <t>Manchester City FC</t>
         </is>
       </c>
       <c r="F14" s="53" t="inlineStr">
         <is>
-          <t>Fenerbahçe SK</t>
+          <t>Paris Saint-Germain FC</t>
         </is>
       </c>
       <c r="G14" s="52" t="inlineStr">
@@ -12713,11 +12718,11 @@
       </c>
       <c r="H14" s="52" t="inlineStr">
         <is>
-          <t>1X</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I14" s="54" t="n">
-        <v>84.40000000000001</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15">
@@ -12743,12 +12748,12 @@
       </c>
       <c r="E15" s="53" t="inlineStr">
         <is>
-          <t>Manchester City FC</t>
+          <t>AS Roma</t>
         </is>
       </c>
       <c r="F15" s="53" t="inlineStr">
         <is>
-          <t>Paris Saint-Germain FC</t>
+          <t>Real Madrid CF</t>
         </is>
       </c>
       <c r="G15" s="52" t="inlineStr">
@@ -12758,72 +12763,72 @@
       </c>
       <c r="H15" s="52" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>1X</t>
         </is>
       </c>
       <c r="I15" s="54" t="n">
-        <v>81</v>
+        <v>80.5</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="52" t="inlineStr">
-        <is>
-          <t>14.10.2026</t>
-        </is>
-      </c>
-      <c r="B16" s="52" t="inlineStr">
-        <is>
-          <t>22:00</t>
-        </is>
-      </c>
-      <c r="C16" s="52" t="inlineStr">
+      <c r="A16" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  15.10.2026</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="44" t="inlineStr">
+        <is>
+          <t>15.10.2026</t>
+        </is>
+      </c>
+      <c r="B17" s="44" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="C17" s="44" t="inlineStr">
         <is>
           <t>Avrupa</t>
         </is>
       </c>
-      <c r="D16" s="52" t="inlineStr">
-        <is>
-          <t>UEFA Champions League</t>
-        </is>
-      </c>
-      <c r="E16" s="53" t="inlineStr">
-        <is>
-          <t>AS Roma</t>
-        </is>
-      </c>
-      <c r="F16" s="53" t="inlineStr">
-        <is>
-          <t>Real Madrid CF</t>
-        </is>
-      </c>
-      <c r="G16" s="52" t="inlineStr">
-        <is>
-          <t>Çifte Şans</t>
-        </is>
-      </c>
-      <c r="H16" s="52" t="inlineStr">
-        <is>
-          <t>1X</t>
-        </is>
-      </c>
-      <c r="I16" s="54" t="n">
-        <v>80.5</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  15.10.2026</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="n"/>
-      <c r="C17" s="6" t="n"/>
-      <c r="D17" s="6" t="n"/>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="6" t="n"/>
-      <c r="G17" s="6" t="n"/>
-      <c r="H17" s="6" t="n"/>
-      <c r="I17" s="6" t="n"/>
+      <c r="D17" s="44" t="inlineStr">
+        <is>
+          <t>UEFA Avrupa Ligi</t>
+        </is>
+      </c>
+      <c r="E17" s="50" t="inlineStr">
+        <is>
+          <t>Sparta Prague</t>
+        </is>
+      </c>
+      <c r="F17" s="50" t="inlineStr">
+        <is>
+          <t>Lillestrom</t>
+        </is>
+      </c>
+      <c r="G17" s="44" t="inlineStr">
+        <is>
+          <t>1.5 Üst</t>
+        </is>
+      </c>
+      <c r="H17" s="44" t="inlineStr">
+        <is>
+          <t>Üst</t>
+        </is>
+      </c>
+      <c r="I17" s="51" t="n">
+        <v>93.3</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="44" t="inlineStr">
@@ -12833,7 +12838,7 @@
       </c>
       <c r="B18" s="44" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C18" s="44" t="inlineStr">
@@ -12848,12 +12853,12 @@
       </c>
       <c r="E18" s="50" t="inlineStr">
         <is>
-          <t>Sparta Prague</t>
+          <t>Ferencvaros</t>
         </is>
       </c>
       <c r="F18" s="50" t="inlineStr">
         <is>
-          <t>Lillestrom</t>
+          <t>Plzen</t>
         </is>
       </c>
       <c r="G18" s="44" t="inlineStr">
@@ -12867,7 +12872,7 @@
         </is>
       </c>
       <c r="I18" s="51" t="n">
-        <v>93.3</v>
+        <v>93.09999999999999</v>
       </c>
     </row>
     <row r="19">
@@ -12893,12 +12898,12 @@
       </c>
       <c r="E19" s="50" t="inlineStr">
         <is>
-          <t>Ferencvaros</t>
+          <t>Jagiellonia</t>
         </is>
       </c>
       <c r="F19" s="50" t="inlineStr">
         <is>
-          <t>Plzen</t>
+          <t>Ararat-Armenia</t>
         </is>
       </c>
       <c r="G19" s="44" t="inlineStr">
@@ -12912,7 +12917,7 @@
         </is>
       </c>
       <c r="I19" s="51" t="n">
-        <v>93.09999999999999</v>
+        <v>90.90000000000001</v>
       </c>
     </row>
     <row r="20">
@@ -12923,7 +12928,7 @@
       </c>
       <c r="B20" s="44" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="C20" s="44" t="inlineStr">
@@ -12938,12 +12943,12 @@
       </c>
       <c r="E20" s="50" t="inlineStr">
         <is>
-          <t>Jagiellonia</t>
+          <t>Royale Union SG</t>
         </is>
       </c>
       <c r="F20" s="50" t="inlineStr">
         <is>
-          <t>Ararat-Armenia</t>
+          <t>Real Sociedad</t>
         </is>
       </c>
       <c r="G20" s="44" t="inlineStr">
@@ -12957,7 +12962,7 @@
         </is>
       </c>
       <c r="I20" s="51" t="n">
-        <v>90.90000000000001</v>
+        <v>90.2</v>
       </c>
     </row>
     <row r="21">
@@ -12968,7 +12973,7 @@
       </c>
       <c r="B21" s="44" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C21" s="44" t="inlineStr">
@@ -12983,12 +12988,12 @@
       </c>
       <c r="E21" s="50" t="inlineStr">
         <is>
-          <t>Royale Union SG</t>
+          <t>Benfica</t>
         </is>
       </c>
       <c r="F21" s="50" t="inlineStr">
         <is>
-          <t>Real Sociedad</t>
+          <t>Celtic</t>
         </is>
       </c>
       <c r="G21" s="44" t="inlineStr">
@@ -13006,48 +13011,48 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="44" t="inlineStr">
+      <c r="A22" s="52" t="inlineStr">
         <is>
           <t>15.10.2026</t>
         </is>
       </c>
-      <c r="B22" s="44" t="inlineStr">
+      <c r="B22" s="52" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C22" s="44" t="inlineStr">
+      <c r="C22" s="52" t="inlineStr">
         <is>
           <t>Avrupa</t>
         </is>
       </c>
-      <c r="D22" s="44" t="inlineStr">
+      <c r="D22" s="52" t="inlineStr">
         <is>
           <t>UEFA Avrupa Ligi</t>
         </is>
       </c>
-      <c r="E22" s="50" t="inlineStr">
-        <is>
-          <t>Benfica</t>
-        </is>
-      </c>
-      <c r="F22" s="50" t="inlineStr">
-        <is>
-          <t>Celtic</t>
-        </is>
-      </c>
-      <c r="G22" s="44" t="inlineStr">
-        <is>
-          <t>1.5 Üst</t>
-        </is>
-      </c>
-      <c r="H22" s="44" t="inlineStr">
-        <is>
-          <t>Üst</t>
-        </is>
-      </c>
-      <c r="I22" s="51" t="n">
-        <v>90.2</v>
+      <c r="E22" s="53" t="inlineStr">
+        <is>
+          <t>Ferencvaros</t>
+        </is>
+      </c>
+      <c r="F22" s="53" t="inlineStr">
+        <is>
+          <t>Plzen</t>
+        </is>
+      </c>
+      <c r="G22" s="52" t="inlineStr">
+        <is>
+          <t>Çifte Şans</t>
+        </is>
+      </c>
+      <c r="H22" s="52" t="inlineStr">
+        <is>
+          <t>1X</t>
+        </is>
+      </c>
+      <c r="I22" s="54" t="n">
+        <v>88.40000000000001</v>
       </c>
     </row>
     <row r="23">
@@ -13058,7 +13063,7 @@
       </c>
       <c r="B23" s="52" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="C23" s="52" t="inlineStr">
@@ -13073,12 +13078,12 @@
       </c>
       <c r="E23" s="53" t="inlineStr">
         <is>
-          <t>Ferencvaros</t>
+          <t>Sparta Prague</t>
         </is>
       </c>
       <c r="F23" s="53" t="inlineStr">
         <is>
-          <t>Plzen</t>
+          <t>Lillestrom</t>
         </is>
       </c>
       <c r="G23" s="52" t="inlineStr">
@@ -13092,7 +13097,7 @@
         </is>
       </c>
       <c r="I23" s="54" t="n">
-        <v>88.40000000000001</v>
+        <v>87.59999999999999</v>
       </c>
     </row>
     <row r="24">
@@ -13118,12 +13123,12 @@
       </c>
       <c r="E24" s="53" t="inlineStr">
         <is>
-          <t>Sparta Prague</t>
+          <t>Royale Union SG</t>
         </is>
       </c>
       <c r="F24" s="53" t="inlineStr">
         <is>
-          <t>Lillestrom</t>
+          <t>Real Sociedad</t>
         </is>
       </c>
       <c r="G24" s="52" t="inlineStr">
@@ -13137,7 +13142,7 @@
         </is>
       </c>
       <c r="I24" s="54" t="n">
-        <v>87.59999999999999</v>
+        <v>87.09999999999999</v>
       </c>
     </row>
     <row r="25">
@@ -13148,7 +13153,7 @@
       </c>
       <c r="B25" s="52" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C25" s="52" t="inlineStr">
@@ -13163,12 +13168,12 @@
       </c>
       <c r="E25" s="53" t="inlineStr">
         <is>
-          <t>Royale Union SG</t>
+          <t>Benfica</t>
         </is>
       </c>
       <c r="F25" s="53" t="inlineStr">
         <is>
-          <t>Real Sociedad</t>
+          <t>Celtic</t>
         </is>
       </c>
       <c r="G25" s="52" t="inlineStr">
@@ -13193,7 +13198,7 @@
       </c>
       <c r="B26" s="52" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="C26" s="52" t="inlineStr">
@@ -13208,12 +13213,12 @@
       </c>
       <c r="E26" s="53" t="inlineStr">
         <is>
-          <t>Benfica</t>
+          <t>Salzburg</t>
         </is>
       </c>
       <c r="F26" s="53" t="inlineStr">
         <is>
-          <t>Celtic</t>
+          <t>AC Milan</t>
         </is>
       </c>
       <c r="G26" s="52" t="inlineStr">
@@ -13227,7 +13232,7 @@
         </is>
       </c>
       <c r="I26" s="54" t="n">
-        <v>87.09999999999999</v>
+        <v>84.90000000000001</v>
       </c>
     </row>
     <row r="27">
@@ -13238,7 +13243,7 @@
       </c>
       <c r="B27" s="52" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C27" s="52" t="inlineStr">
@@ -13253,12 +13258,12 @@
       </c>
       <c r="E27" s="53" t="inlineStr">
         <is>
-          <t>Salzburg</t>
+          <t>Jagiellonia</t>
         </is>
       </c>
       <c r="F27" s="53" t="inlineStr">
         <is>
-          <t>AC Milan</t>
+          <t>Ararat-Armenia</t>
         </is>
       </c>
       <c r="G27" s="52" t="inlineStr">
@@ -13272,7 +13277,7 @@
         </is>
       </c>
       <c r="I27" s="54" t="n">
-        <v>84.90000000000001</v>
+        <v>84.59999999999999</v>
       </c>
     </row>
     <row r="28">
@@ -13298,12 +13303,12 @@
       </c>
       <c r="E28" s="53" t="inlineStr">
         <is>
-          <t>Jagiellonia</t>
+          <t>Bournemouth</t>
         </is>
       </c>
       <c r="F28" s="53" t="inlineStr">
         <is>
-          <t>Ararat-Armenia</t>
+          <t>Sturm Graz</t>
         </is>
       </c>
       <c r="G28" s="52" t="inlineStr">
@@ -13317,7 +13322,7 @@
         </is>
       </c>
       <c r="I28" s="54" t="n">
-        <v>84.59999999999999</v>
+        <v>81.2</v>
       </c>
     </row>
     <row r="29">
@@ -13343,12 +13348,12 @@
       </c>
       <c r="E29" s="53" t="inlineStr">
         <is>
-          <t>Bournemouth</t>
+          <t>Din. Zagreb</t>
         </is>
       </c>
       <c r="F29" s="53" t="inlineStr">
         <is>
-          <t>Sturm Graz</t>
+          <t>Anderlecht</t>
         </is>
       </c>
       <c r="G29" s="52" t="inlineStr">
@@ -13366,64 +13371,64 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="52" t="inlineStr">
-        <is>
-          <t>15.10.2026</t>
-        </is>
-      </c>
-      <c r="B30" s="52" t="inlineStr">
-        <is>
-          <t>22:00</t>
-        </is>
-      </c>
-      <c r="C30" s="52" t="inlineStr">
-        <is>
-          <t>Avrupa</t>
-        </is>
-      </c>
-      <c r="D30" s="52" t="inlineStr">
-        <is>
-          <t>UEFA Avrupa Ligi</t>
-        </is>
-      </c>
-      <c r="E30" s="53" t="inlineStr">
-        <is>
-          <t>Din. Zagreb</t>
-        </is>
-      </c>
-      <c r="F30" s="53" t="inlineStr">
-        <is>
-          <t>Anderlecht</t>
-        </is>
-      </c>
-      <c r="G30" s="52" t="inlineStr">
-        <is>
-          <t>Çifte Şans</t>
-        </is>
-      </c>
-      <c r="H30" s="52" t="inlineStr">
-        <is>
-          <t>1X</t>
-        </is>
-      </c>
-      <c r="I30" s="54" t="n">
-        <v>81.2</v>
-      </c>
+      <c r="A30" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  16.10.2026</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="n"/>
+      <c r="C30" s="6" t="n"/>
+      <c r="D30" s="6" t="n"/>
+      <c r="E30" s="6" t="n"/>
+      <c r="F30" s="6" t="n"/>
+      <c r="G30" s="6" t="n"/>
+      <c r="H30" s="6" t="n"/>
+      <c r="I30" s="6" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  16.10.2026</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="n"/>
-      <c r="C31" s="6" t="n"/>
-      <c r="D31" s="6" t="n"/>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="6" t="n"/>
-      <c r="G31" s="6" t="n"/>
-      <c r="H31" s="6" t="n"/>
-      <c r="I31" s="6" t="n"/>
+      <c r="A31" s="44" t="inlineStr">
+        <is>
+          <t>16.10.2026</t>
+        </is>
+      </c>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C31" s="44" t="inlineStr">
+        <is>
+          <t>Almanya</t>
+        </is>
+      </c>
+      <c r="D31" s="44" t="inlineStr">
+        <is>
+          <t>2. Bundesliga</t>
+        </is>
+      </c>
+      <c r="E31" s="50" t="inlineStr">
+        <is>
+          <t>Cottbus</t>
+        </is>
+      </c>
+      <c r="F31" s="50" t="inlineStr">
+        <is>
+          <t>Nurnberg</t>
+        </is>
+      </c>
+      <c r="G31" s="44" t="inlineStr">
+        <is>
+          <t>1.5 Üst</t>
+        </is>
+      </c>
+      <c r="H31" s="44" t="inlineStr">
+        <is>
+          <t>Üst</t>
+        </is>
+      </c>
+      <c r="I31" s="51" t="n">
+        <v>95.59999999999999</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="44" t="inlineStr">
@@ -13433,7 +13438,7 @@
       </c>
       <c r="B32" s="44" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C32" s="44" t="inlineStr">
@@ -13443,17 +13448,17 @@
       </c>
       <c r="D32" s="44" t="inlineStr">
         <is>
-          <t>2. Bundesliga</t>
+          <t>Bundesliga</t>
         </is>
       </c>
       <c r="E32" s="50" t="inlineStr">
         <is>
-          <t>Cottbus</t>
+          <t>Eintracht Frankfurt</t>
         </is>
       </c>
       <c r="F32" s="50" t="inlineStr">
         <is>
-          <t>Nurnberg</t>
+          <t>1. FC Köln</t>
         </is>
       </c>
       <c r="G32" s="44" t="inlineStr">
@@ -13467,7 +13472,7 @@
         </is>
       </c>
       <c r="I32" s="51" t="n">
-        <v>95.59999999999999</v>
+        <v>92.8</v>
       </c>
     </row>
     <row r="33">
@@ -13478,27 +13483,27 @@
       </c>
       <c r="B33" s="44" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="C33" s="44" t="inlineStr">
         <is>
-          <t>Almanya</t>
+          <t>Fransa</t>
         </is>
       </c>
       <c r="D33" s="44" t="inlineStr">
         <is>
-          <t>Bundesliga</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="E33" s="50" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt</t>
+          <t>Le Mans FC</t>
         </is>
       </c>
       <c r="F33" s="50" t="inlineStr">
         <is>
-          <t>1. FC Köln</t>
+          <t>Toulouse FC</t>
         </is>
       </c>
       <c r="G33" s="44" t="inlineStr">
@@ -13512,195 +13517,105 @@
         </is>
       </c>
       <c r="I33" s="51" t="n">
-        <v>92.8</v>
+        <v>90.8</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="44" t="inlineStr">
+      <c r="A34" s="52" t="inlineStr">
         <is>
           <t>16.10.2026</t>
         </is>
       </c>
-      <c r="B34" s="44" t="inlineStr">
+      <c r="B34" s="52" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C34" s="52" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="D34" s="52" t="inlineStr">
+        <is>
+          <t>Süper Lig</t>
+        </is>
+      </c>
+      <c r="E34" s="53" t="inlineStr">
+        <is>
+          <t>Corum</t>
+        </is>
+      </c>
+      <c r="F34" s="53" t="inlineStr">
+        <is>
+          <t>Rizespor</t>
+        </is>
+      </c>
+      <c r="G34" s="52" t="inlineStr">
+        <is>
+          <t>Çifte Şans</t>
+        </is>
+      </c>
+      <c r="H34" s="52" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I34" s="54" t="n">
+        <v>81.59999999999999</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="52" t="inlineStr">
+        <is>
+          <t>16.10.2026</t>
+        </is>
+      </c>
+      <c r="B35" s="52" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C34" s="44" t="inlineStr">
+      <c r="C35" s="52" t="inlineStr">
         <is>
           <t>İspanya</t>
         </is>
       </c>
-      <c r="D34" s="44" t="inlineStr">
+      <c r="D35" s="52" t="inlineStr">
         <is>
           <t>Primera Division</t>
         </is>
       </c>
-      <c r="E34" s="50" t="inlineStr">
+      <c r="E35" s="53" t="inlineStr">
         <is>
           <t>RC Deportivo La Coruña</t>
         </is>
       </c>
-      <c r="F34" s="50" t="inlineStr">
+      <c r="F35" s="53" t="inlineStr">
         <is>
           <t>Levante UD</t>
         </is>
       </c>
-      <c r="G34" s="44" t="inlineStr">
-        <is>
-          <t>1.5 Üst</t>
-        </is>
-      </c>
-      <c r="H34" s="44" t="inlineStr">
-        <is>
-          <t>Üst</t>
-        </is>
-      </c>
-      <c r="I34" s="51" t="n">
-        <v>92.09999999999999</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="44" t="inlineStr">
-        <is>
-          <t>16.10.2026</t>
-        </is>
-      </c>
-      <c r="B35" s="44" t="inlineStr">
-        <is>
-          <t>21:45</t>
-        </is>
-      </c>
-      <c r="C35" s="44" t="inlineStr">
-        <is>
-          <t>Fransa</t>
-        </is>
-      </c>
-      <c r="D35" s="44" t="inlineStr">
-        <is>
-          <t>Ligue 1</t>
-        </is>
-      </c>
-      <c r="E35" s="50" t="inlineStr">
-        <is>
-          <t>Le Mans FC</t>
-        </is>
-      </c>
-      <c r="F35" s="50" t="inlineStr">
-        <is>
-          <t>Toulouse FC</t>
-        </is>
-      </c>
-      <c r="G35" s="44" t="inlineStr">
-        <is>
-          <t>1.5 Üst</t>
-        </is>
-      </c>
-      <c r="H35" s="44" t="inlineStr">
-        <is>
-          <t>Üst</t>
-        </is>
-      </c>
-      <c r="I35" s="51" t="n">
-        <v>90.8</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="52" t="inlineStr">
-        <is>
-          <t>16.10.2026</t>
-        </is>
-      </c>
-      <c r="B36" s="52" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="C36" s="52" t="inlineStr">
-        <is>
-          <t>Türkiye</t>
-        </is>
-      </c>
-      <c r="D36" s="52" t="inlineStr">
-        <is>
-          <t>Süper Lig</t>
-        </is>
-      </c>
-      <c r="E36" s="53" t="inlineStr">
-        <is>
-          <t>Corum</t>
-        </is>
-      </c>
-      <c r="F36" s="53" t="inlineStr">
-        <is>
-          <t>Rizespor</t>
-        </is>
-      </c>
-      <c r="G36" s="52" t="inlineStr">
+      <c r="G35" s="52" t="inlineStr">
         <is>
           <t>Çifte Şans</t>
         </is>
       </c>
-      <c r="H36" s="52" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="I36" s="54" t="n">
-        <v>81.59999999999999</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="52" t="inlineStr">
-        <is>
-          <t>16.10.2026</t>
-        </is>
-      </c>
-      <c r="B37" s="52" t="inlineStr">
-        <is>
-          <t>22:00</t>
-        </is>
-      </c>
-      <c r="C37" s="52" t="inlineStr">
-        <is>
-          <t>İspanya</t>
-        </is>
-      </c>
-      <c r="D37" s="52" t="inlineStr">
-        <is>
-          <t>Primera Division</t>
-        </is>
-      </c>
-      <c r="E37" s="53" t="inlineStr">
-        <is>
-          <t>RC Deportivo La Coruña</t>
-        </is>
-      </c>
-      <c r="F37" s="53" t="inlineStr">
-        <is>
-          <t>Levante UD</t>
-        </is>
-      </c>
-      <c r="G37" s="52" t="inlineStr">
-        <is>
-          <t>Çifte Şans</t>
-        </is>
-      </c>
-      <c r="H37" s="52" t="inlineStr">
+      <c r="H35" s="52" t="inlineStr">
         <is>
           <t>1X</t>
         </is>
       </c>
-      <c r="I37" s="54" t="n">
-        <v>80</v>
+      <c r="I35" s="54" t="n">
+        <v>80.2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I37"/>
+  <autoFilter ref="A1:I35"/>
   <mergeCells count="3">
-    <mergeCell ref="A17:I17"/>
-    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="A30:I30"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A16:I16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13731,7 +13646,7 @@
     <row r="3">
       <c r="A3" s="56" t="inlineStr">
         <is>
-          <t>Oluşturulma zamanı: 14.10.2026 08:35</t>
+          <t>Oluşturulma zamanı: 14.10.2026 13:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Güncelle: otomatik GitHub Actions güncellemesi (2026-10-15 10:38 UTC)
</commit_message>
<xml_diff>
--- a/maclar_ve_tahminler.xlsx
+++ b/maclar_ve_tahminler.xlsx
@@ -5095,7 +5095,7 @@
       </c>
       <c r="AH32" s="40" t="inlineStr">
         <is>
-          <t>23°C, Bulutlu, 15 km/sa</t>
+          <t>22°C, Parçalı bulutlu, 9 km/sa</t>
         </is>
       </c>
       <c r="AI32" s="40" t="inlineStr">
@@ -5236,7 +5236,7 @@
       </c>
       <c r="AH33" s="46" t="inlineStr">
         <is>
-          <t>18°C, Bulutlu, 20 km/sa</t>
+          <t>18°C, Bulutlu, 17 km/sa</t>
         </is>
       </c>
       <c r="AI33" s="46" t="inlineStr">
@@ -5377,7 +5377,7 @@
       </c>
       <c r="AH34" s="40" t="inlineStr">
         <is>
-          <t>17°C, Bulutlu, 5 km/sa</t>
+          <t>16°C, Parçalı bulutlu, 4 km/sa</t>
         </is>
       </c>
       <c r="AI34" s="40" t="inlineStr">
@@ -5518,7 +5518,7 @@
       </c>
       <c r="AH35" s="46" t="inlineStr">
         <is>
-          <t>12°C, Bulutlu, 4 km/sa</t>
+          <t>12°C, Bulutlu, 5 km/sa</t>
         </is>
       </c>
       <c r="AI35" s="46" t="inlineStr">
@@ -5659,7 +5659,7 @@
       </c>
       <c r="AH36" s="40" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22°C, Açık, 3 km/sa</t>
         </is>
       </c>
       <c r="AI36" s="40" t="inlineStr">
@@ -5800,7 +5800,7 @@
       </c>
       <c r="AH37" s="46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>20°C, Bulutlu, 8 km/sa</t>
         </is>
       </c>
       <c r="AI37" s="46" t="inlineStr">
@@ -6213,7 +6213,7 @@
       <c r="AE40" s="40" t="n"/>
       <c r="AF40" s="40" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Jorgji E.</t>
         </is>
       </c>
       <c r="AG40" s="40" t="inlineStr">
@@ -21227,7 +21227,7 @@
     <row r="3">
       <c r="A3" s="57" t="inlineStr">
         <is>
-          <t>Oluşturulma zamanı: 15.10.2026 08:36</t>
+          <t>Oluşturulma zamanı: 15.10.2026 13:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Güncelle: otomatik GitHub Actions güncellemesi (2026-10-16 15:36 UTC)
</commit_message>
<xml_diff>
--- a/maclar_ve_tahminler.xlsx
+++ b/maclar_ve_tahminler.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Maçlar ve Tahminler'!$A$2:$AI$154</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Öne Çıkanlar'!$A$1:$I$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Öne Çıkanlar'!$A$1:$I$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -8008,12 +8008,13 @@
       </c>
       <c r="AH53" s="40" t="inlineStr">
         <is>
-          <t>16°C, Az bulutlu, 7 km/sa</t>
+          <t>17°C, Az bulutlu, 7 km/sa</t>
         </is>
       </c>
       <c r="AI53" s="40" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Kesin) Lotka, Bittencourt, Butler, Cigerci, Erlein, Guwara, Hannemann, Kinsombi, Manu, Michelbrink, Rorig
+DEP: (Kesin) Reichert, Fernandez, Ghrieb, Janisch, Justvan, Kalogeropoulos, Markhiev, Otto, Porstner, Scobel, Zoma</t>
         </is>
       </c>
     </row>
@@ -8149,12 +8150,13 @@
       </c>
       <c r="AH54" s="46" t="inlineStr">
         <is>
-          <t>18°C, Bulutlu, 7 km/sa</t>
+          <t>18°C, Bulutlu, 9 km/sa</t>
         </is>
       </c>
       <c r="AI54" s="46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Kesin) Weiner, Balzi, Harres, Kapralik, Madsen, Meffert, Parduzi, Schonlau, Sekine, Therkelsen, Wiese
+DEP: (Kesin) Gersbeck, Adewumi, Brekalo, Eitschberger, Gechter, Gronning Andersen, Kolbe, Seguin, Sessa, Thorsteinsson, Zeefuik</t>
         </is>
       </c>
     </row>
@@ -8225,59 +8227,63 @@
         </is>
       </c>
       <c r="N55" s="43" t="n">
-        <v>62.9</v>
+        <v>65.5</v>
       </c>
       <c r="O55" s="43" t="n">
-        <v>18.4</v>
+        <v>17.7</v>
       </c>
       <c r="P55" s="43" t="n">
-        <v>18.7</v>
+        <v>16.8</v>
       </c>
       <c r="Q55" s="44" t="n">
         <v>2.77</v>
       </c>
       <c r="R55" s="44" t="n">
-        <v>1.19</v>
+        <v>1.01</v>
       </c>
       <c r="S55" s="43" t="n">
-        <v>64</v>
+        <v>62.5</v>
       </c>
       <c r="T55" s="43" t="n">
-        <v>36</v>
+        <v>37.5</v>
       </c>
       <c r="U55" s="43" t="n">
-        <v>60.5</v>
+        <v>57.7</v>
       </c>
       <c r="V55" s="43" t="n">
-        <v>39.5</v>
+        <v>42.3</v>
       </c>
       <c r="W55" s="43" t="n">
-        <v>89.90000000000001</v>
+        <v>88.5</v>
       </c>
       <c r="X55" s="43" t="n">
-        <v>81.3</v>
+        <v>83.2</v>
       </c>
       <c r="Y55" s="43" t="n">
-        <v>37.1</v>
+        <v>34.5</v>
       </c>
       <c r="Z55" s="43" t="n">
-        <v>81.59999999999999</v>
+        <v>82.3</v>
       </c>
       <c r="AA55" s="43" t="n">
-        <v>54</v>
+        <v>56.4</v>
       </c>
       <c r="AB55" s="43" t="n">
         <v>30.1</v>
       </c>
       <c r="AC55" s="43" t="n">
-        <v>15.9</v>
+        <v>13.5</v>
       </c>
       <c r="AD55" s="45" t="inlineStr">
         <is>
           <t>2-1 (%9)</t>
         </is>
       </c>
-      <c r="AE55" s="40" t="n"/>
+      <c r="AE55" s="40" t="inlineStr">
+        <is>
+          <t>Dep kilit oyuncu eksik (Bulut E.) -&gt; hücum -%15</t>
+        </is>
+      </c>
       <c r="AF55" s="40" t="inlineStr">
         <is>
           <t>Celik D.</t>
@@ -8290,12 +8296,13 @@
       </c>
       <c r="AH55" s="40" t="inlineStr">
         <is>
-          <t>12°C, Sağanak, 7 km/sa</t>
+          <t>12°C, Bulutlu, 8 km/sa</t>
         </is>
       </c>
       <c r="AI55" s="40" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Tahmini) Marcos Felipe, Sazdagi, Soyuncu, Smolcic, Borza, Ramadani, Alexandre Penetra, Under, Diomande, Kyziridis, Ramirez Diaz
+DEP: (Tahmini) Fofana, Pala, Mocsi, Sagnan, Ariss, Antalyali, Kutucu, Olawoyin, Laci, Mebude, Sowe</t>
         </is>
       </c>
     </row>
@@ -8436,7 +8443,8 @@
       </c>
       <c r="AI56" s="46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Tahmini) Escales, Delphis, Veillon, Do Marcolino, Kouadio, Kone, Dion, Venot, Larose, Rambaud, Billemaz
+DEP: (Tahmini) Basilio, Fernandez, Nahounou, Mendy, Tacafred, Gelin, Housni, Kandil, Bouabdelli, Raheriniaina, Ba</t>
         </is>
       </c>
     </row>
@@ -8507,59 +8515,63 @@
         </is>
       </c>
       <c r="N57" s="43" t="n">
-        <v>41.7</v>
+        <v>37.9</v>
       </c>
       <c r="O57" s="43" t="n">
-        <v>30.7</v>
+        <v>32.2</v>
       </c>
       <c r="P57" s="43" t="n">
-        <v>27.6</v>
+        <v>29.9</v>
       </c>
       <c r="Q57" s="44" t="n">
-        <v>1.15</v>
+        <v>0.98</v>
       </c>
       <c r="R57" s="44" t="n">
         <v>0.86</v>
       </c>
       <c r="S57" s="43" t="n">
-        <v>43.3</v>
+        <v>40.8</v>
       </c>
       <c r="T57" s="43" t="n">
-        <v>56.7</v>
+        <v>59.2</v>
       </c>
       <c r="U57" s="43" t="n">
-        <v>48.4</v>
+        <v>46.6</v>
       </c>
       <c r="V57" s="43" t="n">
-        <v>51.6</v>
+        <v>53.4</v>
       </c>
       <c r="W57" s="43" t="n">
-        <v>60.3</v>
+        <v>55.4</v>
       </c>
       <c r="X57" s="43" t="n">
-        <v>72.40000000000001</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="Y57" s="43" t="n">
-        <v>58.3</v>
+        <v>62.1</v>
       </c>
       <c r="Z57" s="43" t="n">
-        <v>69.3</v>
+        <v>67.8</v>
       </c>
       <c r="AA57" s="43" t="n">
-        <v>30.1</v>
+        <v>26.2</v>
       </c>
       <c r="AB57" s="43" t="n">
-        <v>49</v>
+        <v>51.5</v>
       </c>
       <c r="AC57" s="43" t="n">
-        <v>20.9</v>
+        <v>22.3</v>
       </c>
       <c r="AD57" s="45" t="inlineStr">
         <is>
-          <t>1-0 (%15)</t>
-        </is>
-      </c>
-      <c r="AE57" s="40" t="n"/>
+          <t>0-0 (%17)</t>
+        </is>
+      </c>
+      <c r="AE57" s="40" t="inlineStr">
+        <is>
+          <t>Ev kilit oyuncu eksik (Diaby Y.) -&gt; hücum -%15</t>
+        </is>
+      </c>
       <c r="AF57" s="40" t="inlineStr">
         <is>
           <t>Roffet B.</t>
@@ -8572,12 +8584,13 @@
       </c>
       <c r="AH57" s="40" t="inlineStr">
         <is>
-          <t>20°C, Açık, 3 km/sa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AI57" s="40" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Tahmini) Olliero, Zahui, Pelon, Vidal, Xantippe, Magnin, Akpa Akpro, Diba, Bernadou, Mouazan, Bonnet
+DEP: (Tahmini) Noukeu, Thiam, Kerriou, Pinot, Martin, Fatar, Bultel, Binet, Boyer, Hbouch, Soumah</t>
         </is>
       </c>
     </row>
@@ -8648,59 +8661,63 @@
         </is>
       </c>
       <c r="N58" s="43" t="n">
-        <v>40.2</v>
+        <v>39</v>
       </c>
       <c r="O58" s="43" t="n">
-        <v>27.4</v>
+        <v>29.3</v>
       </c>
       <c r="P58" s="43" t="n">
-        <v>32.4</v>
+        <v>31.7</v>
       </c>
       <c r="Q58" s="44" t="n">
-        <v>1.46</v>
+        <v>1.24</v>
       </c>
       <c r="R58" s="44" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="S58" s="43" t="n">
-        <v>52.5</v>
+        <v>47.7</v>
       </c>
       <c r="T58" s="43" t="n">
-        <v>47.5</v>
+        <v>52.3</v>
       </c>
       <c r="U58" s="43" t="n">
-        <v>56.4</v>
+        <v>52.4</v>
       </c>
       <c r="V58" s="43" t="n">
-        <v>43.6</v>
+        <v>47.6</v>
       </c>
       <c r="W58" s="43" t="n">
-        <v>76.7</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="X58" s="43" t="n">
-        <v>67.59999999999999</v>
+        <v>68.3</v>
       </c>
       <c r="Y58" s="43" t="n">
-        <v>59.8</v>
+        <v>61</v>
       </c>
       <c r="Z58" s="43" t="n">
-        <v>72.59999999999999</v>
+        <v>70.7</v>
       </c>
       <c r="AA58" s="43" t="n">
-        <v>31.7</v>
+        <v>29.5</v>
       </c>
       <c r="AB58" s="43" t="n">
-        <v>41.1</v>
+        <v>45.2</v>
       </c>
       <c r="AC58" s="43" t="n">
-        <v>27.2</v>
+        <v>25.4</v>
       </c>
       <c r="AD58" s="45" t="inlineStr">
         <is>
-          <t>1-1 (%13)</t>
-        </is>
-      </c>
-      <c r="AE58" s="46" t="n"/>
+          <t>1-1 (%14)</t>
+        </is>
+      </c>
+      <c r="AE58" s="46" t="inlineStr">
+        <is>
+          <t>Ev kilit oyuncu eksik (Gomis D.) -&gt; hücum -%15 | Dep kilit oyuncu eksik (Benet J.) -&gt; hücum -%15</t>
+        </is>
+      </c>
       <c r="AF58" s="46" t="inlineStr">
         <is>
           <t>Vincent T.</t>
@@ -8713,12 +8730,13 @@
       </c>
       <c r="AH58" s="46" t="inlineStr">
         <is>
-          <t>14°C, Açık, 14 km/sa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AI58" s="46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Tahmini) Ortola, Matumona, Koffi, Dianganga, Ollila, Averlant, Ducrocq, Louiserre, Ben Brahim, Ahile, Bokangu
+DEP: (Tahmini) Maubleu, Pouilly, Paquiez, Briancon, Bamba, Abdallah, Fall, Sebas, Rajot, Benali, Leye</t>
         </is>
       </c>
     </row>
@@ -8859,7 +8877,8 @@
       </c>
       <c r="AI59" s="40" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Tahmini) Hautbois, Mouton, Lo, Bianda, Gaudin, Sanna, Beaudouin, Mandouki, Houdayer, Kante, Clavreul
+DEP: (Tahmini) Guivarch, Coulibaly, Salmier, Kabeya, Kone, Grillot, Diop, Hunou, Astic, Bianchini, Okou</t>
         </is>
       </c>
     </row>
@@ -8930,59 +8949,63 @@
         </is>
       </c>
       <c r="N60" s="43" t="n">
-        <v>55.5</v>
+        <v>58.6</v>
       </c>
       <c r="O60" s="43" t="n">
-        <v>21.8</v>
+        <v>21.4</v>
       </c>
       <c r="P60" s="43" t="n">
-        <v>22.7</v>
+        <v>20</v>
       </c>
       <c r="Q60" s="44" t="n">
         <v>2.42</v>
       </c>
       <c r="R60" s="44" t="n">
-        <v>1.38</v>
+        <v>1.17</v>
       </c>
       <c r="S60" s="43" t="n">
-        <v>62.6</v>
+        <v>60.8</v>
       </c>
       <c r="T60" s="43" t="n">
-        <v>37.4</v>
+        <v>39.2</v>
       </c>
       <c r="U60" s="43" t="n">
-        <v>62.5</v>
+        <v>59.8</v>
       </c>
       <c r="V60" s="43" t="n">
-        <v>37.5</v>
+        <v>40.2</v>
       </c>
       <c r="W60" s="43" t="n">
-        <v>89.59999999999999</v>
+        <v>87.7</v>
       </c>
       <c r="X60" s="43" t="n">
-        <v>77.3</v>
+        <v>80</v>
       </c>
       <c r="Y60" s="43" t="n">
-        <v>44.5</v>
+        <v>41.4</v>
       </c>
       <c r="Z60" s="43" t="n">
-        <v>78.2</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="AA60" s="43" t="n">
-        <v>46.6</v>
+        <v>49.2</v>
       </c>
       <c r="AB60" s="43" t="n">
-        <v>32.6</v>
+        <v>33.1</v>
       </c>
       <c r="AC60" s="43" t="n">
-        <v>20.8</v>
+        <v>17.8</v>
       </c>
       <c r="AD60" s="45" t="inlineStr">
         <is>
           <t>2-1 (%9)</t>
         </is>
       </c>
-      <c r="AE60" s="46" t="n"/>
+      <c r="AE60" s="46" t="inlineStr">
+        <is>
+          <t>Dep kilit oyuncu eksik (Tavares J.) -&gt; hücum -%15</t>
+        </is>
+      </c>
       <c r="AF60" s="46" t="inlineStr">
         <is>
           <t>Rosier E.</t>
@@ -9000,7 +9023,8 @@
       </c>
       <c r="AI60" s="46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Tahmini) Hulsmann, Zohouri, Elie, Kotto, Guindo, Leoni, Kouranfal, El Kachati, Fofana, Daramy, Soumano
+DEP: (Tahmini) Delecroix, Hamada, Lacroix, Bernard, Faty, Marie, Chouchane, Lembezat, Ndezi, Dong, Lago</t>
         </is>
       </c>
     </row>
@@ -9071,59 +9095,63 @@
         </is>
       </c>
       <c r="N61" s="43" t="n">
-        <v>46.4</v>
+        <v>49</v>
       </c>
       <c r="O61" s="43" t="n">
-        <v>22.3</v>
+        <v>22.8</v>
       </c>
       <c r="P61" s="43" t="n">
-        <v>31.2</v>
+        <v>28.2</v>
       </c>
       <c r="Q61" s="44" t="n">
-        <v>2.34</v>
+        <v>2.25</v>
       </c>
       <c r="R61" s="44" t="n">
-        <v>1.88</v>
+        <v>1.59</v>
       </c>
       <c r="S61" s="43" t="n">
-        <v>66.3</v>
+        <v>63</v>
       </c>
       <c r="T61" s="43" t="n">
-        <v>33.7</v>
+        <v>37</v>
       </c>
       <c r="U61" s="43" t="n">
-        <v>67.09999999999999</v>
+        <v>64</v>
       </c>
       <c r="V61" s="43" t="n">
-        <v>32.9</v>
+        <v>36</v>
       </c>
       <c r="W61" s="43" t="n">
-        <v>92.40000000000001</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="X61" s="43" t="n">
-        <v>68.8</v>
+        <v>71.8</v>
       </c>
       <c r="Y61" s="43" t="n">
-        <v>53.6</v>
+        <v>51</v>
       </c>
       <c r="Z61" s="43" t="n">
-        <v>77.7</v>
+        <v>77.2</v>
       </c>
       <c r="AA61" s="43" t="n">
-        <v>37.8</v>
+        <v>40</v>
       </c>
       <c r="AB61" s="43" t="n">
-        <v>34.5</v>
+        <v>35.4</v>
       </c>
       <c r="AC61" s="43" t="n">
-        <v>27.7</v>
+        <v>24.5</v>
       </c>
       <c r="AD61" s="45" t="inlineStr">
         <is>
-          <t>2-1 (%8)</t>
-        </is>
-      </c>
-      <c r="AE61" s="40" t="n"/>
+          <t>2-1 (%9)</t>
+        </is>
+      </c>
+      <c r="AE61" s="40" t="inlineStr">
+        <is>
+          <t>Dep kilit oyuncu eksik (Dallinga T.) -&gt; hücum -%15</t>
+        </is>
+      </c>
       <c r="AF61" s="40" t="inlineStr">
         <is>
           <t>Brand B.</t>
@@ -9141,7 +9169,8 @@
       </c>
       <c r="AI61" s="40" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Tahmini) Atubolu, Baum, Koch, Brassier, Kosugi, Doan, Aseko-Nkili, Onyedika, Uzun, Ebnoutalib, Burkardt
+DEP: (Tahmini) Schwabe, Sebulonsen, Simpson-Pusey, Lochoshvili, Sosa, Krauss, Johannesson, Maina, Moore, El Mala, Bulter</t>
         </is>
       </c>
     </row>
@@ -9212,56 +9241,56 @@
         </is>
       </c>
       <c r="N62" s="43" t="n">
-        <v>53.2</v>
+        <v>53.3</v>
       </c>
       <c r="O62" s="43" t="n">
-        <v>24.4</v>
+        <v>22.9</v>
       </c>
       <c r="P62" s="43" t="n">
-        <v>22.4</v>
+        <v>23.8</v>
       </c>
       <c r="Q62" s="44" t="n">
-        <v>2.27</v>
+        <v>2.34</v>
       </c>
       <c r="R62" s="44" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="S62" s="43" t="n">
-        <v>60.6</v>
+        <v>62.1</v>
       </c>
       <c r="T62" s="43" t="n">
-        <v>39.4</v>
+        <v>37.9</v>
       </c>
       <c r="U62" s="43" t="n">
-        <v>61.7</v>
+        <v>62.7</v>
       </c>
       <c r="V62" s="43" t="n">
-        <v>38.3</v>
+        <v>37.3</v>
       </c>
       <c r="W62" s="43" t="n">
-        <v>88.8</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="X62" s="43" t="n">
-        <v>77.59999999999999</v>
+        <v>76.2</v>
       </c>
       <c r="Y62" s="43" t="n">
-        <v>46.8</v>
+        <v>46.7</v>
       </c>
       <c r="Z62" s="43" t="n">
-        <v>75.59999999999999</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="AA62" s="43" t="n">
-        <v>45.7</v>
+        <v>44.7</v>
       </c>
       <c r="AB62" s="43" t="n">
-        <v>33.6</v>
+        <v>33.7</v>
       </c>
       <c r="AC62" s="43" t="n">
-        <v>20.8</v>
+        <v>21.6</v>
       </c>
       <c r="AD62" s="45" t="inlineStr">
         <is>
-          <t>1-1 (%10)</t>
+          <t>2-1 (%9)</t>
         </is>
       </c>
       <c r="AE62" s="46" t="n"/>
@@ -11186,56 +11215,56 @@
         </is>
       </c>
       <c r="N76" s="43" t="n">
-        <v>30.6</v>
+        <v>32.5</v>
       </c>
       <c r="O76" s="43" t="n">
-        <v>28.2</v>
+        <v>26.7</v>
       </c>
       <c r="P76" s="43" t="n">
-        <v>41.2</v>
+        <v>40.8</v>
       </c>
       <c r="Q76" s="44" t="n">
-        <v>1.47</v>
+        <v>1.51</v>
       </c>
       <c r="R76" s="44" t="n">
-        <v>1.82</v>
+        <v>1.8</v>
       </c>
       <c r="S76" s="43" t="n">
-        <v>57.9</v>
+        <v>58.2</v>
       </c>
       <c r="T76" s="43" t="n">
-        <v>42.1</v>
+        <v>41.8</v>
       </c>
       <c r="U76" s="43" t="n">
-        <v>61.5</v>
+        <v>61.2</v>
       </c>
       <c r="V76" s="43" t="n">
-        <v>38.5</v>
+        <v>38.8</v>
       </c>
       <c r="W76" s="43" t="n">
-        <v>86</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="X76" s="43" t="n">
-        <v>58.8</v>
+        <v>59.2</v>
       </c>
       <c r="Y76" s="43" t="n">
-        <v>69.40000000000001</v>
+        <v>67.5</v>
       </c>
       <c r="Z76" s="43" t="n">
-        <v>71.8</v>
+        <v>73.3</v>
       </c>
       <c r="AA76" s="43" t="n">
-        <v>27.1</v>
+        <v>27.5</v>
       </c>
       <c r="AB76" s="43" t="n">
-        <v>36.5</v>
+        <v>37.4</v>
       </c>
       <c r="AC76" s="43" t="n">
-        <v>36.4</v>
+        <v>35.1</v>
       </c>
       <c r="AD76" s="45" t="inlineStr">
         <is>
-          <t>1-1 (%12)</t>
+          <t>1-1 (%11)</t>
         </is>
       </c>
       <c r="AE76" s="46" t="n"/>
@@ -11750,56 +11779,56 @@
         </is>
       </c>
       <c r="N80" s="43" t="n">
-        <v>33.1</v>
+        <v>33.5</v>
       </c>
       <c r="O80" s="43" t="n">
-        <v>24.2</v>
+        <v>24.3</v>
       </c>
       <c r="P80" s="43" t="n">
-        <v>42.7</v>
+        <v>42.2</v>
       </c>
       <c r="Q80" s="44" t="n">
         <v>1.62</v>
       </c>
       <c r="R80" s="44" t="n">
-        <v>2.01</v>
+        <v>1.97</v>
       </c>
       <c r="S80" s="43" t="n">
-        <v>61.2</v>
+        <v>60.8</v>
       </c>
       <c r="T80" s="43" t="n">
-        <v>38.8</v>
+        <v>39.2</v>
       </c>
       <c r="U80" s="43" t="n">
-        <v>63</v>
+        <v>62.8</v>
       </c>
       <c r="V80" s="43" t="n">
-        <v>37</v>
+        <v>37.2</v>
       </c>
       <c r="W80" s="43" t="n">
-        <v>87.7</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="X80" s="43" t="n">
-        <v>57.3</v>
+        <v>57.8</v>
       </c>
       <c r="Y80" s="43" t="n">
-        <v>66.90000000000001</v>
+        <v>66.5</v>
       </c>
       <c r="Z80" s="43" t="n">
-        <v>75.8</v>
+        <v>75.7</v>
       </c>
       <c r="AA80" s="43" t="n">
-        <v>26.5</v>
+        <v>27.1</v>
       </c>
       <c r="AB80" s="43" t="n">
-        <v>37.9</v>
+        <v>37.2</v>
       </c>
       <c r="AC80" s="43" t="n">
         <v>35.6</v>
       </c>
       <c r="AD80" s="45" t="inlineStr">
         <is>
-          <t>1-2 (%9)</t>
+          <t>1-1 (%9)</t>
         </is>
       </c>
       <c r="AE80" s="46" t="n"/>
@@ -11891,49 +11920,49 @@
         </is>
       </c>
       <c r="N81" s="43" t="n">
-        <v>41.6</v>
+        <v>42</v>
       </c>
       <c r="O81" s="43" t="n">
-        <v>23.4</v>
+        <v>23.5</v>
       </c>
       <c r="P81" s="43" t="n">
-        <v>35</v>
+        <v>34.6</v>
       </c>
       <c r="Q81" s="44" t="n">
-        <v>1.96</v>
+        <v>1.97</v>
       </c>
       <c r="R81" s="44" t="n">
-        <v>1.84</v>
+        <v>1.82</v>
       </c>
       <c r="S81" s="43" t="n">
-        <v>62.7</v>
+        <v>62.6</v>
       </c>
       <c r="T81" s="43" t="n">
-        <v>37.3</v>
+        <v>37.4</v>
       </c>
       <c r="U81" s="43" t="n">
-        <v>64.59999999999999</v>
+        <v>64.5</v>
       </c>
       <c r="V81" s="43" t="n">
-        <v>35.4</v>
+        <v>35.5</v>
       </c>
       <c r="W81" s="43" t="n">
         <v>89.2</v>
       </c>
       <c r="X81" s="43" t="n">
-        <v>65</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="Y81" s="43" t="n">
-        <v>58.4</v>
+        <v>58</v>
       </c>
       <c r="Z81" s="43" t="n">
-        <v>76.59999999999999</v>
+        <v>76.5</v>
       </c>
       <c r="AA81" s="43" t="n">
-        <v>32.9</v>
+        <v>33.6</v>
       </c>
       <c r="AB81" s="43" t="n">
-        <v>37</v>
+        <v>36.2</v>
       </c>
       <c r="AC81" s="43" t="n">
         <v>30.2</v>
@@ -12032,19 +12061,19 @@
         </is>
       </c>
       <c r="N82" s="43" t="n">
-        <v>63.4</v>
+        <v>64</v>
       </c>
       <c r="O82" s="43" t="n">
-        <v>18.6</v>
+        <v>18.4</v>
       </c>
       <c r="P82" s="43" t="n">
-        <v>18</v>
+        <v>17.6</v>
       </c>
       <c r="Q82" s="44" t="n">
-        <v>2.89</v>
+        <v>2.91</v>
       </c>
       <c r="R82" s="44" t="n">
-        <v>1.25</v>
+        <v>1.23</v>
       </c>
       <c r="S82" s="43" t="n">
         <v>65.59999999999999</v>
@@ -12053,31 +12082,31 @@
         <v>34.4</v>
       </c>
       <c r="U82" s="43" t="n">
-        <v>62</v>
+        <v>61.7</v>
       </c>
       <c r="V82" s="43" t="n">
-        <v>38</v>
+        <v>38.3</v>
       </c>
       <c r="W82" s="43" t="n">
         <v>91.8</v>
       </c>
       <c r="X82" s="43" t="n">
-        <v>82</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="Y82" s="43" t="n">
-        <v>36.6</v>
+        <v>36</v>
       </c>
       <c r="Z82" s="43" t="n">
-        <v>81.40000000000001</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="AA82" s="43" t="n">
-        <v>51.6</v>
+        <v>53</v>
       </c>
       <c r="AB82" s="43" t="n">
-        <v>32.4</v>
+        <v>31.4</v>
       </c>
       <c r="AC82" s="43" t="n">
-        <v>16</v>
+        <v>15.6</v>
       </c>
       <c r="AD82" s="45" t="inlineStr">
         <is>
@@ -12173,49 +12202,49 @@
         </is>
       </c>
       <c r="N83" s="43" t="n">
-        <v>44.2</v>
+        <v>44.6</v>
       </c>
       <c r="O83" s="43" t="n">
         <v>24.1</v>
       </c>
       <c r="P83" s="43" t="n">
-        <v>31.7</v>
+        <v>31.3</v>
       </c>
       <c r="Q83" s="44" t="n">
-        <v>1.95</v>
+        <v>1.96</v>
       </c>
       <c r="R83" s="44" t="n">
-        <v>1.59</v>
+        <v>1.57</v>
       </c>
       <c r="S83" s="43" t="n">
-        <v>60.4</v>
+        <v>60.3</v>
       </c>
       <c r="T83" s="43" t="n">
-        <v>39.6</v>
+        <v>39.7</v>
       </c>
       <c r="U83" s="43" t="n">
-        <v>62.5</v>
+        <v>62.3</v>
       </c>
       <c r="V83" s="43" t="n">
-        <v>37.5</v>
+        <v>37.7</v>
       </c>
       <c r="W83" s="43" t="n">
-        <v>86.90000000000001</v>
+        <v>86.7</v>
       </c>
       <c r="X83" s="43" t="n">
-        <v>68.3</v>
+        <v>68.7</v>
       </c>
       <c r="Y83" s="43" t="n">
-        <v>55.8</v>
+        <v>55.4</v>
       </c>
       <c r="Z83" s="43" t="n">
         <v>75.90000000000001</v>
       </c>
       <c r="AA83" s="43" t="n">
-        <v>35</v>
+        <v>35.8</v>
       </c>
       <c r="AB83" s="43" t="n">
-        <v>38.4</v>
+        <v>37.6</v>
       </c>
       <c r="AC83" s="43" t="n">
         <v>26.6</v>
@@ -12314,52 +12343,52 @@
         </is>
       </c>
       <c r="N84" s="43" t="n">
-        <v>58.9</v>
+        <v>57.3</v>
       </c>
       <c r="O84" s="43" t="n">
-        <v>19.1</v>
+        <v>19.7</v>
       </c>
       <c r="P84" s="43" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q84" s="44" t="n">
-        <v>3.18</v>
+        <v>3.07</v>
       </c>
       <c r="R84" s="44" t="n">
-        <v>1.76</v>
+        <v>1.77</v>
       </c>
       <c r="S84" s="43" t="n">
-        <v>71.7</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="T84" s="43" t="n">
-        <v>28.3</v>
+        <v>29.1</v>
       </c>
       <c r="U84" s="43" t="n">
-        <v>68.8</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="V84" s="43" t="n">
-        <v>31.2</v>
+        <v>31.4</v>
       </c>
       <c r="W84" s="43" t="n">
-        <v>95.7</v>
+        <v>95.3</v>
       </c>
       <c r="X84" s="43" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="Y84" s="43" t="n">
-        <v>41.1</v>
+        <v>42.7</v>
       </c>
       <c r="Z84" s="43" t="n">
-        <v>80.90000000000001</v>
+        <v>80.3</v>
       </c>
       <c r="AA84" s="43" t="n">
-        <v>49.6</v>
+        <v>48.9</v>
       </c>
       <c r="AB84" s="43" t="n">
-        <v>29.9</v>
+        <v>29.7</v>
       </c>
       <c r="AC84" s="43" t="n">
-        <v>20.6</v>
+        <v>21.4</v>
       </c>
       <c r="AD84" s="45" t="inlineStr">
         <is>
@@ -13160,52 +13189,52 @@
         </is>
       </c>
       <c r="N90" s="43" t="n">
-        <v>46.2</v>
+        <v>41.9</v>
       </c>
       <c r="O90" s="43" t="n">
-        <v>25.5</v>
+        <v>25.2</v>
       </c>
       <c r="P90" s="43" t="n">
-        <v>28.3</v>
+        <v>33</v>
       </c>
       <c r="Q90" s="44" t="n">
-        <v>2.18</v>
+        <v>1.98</v>
       </c>
       <c r="R90" s="44" t="n">
-        <v>1.61</v>
+        <v>1.72</v>
       </c>
       <c r="S90" s="43" t="n">
-        <v>62.7</v>
+        <v>61.8</v>
       </c>
       <c r="T90" s="43" t="n">
-        <v>37.3</v>
+        <v>38.2</v>
       </c>
       <c r="U90" s="43" t="n">
-        <v>64.8</v>
+        <v>64.2</v>
       </c>
       <c r="V90" s="43" t="n">
-        <v>35.2</v>
+        <v>35.8</v>
       </c>
       <c r="W90" s="43" t="n">
-        <v>90.8</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="X90" s="43" t="n">
-        <v>71.7</v>
+        <v>67</v>
       </c>
       <c r="Y90" s="43" t="n">
-        <v>53.8</v>
+        <v>58.1</v>
       </c>
       <c r="Z90" s="43" t="n">
-        <v>74.5</v>
+        <v>74.8</v>
       </c>
       <c r="AA90" s="43" t="n">
-        <v>40.6</v>
+        <v>35.8</v>
       </c>
       <c r="AB90" s="43" t="n">
-        <v>33.2</v>
+        <v>35</v>
       </c>
       <c r="AC90" s="43" t="n">
-        <v>26.2</v>
+        <v>29.3</v>
       </c>
       <c r="AD90" s="45" t="inlineStr">
         <is>
@@ -13865,52 +13894,52 @@
         </is>
       </c>
       <c r="N95" s="43" t="n">
-        <v>54.9</v>
+        <v>55.6</v>
       </c>
       <c r="O95" s="43" t="n">
-        <v>20.7</v>
+        <v>20.6</v>
       </c>
       <c r="P95" s="43" t="n">
-        <v>24.4</v>
+        <v>23.8</v>
       </c>
       <c r="Q95" s="44" t="n">
-        <v>2.7</v>
+        <v>2.71</v>
       </c>
       <c r="R95" s="44" t="n">
-        <v>1.65</v>
+        <v>1.61</v>
       </c>
       <c r="S95" s="43" t="n">
-        <v>67.3</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="T95" s="43" t="n">
-        <v>32.7</v>
+        <v>32.9</v>
       </c>
       <c r="U95" s="43" t="n">
-        <v>66.40000000000001</v>
+        <v>66</v>
       </c>
       <c r="V95" s="43" t="n">
-        <v>33.6</v>
+        <v>34</v>
       </c>
       <c r="W95" s="43" t="n">
-        <v>93.09999999999999</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="X95" s="43" t="n">
-        <v>75.59999999999999</v>
+        <v>76.2</v>
       </c>
       <c r="Y95" s="43" t="n">
-        <v>45.1</v>
+        <v>44.4</v>
       </c>
       <c r="Z95" s="43" t="n">
-        <v>79.3</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="AA95" s="43" t="n">
-        <v>44.8</v>
+        <v>46</v>
       </c>
       <c r="AB95" s="43" t="n">
-        <v>33</v>
+        <v>32.2</v>
       </c>
       <c r="AC95" s="43" t="n">
-        <v>22.2</v>
+        <v>21.8</v>
       </c>
       <c r="AD95" s="45" t="inlineStr">
         <is>
@@ -14570,56 +14599,56 @@
         </is>
       </c>
       <c r="N100" s="43" t="n">
-        <v>55.9</v>
+        <v>58.2</v>
       </c>
       <c r="O100" s="43" t="n">
-        <v>25.2</v>
+        <v>22.2</v>
       </c>
       <c r="P100" s="43" t="n">
-        <v>18.9</v>
+        <v>19.7</v>
       </c>
       <c r="Q100" s="44" t="n">
-        <v>2.07</v>
+        <v>2.37</v>
       </c>
       <c r="R100" s="44" t="n">
-        <v>0.96</v>
+        <v>1.12</v>
       </c>
       <c r="S100" s="43" t="n">
-        <v>55.3</v>
+        <v>59.8</v>
       </c>
       <c r="T100" s="43" t="n">
-        <v>44.7</v>
+        <v>40.2</v>
       </c>
       <c r="U100" s="43" t="n">
-        <v>56.1</v>
+        <v>59.1</v>
       </c>
       <c r="V100" s="43" t="n">
-        <v>43.9</v>
+        <v>40.9</v>
       </c>
       <c r="W100" s="43" t="n">
-        <v>82.3</v>
+        <v>87</v>
       </c>
       <c r="X100" s="43" t="n">
-        <v>81.09999999999999</v>
+        <v>80.3</v>
       </c>
       <c r="Y100" s="43" t="n">
-        <v>44.1</v>
+        <v>41.8</v>
       </c>
       <c r="Z100" s="43" t="n">
-        <v>74.8</v>
+        <v>77.8</v>
       </c>
       <c r="AA100" s="43" t="n">
-        <v>46.9</v>
+        <v>48.5</v>
       </c>
       <c r="AB100" s="43" t="n">
-        <v>36.6</v>
+        <v>34.2</v>
       </c>
       <c r="AC100" s="43" t="n">
-        <v>16.6</v>
+        <v>17.2</v>
       </c>
       <c r="AD100" s="45" t="inlineStr">
         <is>
-          <t>1-1 (%12)</t>
+          <t>2-1 (%10)</t>
         </is>
       </c>
       <c r="AE100" s="46" t="n"/>
@@ -17531,19 +17560,19 @@
         </is>
       </c>
       <c r="N121" s="43" t="n">
-        <v>56.5</v>
+        <v>54.5</v>
       </c>
       <c r="O121" s="43" t="n">
-        <v>23.2</v>
+        <v>22.8</v>
       </c>
       <c r="P121" s="43" t="n">
-        <v>20.3</v>
+        <v>22.7</v>
       </c>
       <c r="Q121" s="44" t="n">
-        <v>2.53</v>
+        <v>2.44</v>
       </c>
       <c r="R121" s="44" t="n">
-        <v>1.25</v>
+        <v>1.34</v>
       </c>
       <c r="S121" s="43" t="n">
         <v>62.5</v>
@@ -17552,31 +17581,31 @@
         <v>37.5</v>
       </c>
       <c r="U121" s="43" t="n">
-        <v>61.8</v>
+        <v>62.3</v>
       </c>
       <c r="V121" s="43" t="n">
-        <v>38.2</v>
+        <v>37.7</v>
       </c>
       <c r="W121" s="43" t="n">
-        <v>90.5</v>
+        <v>89.8</v>
       </c>
       <c r="X121" s="43" t="n">
-        <v>79.7</v>
+        <v>77.3</v>
       </c>
       <c r="Y121" s="43" t="n">
-        <v>43.5</v>
+        <v>45.5</v>
       </c>
       <c r="Z121" s="43" t="n">
-        <v>76.8</v>
+        <v>77.2</v>
       </c>
       <c r="AA121" s="43" t="n">
-        <v>50.2</v>
+        <v>47</v>
       </c>
       <c r="AB121" s="43" t="n">
-        <v>31.6</v>
+        <v>33</v>
       </c>
       <c r="AC121" s="43" t="n">
-        <v>18.2</v>
+        <v>20</v>
       </c>
       <c r="AD121" s="45" t="inlineStr">
         <is>
@@ -18941,56 +18970,56 @@
         </is>
       </c>
       <c r="N131" s="43" t="n">
-        <v>58.8</v>
+        <v>60.9</v>
       </c>
       <c r="O131" s="43" t="n">
-        <v>23.6</v>
+        <v>20.9</v>
       </c>
       <c r="P131" s="43" t="n">
-        <v>17.5</v>
+        <v>18.2</v>
       </c>
       <c r="Q131" s="44" t="n">
-        <v>2.29</v>
+        <v>2.61</v>
       </c>
       <c r="R131" s="44" t="n">
-        <v>0.95</v>
+        <v>1.11</v>
       </c>
       <c r="S131" s="43" t="n">
-        <v>57.4</v>
+        <v>62</v>
       </c>
       <c r="T131" s="43" t="n">
-        <v>42.6</v>
+        <v>38</v>
       </c>
       <c r="U131" s="43" t="n">
-        <v>56.6</v>
+        <v>59.6</v>
       </c>
       <c r="V131" s="43" t="n">
-        <v>43.4</v>
+        <v>40.4</v>
       </c>
       <c r="W131" s="43" t="n">
-        <v>85</v>
+        <v>89.2</v>
       </c>
       <c r="X131" s="43" t="n">
-        <v>82.5</v>
+        <v>81.8</v>
       </c>
       <c r="Y131" s="43" t="n">
-        <v>41.2</v>
+        <v>39.1</v>
       </c>
       <c r="Z131" s="43" t="n">
-        <v>76.40000000000001</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="AA131" s="43" t="n">
-        <v>50.5</v>
+        <v>52.1</v>
       </c>
       <c r="AB131" s="43" t="n">
-        <v>34.3</v>
+        <v>32.1</v>
       </c>
       <c r="AC131" s="43" t="n">
-        <v>15.2</v>
+        <v>15.8</v>
       </c>
       <c r="AD131" s="45" t="inlineStr">
         <is>
-          <t>2-0 (%10)</t>
+          <t>2-1 (%9)</t>
         </is>
       </c>
       <c r="AE131" s="40" t="n"/>
@@ -19646,52 +19675,52 @@
         </is>
       </c>
       <c r="N136" s="43" t="n">
-        <v>54</v>
+        <v>53.9</v>
       </c>
       <c r="O136" s="43" t="n">
-        <v>20.5</v>
+        <v>20.8</v>
       </c>
       <c r="P136" s="43" t="n">
-        <v>25.5</v>
+        <v>25.2</v>
       </c>
       <c r="Q136" s="44" t="n">
-        <v>2.81</v>
+        <v>2.72</v>
       </c>
       <c r="R136" s="44" t="n">
-        <v>1.82</v>
+        <v>1.72</v>
       </c>
       <c r="S136" s="43" t="n">
-        <v>69.40000000000001</v>
+        <v>68</v>
       </c>
       <c r="T136" s="43" t="n">
-        <v>30.6</v>
+        <v>32</v>
       </c>
       <c r="U136" s="43" t="n">
-        <v>68.40000000000001</v>
+        <v>67.2</v>
       </c>
       <c r="V136" s="43" t="n">
-        <v>31.6</v>
+        <v>32.8</v>
       </c>
       <c r="W136" s="43" t="n">
-        <v>94.5</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="X136" s="43" t="n">
-        <v>74.5</v>
+        <v>74.8</v>
       </c>
       <c r="Y136" s="43" t="n">
-        <v>46</v>
+        <v>46.1</v>
       </c>
       <c r="Z136" s="43" t="n">
-        <v>79.5</v>
+        <v>79.2</v>
       </c>
       <c r="AA136" s="43" t="n">
-        <v>44.5</v>
+        <v>45.1</v>
       </c>
       <c r="AB136" s="43" t="n">
         <v>31.9</v>
       </c>
       <c r="AC136" s="43" t="n">
-        <v>23.6</v>
+        <v>23.1</v>
       </c>
       <c r="AD136" s="45" t="inlineStr">
         <is>
@@ -20495,53 +20524,53 @@
         <v>49</v>
       </c>
       <c r="O142" s="43" t="n">
-        <v>21.2</v>
+        <v>21.6</v>
       </c>
       <c r="P142" s="43" t="n">
-        <v>29.8</v>
+        <v>29.4</v>
       </c>
       <c r="Q142" s="44" t="n">
-        <v>2.78</v>
+        <v>2.67</v>
       </c>
       <c r="R142" s="44" t="n">
-        <v>2.11</v>
+        <v>1.98</v>
       </c>
       <c r="S142" s="43" t="n">
-        <v>71.3</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="T142" s="43" t="n">
-        <v>28.7</v>
+        <v>30.4</v>
       </c>
       <c r="U142" s="43" t="n">
-        <v>70.8</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="V142" s="43" t="n">
-        <v>29.2</v>
+        <v>30.6</v>
       </c>
       <c r="W142" s="43" t="n">
-        <v>95.5</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="X142" s="43" t="n">
-        <v>70.2</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="Y142" s="43" t="n">
         <v>51</v>
       </c>
       <c r="Z142" s="43" t="n">
-        <v>78.8</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="AA142" s="43" t="n">
-        <v>41.3</v>
+        <v>41.7</v>
       </c>
       <c r="AB142" s="43" t="n">
-        <v>31.4</v>
+        <v>31.5</v>
       </c>
       <c r="AC142" s="43" t="n">
-        <v>27.4</v>
+        <v>26.8</v>
       </c>
       <c r="AD142" s="45" t="inlineStr">
         <is>
-          <t>2-2 (%6)</t>
+          <t>2-1 (%7)</t>
         </is>
       </c>
       <c r="AE142" s="46" t="n"/>
@@ -20633,52 +20662,52 @@
         </is>
       </c>
       <c r="N143" s="43" t="n">
-        <v>64.40000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="O143" s="43" t="n">
-        <v>20.8</v>
+        <v>18.3</v>
       </c>
       <c r="P143" s="43" t="n">
-        <v>14.9</v>
+        <v>13.9</v>
       </c>
       <c r="Q143" s="44" t="n">
-        <v>2.6</v>
+        <v>2.77</v>
       </c>
       <c r="R143" s="44" t="n">
-        <v>0.91</v>
+        <v>0.85</v>
       </c>
       <c r="S143" s="43" t="n">
-        <v>60</v>
+        <v>61.1</v>
       </c>
       <c r="T143" s="43" t="n">
-        <v>40</v>
+        <v>38.9</v>
       </c>
       <c r="U143" s="43" t="n">
-        <v>56.5</v>
+        <v>55.4</v>
       </c>
       <c r="V143" s="43" t="n">
-        <v>43.5</v>
+        <v>44.6</v>
       </c>
       <c r="W143" s="43" t="n">
-        <v>87.90000000000001</v>
+        <v>88.2</v>
       </c>
       <c r="X143" s="43" t="n">
-        <v>85.09999999999999</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="Y143" s="43" t="n">
-        <v>35.6</v>
+        <v>32.2</v>
       </c>
       <c r="Z143" s="43" t="n">
-        <v>79.2</v>
+        <v>81.7</v>
       </c>
       <c r="AA143" s="43" t="n">
-        <v>55.9</v>
+        <v>57.8</v>
       </c>
       <c r="AB143" s="43" t="n">
-        <v>31.3</v>
+        <v>30.8</v>
       </c>
       <c r="AC143" s="43" t="n">
-        <v>12.9</v>
+        <v>11.3</v>
       </c>
       <c r="AD143" s="45" t="inlineStr">
         <is>
@@ -21338,25 +21367,25 @@
         </is>
       </c>
       <c r="N148" s="43" t="n">
-        <v>46.9</v>
+        <v>48.7</v>
       </c>
       <c r="O148" s="43" t="n">
-        <v>26.8</v>
+        <v>24.9</v>
       </c>
       <c r="P148" s="43" t="n">
-        <v>26.3</v>
+        <v>26.4</v>
       </c>
       <c r="Q148" s="44" t="n">
-        <v>2</v>
+        <v>2.07</v>
       </c>
       <c r="R148" s="44" t="n">
-        <v>1.35</v>
+        <v>1.37</v>
       </c>
       <c r="S148" s="43" t="n">
-        <v>58.6</v>
+        <v>59.4</v>
       </c>
       <c r="T148" s="43" t="n">
-        <v>41.4</v>
+        <v>40.6</v>
       </c>
       <c r="U148" s="43" t="n">
         <v>61.2</v>
@@ -21365,29 +21394,29 @@
         <v>38.8</v>
       </c>
       <c r="W148" s="43" t="n">
-        <v>86.59999999999999</v>
+        <v>86.5</v>
       </c>
       <c r="X148" s="43" t="n">
-        <v>73.7</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="Y148" s="43" t="n">
-        <v>53.1</v>
+        <v>51.3</v>
       </c>
       <c r="Z148" s="43" t="n">
-        <v>73.2</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="AA148" s="43" t="n">
-        <v>40.8</v>
+        <v>41</v>
       </c>
       <c r="AB148" s="43" t="n">
-        <v>35.6</v>
+        <v>36</v>
       </c>
       <c r="AC148" s="43" t="n">
-        <v>23.6</v>
+        <v>23</v>
       </c>
       <c r="AD148" s="45" t="inlineStr">
         <is>
-          <t>1-1 (%11)</t>
+          <t>1-1 (%10)</t>
         </is>
       </c>
       <c r="AE148" s="46" t="n"/>
@@ -22284,7 +22313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -22413,27 +22442,27 @@
       </c>
       <c r="B4" s="45" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="C4" s="45" t="inlineStr">
         <is>
-          <t>Almanya</t>
+          <t>Fransa</t>
         </is>
       </c>
       <c r="D4" s="45" t="inlineStr">
         <is>
-          <t>Bundesliga</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="E4" s="51" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt</t>
+          <t>Le Mans FC</t>
         </is>
       </c>
       <c r="F4" s="51" t="inlineStr">
         <is>
-          <t>1. FC Köln</t>
+          <t>Toulouse FC</t>
         </is>
       </c>
       <c r="G4" s="45" t="inlineStr">
@@ -22447,52 +22476,52 @@
         </is>
       </c>
       <c r="I4" s="52" t="n">
-        <v>92.40000000000001</v>
+        <v>92.09999999999999</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="45" t="inlineStr">
+      <c r="A5" s="53" t="inlineStr">
         <is>
           <t>16.10.2026</t>
         </is>
       </c>
-      <c r="B5" s="45" t="inlineStr">
+      <c r="B5" s="53" t="inlineStr">
         <is>
           <t>21:45</t>
         </is>
       </c>
-      <c r="C5" s="45" t="inlineStr">
-        <is>
-          <t>Fransa</t>
-        </is>
-      </c>
-      <c r="D5" s="45" t="inlineStr">
-        <is>
-          <t>Ligue 1</t>
-        </is>
-      </c>
-      <c r="E5" s="51" t="inlineStr">
-        <is>
-          <t>Le Mans FC</t>
-        </is>
-      </c>
-      <c r="F5" s="51" t="inlineStr">
-        <is>
-          <t>Toulouse FC</t>
-        </is>
-      </c>
-      <c r="G5" s="45" t="inlineStr">
-        <is>
-          <t>1.5 Üst</t>
-        </is>
-      </c>
-      <c r="H5" s="45" t="inlineStr">
-        <is>
-          <t>Üst</t>
-        </is>
-      </c>
-      <c r="I5" s="52" t="n">
-        <v>92.09999999999999</v>
+      <c r="C5" s="53" t="inlineStr">
+        <is>
+          <t>Avrupa</t>
+        </is>
+      </c>
+      <c r="D5" s="53" t="inlineStr">
+        <is>
+          <t>UEFA Avrupa Konferans Ligi</t>
+        </is>
+      </c>
+      <c r="E5" s="54" t="inlineStr">
+        <is>
+          <t>Larne</t>
+        </is>
+      </c>
+      <c r="F5" s="54" t="inlineStr">
+        <is>
+          <t>Coleraine</t>
+        </is>
+      </c>
+      <c r="G5" s="53" t="inlineStr">
+        <is>
+          <t>Çifte Şans</t>
+        </is>
+      </c>
+      <c r="H5" s="53" t="inlineStr">
+        <is>
+          <t>1X</t>
+        </is>
+      </c>
+      <c r="I5" s="55" t="n">
+        <v>86.5</v>
       </c>
     </row>
     <row r="6">
@@ -22503,27 +22532,27 @@
       </c>
       <c r="B6" s="53" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C6" s="53" t="inlineStr">
         <is>
-          <t>Avrupa</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="D6" s="53" t="inlineStr">
         <is>
-          <t>UEFA Avrupa Konferans Ligi</t>
+          <t>Süper Lig</t>
         </is>
       </c>
       <c r="E6" s="54" t="inlineStr">
         <is>
-          <t>Larne</t>
+          <t>Corum</t>
         </is>
       </c>
       <c r="F6" s="54" t="inlineStr">
         <is>
-          <t>Coleraine</t>
+          <t>Rizespor</t>
         </is>
       </c>
       <c r="G6" s="53" t="inlineStr">
@@ -22537,7 +22566,7 @@
         </is>
       </c>
       <c r="I6" s="55" t="n">
-        <v>86.5</v>
+        <v>83.2</v>
       </c>
     </row>
     <row r="7">
@@ -22548,27 +22577,27 @@
       </c>
       <c r="B7" s="53" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C7" s="53" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Fransa</t>
         </is>
       </c>
       <c r="D7" s="53" t="inlineStr">
         <is>
-          <t>Süper Lig</t>
+          <t>Ligue 2 (Fransa)</t>
         </is>
       </c>
       <c r="E7" s="54" t="inlineStr">
         <is>
-          <t>Corum</t>
+          <t>Reims</t>
         </is>
       </c>
       <c r="F7" s="54" t="inlineStr">
         <is>
-          <t>Rizespor</t>
+          <t>Dijon</t>
         </is>
       </c>
       <c r="G7" s="53" t="inlineStr">
@@ -22578,11 +22607,11 @@
       </c>
       <c r="H7" s="53" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>1X</t>
         </is>
       </c>
       <c r="I7" s="55" t="n">
-        <v>81.59999999999999</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8">
@@ -22642,7 +22671,7 @@
         </is>
       </c>
       <c r="I9" s="52" t="n">
-        <v>95.7</v>
+        <v>95.3</v>
       </c>
     </row>
     <row r="10">
@@ -22838,22 +22867,22 @@
       </c>
       <c r="C14" s="45" t="inlineStr">
         <is>
-          <t>Almanya</t>
+          <t>İngiltere</t>
         </is>
       </c>
       <c r="D14" s="45" t="inlineStr">
         <is>
-          <t>Bundesliga</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="E14" s="51" t="inlineStr">
         <is>
-          <t>FC Bayern München</t>
+          <t>Newcastle United FC</t>
         </is>
       </c>
       <c r="F14" s="51" t="inlineStr">
         <is>
-          <t>RB Leipzig</t>
+          <t>Aston Villa FC</t>
         </is>
       </c>
       <c r="G14" s="45" t="inlineStr">
@@ -22867,7 +22896,7 @@
         </is>
       </c>
       <c r="I14" s="52" t="n">
-        <v>93.09999999999999</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15">
@@ -22883,22 +22912,22 @@
       </c>
       <c r="C15" s="45" t="inlineStr">
         <is>
-          <t>İngiltere</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D15" s="45" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>Bundesliga</t>
         </is>
       </c>
       <c r="E15" s="51" t="inlineStr">
         <is>
-          <t>Newcastle United FC</t>
+          <t>FC Bayern München</t>
         </is>
       </c>
       <c r="F15" s="51" t="inlineStr">
         <is>
-          <t>Aston Villa FC</t>
+          <t>RB Leipzig</t>
         </is>
       </c>
       <c r="G15" s="45" t="inlineStr">
@@ -22912,7 +22941,7 @@
         </is>
       </c>
       <c r="I15" s="52" t="n">
-        <v>93</v>
+        <v>92.90000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -22968,27 +22997,27 @@
       </c>
       <c r="B17" s="45" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C17" s="45" t="inlineStr">
         <is>
-          <t>İtalya</t>
+          <t>İngiltere</t>
         </is>
       </c>
       <c r="D17" s="45" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="E17" s="51" t="inlineStr">
         <is>
-          <t>Bologna FC 1909</t>
+          <t>Manchester City FC</t>
         </is>
       </c>
       <c r="F17" s="51" t="inlineStr">
         <is>
-          <t>FC Internazionale Milano</t>
+          <t>Ipswich Town FC</t>
         </is>
       </c>
       <c r="G17" s="45" t="inlineStr">
@@ -23002,7 +23031,7 @@
         </is>
       </c>
       <c r="I17" s="52" t="n">
-        <v>90.8</v>
+        <v>90.5</v>
       </c>
     </row>
     <row r="18">
@@ -23013,27 +23042,27 @@
       </c>
       <c r="B18" s="45" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C18" s="45" t="inlineStr">
         <is>
-          <t>İngiltere</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D18" s="45" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>2. Bundesliga</t>
         </is>
       </c>
       <c r="E18" s="51" t="inlineStr">
         <is>
-          <t>Manchester City FC</t>
+          <t>Greuther Furth</t>
         </is>
       </c>
       <c r="F18" s="51" t="inlineStr">
         <is>
-          <t>Ipswich Town FC</t>
+          <t>Braunschweig</t>
         </is>
       </c>
       <c r="G18" s="45" t="inlineStr">
@@ -23047,52 +23076,52 @@
         </is>
       </c>
       <c r="I18" s="52" t="n">
-        <v>90.5</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="45" t="inlineStr">
+      <c r="A19" s="53" t="inlineStr">
         <is>
           <t>17.10.2026</t>
         </is>
       </c>
-      <c r="B19" s="45" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="C19" s="45" t="inlineStr">
-        <is>
-          <t>Almanya</t>
-        </is>
-      </c>
-      <c r="D19" s="45" t="inlineStr">
-        <is>
-          <t>2. Bundesliga</t>
-        </is>
-      </c>
-      <c r="E19" s="51" t="inlineStr">
-        <is>
-          <t>Greuther Furth</t>
-        </is>
-      </c>
-      <c r="F19" s="51" t="inlineStr">
-        <is>
-          <t>Braunschweig</t>
-        </is>
-      </c>
-      <c r="G19" s="45" t="inlineStr">
-        <is>
-          <t>1.5 Üst</t>
-        </is>
-      </c>
-      <c r="H19" s="45" t="inlineStr">
-        <is>
-          <t>Üst</t>
-        </is>
-      </c>
-      <c r="I19" s="52" t="n">
-        <v>90</v>
+      <c r="B19" s="53" t="inlineStr">
+        <is>
+          <t>03:30</t>
+        </is>
+      </c>
+      <c r="C19" s="53" t="inlineStr">
+        <is>
+          <t>Arjantin</t>
+        </is>
+      </c>
+      <c r="D19" s="53" t="inlineStr">
+        <is>
+          <t>Liga Profesional (Arjantin)</t>
+        </is>
+      </c>
+      <c r="E19" s="54" t="inlineStr">
+        <is>
+          <t>Boca Juniors</t>
+        </is>
+      </c>
+      <c r="F19" s="54" t="inlineStr">
+        <is>
+          <t>Talleres Cordoba</t>
+        </is>
+      </c>
+      <c r="G19" s="53" t="inlineStr">
+        <is>
+          <t>Çifte Şans</t>
+        </is>
+      </c>
+      <c r="H19" s="53" t="inlineStr">
+        <is>
+          <t>1X</t>
+        </is>
+      </c>
+      <c r="I19" s="55" t="n">
+        <v>86.5</v>
       </c>
     </row>
     <row r="20">
@@ -23103,27 +23132,27 @@
       </c>
       <c r="B20" s="53" t="inlineStr">
         <is>
-          <t>03:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C20" s="53" t="inlineStr">
         <is>
-          <t>Arjantin</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D20" s="53" t="inlineStr">
         <is>
-          <t>Liga Profesional (Arjantin)</t>
+          <t>MLS</t>
         </is>
       </c>
       <c r="E20" s="54" t="inlineStr">
         <is>
-          <t>Boca Juniors</t>
+          <t>Philadelphia Union</t>
         </is>
       </c>
       <c r="F20" s="54" t="inlineStr">
         <is>
-          <t>Talleres Cordoba</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="G20" s="53" t="inlineStr">
@@ -23137,7 +23166,7 @@
         </is>
       </c>
       <c r="I20" s="55" t="n">
-        <v>86.5</v>
+        <v>84.7</v>
       </c>
     </row>
     <row r="21">
@@ -23148,27 +23177,27 @@
       </c>
       <c r="B21" s="53" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C21" s="53" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="D21" s="53" t="inlineStr">
         <is>
-          <t>MLS</t>
+          <t>Süper Lig</t>
         </is>
       </c>
       <c r="E21" s="54" t="inlineStr">
         <is>
-          <t>Philadelphia Union</t>
+          <t>Amedspor</t>
         </is>
       </c>
       <c r="F21" s="54" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Konyaspor</t>
         </is>
       </c>
       <c r="G21" s="53" t="inlineStr">
@@ -23182,7 +23211,7 @@
         </is>
       </c>
       <c r="I21" s="55" t="n">
-        <v>84.7</v>
+        <v>84.59999999999999</v>
       </c>
     </row>
     <row r="22">
@@ -23193,7 +23222,7 @@
       </c>
       <c r="B22" s="53" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C22" s="53" t="inlineStr">
@@ -23208,12 +23237,12 @@
       </c>
       <c r="E22" s="54" t="inlineStr">
         <is>
-          <t>Amedspor</t>
+          <t>Erzurumspor</t>
         </is>
       </c>
       <c r="F22" s="54" t="inlineStr">
         <is>
-          <t>Konyaspor</t>
+          <t>Eyupspor</t>
         </is>
       </c>
       <c r="G22" s="53" t="inlineStr">
@@ -23227,7 +23256,7 @@
         </is>
       </c>
       <c r="I22" s="55" t="n">
-        <v>84.59999999999999</v>
+        <v>82.40000000000001</v>
       </c>
     </row>
     <row r="23">
@@ -23238,27 +23267,27 @@
       </c>
       <c r="B23" s="53" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C23" s="53" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D23" s="53" t="inlineStr">
         <is>
-          <t>Süper Lig</t>
+          <t>Bundesliga</t>
         </is>
       </c>
       <c r="E23" s="54" t="inlineStr">
         <is>
-          <t>Erzurumspor</t>
+          <t>SV Werder Bremen</t>
         </is>
       </c>
       <c r="F23" s="54" t="inlineStr">
         <is>
-          <t>Eyupspor</t>
+          <t>SC Paderborn 07</t>
         </is>
       </c>
       <c r="G23" s="53" t="inlineStr">
@@ -23283,7 +23312,7 @@
       </c>
       <c r="B24" s="53" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C24" s="53" t="inlineStr">
@@ -23293,17 +23322,17 @@
       </c>
       <c r="D24" s="53" t="inlineStr">
         <is>
-          <t>Bundesliga</t>
+          <t>2. Bundesliga</t>
         </is>
       </c>
       <c r="E24" s="54" t="inlineStr">
         <is>
-          <t>SV Werder Bremen</t>
+          <t>Wolfsburg</t>
         </is>
       </c>
       <c r="F24" s="54" t="inlineStr">
         <is>
-          <t>SC Paderborn 07</t>
+          <t>Heidenheim</t>
         </is>
       </c>
       <c r="G24" s="53" t="inlineStr">
@@ -23313,11 +23342,11 @@
       </c>
       <c r="H24" s="53" t="inlineStr">
         <is>
-          <t>1X</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I24" s="55" t="n">
-        <v>82</v>
+        <v>81.7</v>
       </c>
     </row>
     <row r="25">
@@ -23328,27 +23357,27 @@
       </c>
       <c r="B25" s="53" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C25" s="53" t="inlineStr">
         <is>
-          <t>Almanya</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="D25" s="53" t="inlineStr">
         <is>
-          <t>2. Bundesliga</t>
+          <t>Süper Lig</t>
         </is>
       </c>
       <c r="E25" s="54" t="inlineStr">
         <is>
-          <t>Wolfsburg</t>
+          <t>Fenerbahce</t>
         </is>
       </c>
       <c r="F25" s="54" t="inlineStr">
         <is>
-          <t>Heidenheim</t>
+          <t>Alanyaspor</t>
         </is>
       </c>
       <c r="G25" s="53" t="inlineStr">
@@ -23358,11 +23387,11 @@
       </c>
       <c r="H25" s="53" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>1X</t>
         </is>
       </c>
       <c r="I25" s="55" t="n">
-        <v>81.7</v>
+        <v>81.5</v>
       </c>
     </row>
     <row r="26">
@@ -23373,27 +23402,27 @@
       </c>
       <c r="B26" s="53" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C26" s="53" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>İngiltere</t>
         </is>
       </c>
       <c r="D26" s="53" t="inlineStr">
         <is>
-          <t>Süper Lig</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="E26" s="54" t="inlineStr">
         <is>
-          <t>Fenerbahce</t>
+          <t>Brentford FC</t>
         </is>
       </c>
       <c r="F26" s="54" t="inlineStr">
         <is>
-          <t>Alanyaspor</t>
+          <t>Liverpool FC</t>
         </is>
       </c>
       <c r="G26" s="53" t="inlineStr">
@@ -23407,7 +23436,7 @@
         </is>
       </c>
       <c r="I26" s="55" t="n">
-        <v>81.5</v>
+        <v>81.2</v>
       </c>
     </row>
     <row r="27">
@@ -23418,27 +23447,27 @@
       </c>
       <c r="B27" s="53" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C27" s="53" t="inlineStr">
         <is>
-          <t>İngiltere</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D27" s="53" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>Bundesliga</t>
         </is>
       </c>
       <c r="E27" s="54" t="inlineStr">
         <is>
-          <t>Brentford FC</t>
+          <t>FC Schalke 04</t>
         </is>
       </c>
       <c r="F27" s="54" t="inlineStr">
         <is>
-          <t>Liverpool FC</t>
+          <t>1. FSV Mainz 05</t>
         </is>
       </c>
       <c r="G27" s="53" t="inlineStr">
@@ -23448,11 +23477,11 @@
       </c>
       <c r="H27" s="53" t="inlineStr">
         <is>
-          <t>1X</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I27" s="55" t="n">
-        <v>81.2</v>
+        <v>80.3</v>
       </c>
     </row>
     <row r="28">
@@ -23497,68 +23526,68 @@
         </is>
       </c>
       <c r="I28" s="55" t="n">
-        <v>81.09999999999999</v>
+        <v>80.3</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="53" t="inlineStr">
-        <is>
-          <t>17.10.2026</t>
-        </is>
-      </c>
-      <c r="B29" s="53" t="inlineStr">
-        <is>
-          <t>16:30</t>
-        </is>
-      </c>
-      <c r="C29" s="53" t="inlineStr">
-        <is>
-          <t>Almanya</t>
-        </is>
-      </c>
-      <c r="D29" s="53" t="inlineStr">
-        <is>
-          <t>Bundesliga</t>
-        </is>
-      </c>
-      <c r="E29" s="54" t="inlineStr">
-        <is>
-          <t>FC Schalke 04</t>
-        </is>
-      </c>
-      <c r="F29" s="54" t="inlineStr">
-        <is>
-          <t>1. FSV Mainz 05</t>
-        </is>
-      </c>
-      <c r="G29" s="53" t="inlineStr">
-        <is>
-          <t>Çifte Şans</t>
-        </is>
-      </c>
-      <c r="H29" s="53" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="I29" s="55" t="n">
-        <v>80.90000000000001</v>
-      </c>
+      <c r="A29" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  18.10.2026</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="n"/>
+      <c r="C29" s="6" t="n"/>
+      <c r="D29" s="6" t="n"/>
+      <c r="E29" s="6" t="n"/>
+      <c r="F29" s="6" t="n"/>
+      <c r="G29" s="6" t="n"/>
+      <c r="H29" s="6" t="n"/>
+      <c r="I29" s="6" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  18.10.2026</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="n"/>
-      <c r="C30" s="6" t="n"/>
-      <c r="D30" s="6" t="n"/>
-      <c r="E30" s="6" t="n"/>
-      <c r="F30" s="6" t="n"/>
-      <c r="G30" s="6" t="n"/>
-      <c r="H30" s="6" t="n"/>
-      <c r="I30" s="6" t="n"/>
+      <c r="A30" s="45" t="inlineStr">
+        <is>
+          <t>18.10.2026</t>
+        </is>
+      </c>
+      <c r="B30" s="45" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C30" s="45" t="inlineStr">
+        <is>
+          <t>İspanya</t>
+        </is>
+      </c>
+      <c r="D30" s="45" t="inlineStr">
+        <is>
+          <t>Primera Division</t>
+        </is>
+      </c>
+      <c r="E30" s="51" t="inlineStr">
+        <is>
+          <t>CA Osasuna</t>
+        </is>
+      </c>
+      <c r="F30" s="51" t="inlineStr">
+        <is>
+          <t>Real Racing Club de Santander</t>
+        </is>
+      </c>
+      <c r="G30" s="45" t="inlineStr">
+        <is>
+          <t>1.5 Üst</t>
+        </is>
+      </c>
+      <c r="H30" s="45" t="inlineStr">
+        <is>
+          <t>Üst</t>
+        </is>
+      </c>
+      <c r="I30" s="52" t="n">
+        <v>96.09999999999999</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="45" t="inlineStr">
@@ -23568,27 +23597,27 @@
       </c>
       <c r="B31" s="45" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C31" s="45" t="inlineStr">
         <is>
-          <t>İspanya</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D31" s="45" t="inlineStr">
         <is>
-          <t>Primera Division</t>
+          <t>Bundesliga</t>
         </is>
       </c>
       <c r="E31" s="51" t="inlineStr">
         <is>
-          <t>CA Osasuna</t>
+          <t>Borussia Mönchengladbach</t>
         </is>
       </c>
       <c r="F31" s="51" t="inlineStr">
         <is>
-          <t>Real Racing Club de Santander</t>
+          <t>TSG 1899 Hoffenheim</t>
         </is>
       </c>
       <c r="G31" s="45" t="inlineStr">
@@ -23602,7 +23631,7 @@
         </is>
       </c>
       <c r="I31" s="52" t="n">
-        <v>96.09999999999999</v>
+        <v>94.59999999999999</v>
       </c>
     </row>
     <row r="32">
@@ -23613,7 +23642,7 @@
       </c>
       <c r="B32" s="45" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C32" s="45" t="inlineStr">
@@ -23628,12 +23657,12 @@
       </c>
       <c r="E32" s="51" t="inlineStr">
         <is>
-          <t>Borussia Mönchengladbach</t>
+          <t>Bayer 04 Leverkusen</t>
         </is>
       </c>
       <c r="F32" s="51" t="inlineStr">
         <is>
-          <t>TSG 1899 Hoffenheim</t>
+          <t>SC Freiburg</t>
         </is>
       </c>
       <c r="G32" s="45" t="inlineStr">
@@ -23647,7 +23676,7 @@
         </is>
       </c>
       <c r="I32" s="52" t="n">
-        <v>95.5</v>
+        <v>93.59999999999999</v>
       </c>
     </row>
     <row r="33">
@@ -23658,27 +23687,27 @@
       </c>
       <c r="B33" s="45" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>02:30</t>
         </is>
       </c>
       <c r="C33" s="45" t="inlineStr">
         <is>
-          <t>Almanya</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D33" s="45" t="inlineStr">
         <is>
-          <t>Bundesliga</t>
+          <t>MLS</t>
         </is>
       </c>
       <c r="E33" s="51" t="inlineStr">
         <is>
-          <t>Bayer 04 Leverkusen</t>
+          <t>Orlando City</t>
         </is>
       </c>
       <c r="F33" s="51" t="inlineStr">
         <is>
-          <t>SC Freiburg</t>
+          <t>DC United</t>
         </is>
       </c>
       <c r="G33" s="45" t="inlineStr">
@@ -23692,7 +23721,7 @@
         </is>
       </c>
       <c r="I33" s="52" t="n">
-        <v>94.5</v>
+        <v>93</v>
       </c>
     </row>
     <row r="34">
@@ -23718,12 +23747,12 @@
       </c>
       <c r="E34" s="51" t="inlineStr">
         <is>
-          <t>Orlando City</t>
+          <t>New England Revolution</t>
         </is>
       </c>
       <c r="F34" s="51" t="inlineStr">
         <is>
-          <t>DC United</t>
+          <t>Chicago Fire</t>
         </is>
       </c>
       <c r="G34" s="45" t="inlineStr">
@@ -23737,7 +23766,7 @@
         </is>
       </c>
       <c r="I34" s="52" t="n">
-        <v>93</v>
+        <v>91.7</v>
       </c>
     </row>
     <row r="35">
@@ -23748,27 +23777,27 @@
       </c>
       <c r="B35" s="45" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C35" s="45" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="D35" s="45" t="inlineStr">
         <is>
-          <t>MLS</t>
+          <t>TFF 1. Lig</t>
         </is>
       </c>
       <c r="E35" s="51" t="inlineStr">
         <is>
-          <t>New England Revolution</t>
+          <t>Kayserispor</t>
         </is>
       </c>
       <c r="F35" s="51" t="inlineStr">
         <is>
-          <t>Chicago Fire</t>
+          <t>Batman Petrolspor</t>
         </is>
       </c>
       <c r="G35" s="45" t="inlineStr">
@@ -23798,22 +23827,22 @@
       </c>
       <c r="C36" s="45" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>İngiltere</t>
         </is>
       </c>
       <c r="D36" s="45" t="inlineStr">
         <is>
-          <t>TFF 1. Lig</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="E36" s="51" t="inlineStr">
         <is>
-          <t>Kayserispor</t>
+          <t>AFC Bournemouth</t>
         </is>
       </c>
       <c r="F36" s="51" t="inlineStr">
         <is>
-          <t>Batman Petrolspor</t>
+          <t>Sunderland AFC</t>
         </is>
       </c>
       <c r="G36" s="45" t="inlineStr">
@@ -23827,7 +23856,7 @@
         </is>
       </c>
       <c r="I36" s="52" t="n">
-        <v>91.7</v>
+        <v>91.09999999999999</v>
       </c>
     </row>
     <row r="37">
@@ -23838,27 +23867,27 @@
       </c>
       <c r="B37" s="45" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>02:30</t>
         </is>
       </c>
       <c r="C37" s="45" t="inlineStr">
         <is>
-          <t>İngiltere</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D37" s="45" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>MLS</t>
         </is>
       </c>
       <c r="E37" s="51" t="inlineStr">
         <is>
-          <t>AFC Bournemouth</t>
+          <t>Atlanta Utd</t>
         </is>
       </c>
       <c r="F37" s="51" t="inlineStr">
         <is>
-          <t>Sunderland AFC</t>
+          <t>Inter Miami</t>
         </is>
       </c>
       <c r="G37" s="45" t="inlineStr">
@@ -23872,97 +23901,97 @@
         </is>
       </c>
       <c r="I37" s="52" t="n">
-        <v>91.09999999999999</v>
+        <v>90.90000000000001</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="45" t="inlineStr">
+      <c r="A38" s="53" t="inlineStr">
         <is>
           <t>18.10.2026</t>
         </is>
       </c>
-      <c r="B38" s="45" t="inlineStr">
-        <is>
-          <t>02:30</t>
-        </is>
-      </c>
-      <c r="C38" s="45" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D38" s="45" t="inlineStr">
-        <is>
-          <t>MLS</t>
-        </is>
-      </c>
-      <c r="E38" s="51" t="inlineStr">
-        <is>
-          <t>Atlanta Utd</t>
-        </is>
-      </c>
-      <c r="F38" s="51" t="inlineStr">
-        <is>
-          <t>Inter Miami</t>
-        </is>
-      </c>
-      <c r="G38" s="45" t="inlineStr">
-        <is>
-          <t>1.5 Üst</t>
-        </is>
-      </c>
-      <c r="H38" s="45" t="inlineStr">
-        <is>
-          <t>Üst</t>
-        </is>
-      </c>
-      <c r="I38" s="52" t="n">
-        <v>90.90000000000001</v>
+      <c r="B38" s="53" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="C38" s="53" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="D38" s="53" t="inlineStr">
+        <is>
+          <t>TFF 1. Lig</t>
+        </is>
+      </c>
+      <c r="E38" s="54" t="inlineStr">
+        <is>
+          <t>Igdir FK</t>
+        </is>
+      </c>
+      <c r="F38" s="54" t="inlineStr">
+        <is>
+          <t>Boluspor</t>
+        </is>
+      </c>
+      <c r="G38" s="53" t="inlineStr">
+        <is>
+          <t>Çifte Şans</t>
+        </is>
+      </c>
+      <c r="H38" s="53" t="inlineStr">
+        <is>
+          <t>1X</t>
+        </is>
+      </c>
+      <c r="I38" s="55" t="n">
+        <v>89.90000000000001</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="45" t="inlineStr">
+      <c r="A39" s="53" t="inlineStr">
         <is>
           <t>18.10.2026</t>
         </is>
       </c>
-      <c r="B39" s="45" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="C39" s="45" t="inlineStr">
-        <is>
-          <t>İtalya</t>
-        </is>
-      </c>
-      <c r="D39" s="45" t="inlineStr">
-        <is>
-          <t>Serie A</t>
-        </is>
-      </c>
-      <c r="E39" s="51" t="inlineStr">
-        <is>
-          <t>Udinese Calcio</t>
-        </is>
-      </c>
-      <c r="F39" s="51" t="inlineStr">
-        <is>
-          <t>US Lecce</t>
-        </is>
-      </c>
-      <c r="G39" s="45" t="inlineStr">
-        <is>
-          <t>1.5 Üst</t>
-        </is>
-      </c>
-      <c r="H39" s="45" t="inlineStr">
-        <is>
-          <t>Üst</t>
-        </is>
-      </c>
-      <c r="I39" s="52" t="n">
-        <v>90.5</v>
+      <c r="B39" s="53" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C39" s="53" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="D39" s="53" t="inlineStr">
+        <is>
+          <t>TFF 1. Lig</t>
+        </is>
+      </c>
+      <c r="E39" s="54" t="inlineStr">
+        <is>
+          <t>Kayserispor</t>
+        </is>
+      </c>
+      <c r="F39" s="54" t="inlineStr">
+        <is>
+          <t>Batman Petrolspor</t>
+        </is>
+      </c>
+      <c r="G39" s="53" t="inlineStr">
+        <is>
+          <t>Çifte Şans</t>
+        </is>
+      </c>
+      <c r="H39" s="53" t="inlineStr">
+        <is>
+          <t>1X</t>
+        </is>
+      </c>
+      <c r="I39" s="55" t="n">
+        <v>86.2</v>
       </c>
     </row>
     <row r="40">
@@ -23973,27 +24002,27 @@
       </c>
       <c r="B40" s="53" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C40" s="53" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>İtalya</t>
         </is>
       </c>
       <c r="D40" s="53" t="inlineStr">
         <is>
-          <t>TFF 1. Lig</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="E40" s="54" t="inlineStr">
         <is>
-          <t>Igdir FK</t>
+          <t>AC Milan</t>
         </is>
       </c>
       <c r="F40" s="54" t="inlineStr">
         <is>
-          <t>Boluspor</t>
+          <t>Atalanta BC</t>
         </is>
       </c>
       <c r="G40" s="53" t="inlineStr">
@@ -24007,7 +24036,7 @@
         </is>
       </c>
       <c r="I40" s="55" t="n">
-        <v>89.90000000000001</v>
+        <v>86.09999999999999</v>
       </c>
     </row>
     <row r="41">
@@ -24023,22 +24052,22 @@
       </c>
       <c r="C41" s="53" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>İngiltere</t>
         </is>
       </c>
       <c r="D41" s="53" t="inlineStr">
         <is>
-          <t>TFF 1. Lig</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="E41" s="54" t="inlineStr">
         <is>
-          <t>Kayserispor</t>
+          <t>Brighton &amp; Hove Albion FC</t>
         </is>
       </c>
       <c r="F41" s="54" t="inlineStr">
         <is>
-          <t>Batman Petrolspor</t>
+          <t>Crystal Palace FC</t>
         </is>
       </c>
       <c r="G41" s="53" t="inlineStr">
@@ -24052,7 +24081,7 @@
         </is>
       </c>
       <c r="I41" s="55" t="n">
-        <v>86.2</v>
+        <v>86</v>
       </c>
     </row>
     <row r="42">
@@ -24063,27 +24092,27 @@
       </c>
       <c r="B42" s="53" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>05:30</t>
         </is>
       </c>
       <c r="C42" s="53" t="inlineStr">
         <is>
-          <t>İngiltere</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D42" s="53" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>MLS</t>
         </is>
       </c>
       <c r="E42" s="54" t="inlineStr">
         <is>
-          <t>Brighton &amp; Hove Albion FC</t>
+          <t>Seattle Sounders</t>
         </is>
       </c>
       <c r="F42" s="54" t="inlineStr">
         <is>
-          <t>Crystal Palace FC</t>
+          <t>CF Montreal</t>
         </is>
       </c>
       <c r="G42" s="53" t="inlineStr">
@@ -24097,7 +24126,7 @@
         </is>
       </c>
       <c r="I42" s="55" t="n">
-        <v>86</v>
+        <v>84.59999999999999</v>
       </c>
     </row>
     <row r="43">
@@ -24108,27 +24137,27 @@
       </c>
       <c r="B43" s="53" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C43" s="53" t="inlineStr">
         <is>
-          <t>İtalya</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="D43" s="53" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>Süper Lig</t>
         </is>
       </c>
       <c r="E43" s="54" t="inlineStr">
         <is>
-          <t>AC Milan</t>
+          <t>Kasimpasa</t>
         </is>
       </c>
       <c r="F43" s="54" t="inlineStr">
         <is>
-          <t>Atalanta BC</t>
+          <t>Samsunspor</t>
         </is>
       </c>
       <c r="G43" s="53" t="inlineStr">
@@ -24142,7 +24171,7 @@
         </is>
       </c>
       <c r="I43" s="55" t="n">
-        <v>85.09999999999999</v>
+        <v>84.5</v>
       </c>
     </row>
     <row r="44">
@@ -24153,7 +24182,7 @@
       </c>
       <c r="B44" s="53" t="inlineStr">
         <is>
-          <t>05:30</t>
+          <t>02:30</t>
         </is>
       </c>
       <c r="C44" s="53" t="inlineStr">
@@ -24168,12 +24197,12 @@
       </c>
       <c r="E44" s="54" t="inlineStr">
         <is>
-          <t>Seattle Sounders</t>
+          <t>Orlando City</t>
         </is>
       </c>
       <c r="F44" s="54" t="inlineStr">
         <is>
-          <t>CF Montreal</t>
+          <t>DC United</t>
         </is>
       </c>
       <c r="G44" s="53" t="inlineStr">
@@ -24187,7 +24216,7 @@
         </is>
       </c>
       <c r="I44" s="55" t="n">
-        <v>84.59999999999999</v>
+        <v>84.09999999999999</v>
       </c>
     </row>
     <row r="45">
@@ -24198,27 +24227,27 @@
       </c>
       <c r="B45" s="53" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C45" s="53" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>İtalya</t>
         </is>
       </c>
       <c r="D45" s="53" t="inlineStr">
         <is>
-          <t>Süper Lig</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="E45" s="54" t="inlineStr">
         <is>
-          <t>Kasimpasa</t>
+          <t>ACF Fiorentina</t>
         </is>
       </c>
       <c r="F45" s="54" t="inlineStr">
         <is>
-          <t>Samsunspor</t>
+          <t>Como 1907</t>
         </is>
       </c>
       <c r="G45" s="53" t="inlineStr">
@@ -24232,7 +24261,7 @@
         </is>
       </c>
       <c r="I45" s="55" t="n">
-        <v>84.5</v>
+        <v>81.8</v>
       </c>
     </row>
     <row r="46">
@@ -24243,27 +24272,27 @@
       </c>
       <c r="B46" s="53" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C46" s="53" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>İspanya</t>
         </is>
       </c>
       <c r="D46" s="53" t="inlineStr">
         <is>
-          <t>MLS</t>
+          <t>Primera Division</t>
         </is>
       </c>
       <c r="E46" s="54" t="inlineStr">
         <is>
-          <t>Orlando City</t>
+          <t>RC Celta de Vigo</t>
         </is>
       </c>
       <c r="F46" s="54" t="inlineStr">
         <is>
-          <t>DC United</t>
+          <t>Deportivo Alavés</t>
         </is>
       </c>
       <c r="G46" s="53" t="inlineStr">
@@ -24277,7 +24306,7 @@
         </is>
       </c>
       <c r="I46" s="55" t="n">
-        <v>84.09999999999999</v>
+        <v>81.40000000000001</v>
       </c>
     </row>
     <row r="47">
@@ -24288,27 +24317,27 @@
       </c>
       <c r="B47" s="53" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="C47" s="53" t="inlineStr">
         <is>
-          <t>İtalya</t>
+          <t>Fransa</t>
         </is>
       </c>
       <c r="D47" s="53" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="E47" s="54" t="inlineStr">
         <is>
-          <t>ACF Fiorentina</t>
+          <t>Olympique Lyonnais</t>
         </is>
       </c>
       <c r="F47" s="54" t="inlineStr">
         <is>
-          <t>Como 1907</t>
+          <t>OGC Nice</t>
         </is>
       </c>
       <c r="G47" s="53" t="inlineStr">
@@ -24322,254 +24351,164 @@
         </is>
       </c>
       <c r="I47" s="55" t="n">
-        <v>82.5</v>
+        <v>81.2</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="53" t="inlineStr">
-        <is>
-          <t>18.10.2026</t>
-        </is>
-      </c>
-      <c r="B48" s="53" t="inlineStr">
-        <is>
-          <t>17:15</t>
-        </is>
-      </c>
-      <c r="C48" s="53" t="inlineStr">
-        <is>
-          <t>İspanya</t>
-        </is>
-      </c>
-      <c r="D48" s="53" t="inlineStr">
-        <is>
-          <t>Primera Division</t>
-        </is>
-      </c>
-      <c r="E48" s="54" t="inlineStr">
-        <is>
-          <t>RC Celta de Vigo</t>
-        </is>
-      </c>
-      <c r="F48" s="54" t="inlineStr">
-        <is>
-          <t>Deportivo Alavés</t>
-        </is>
-      </c>
-      <c r="G48" s="53" t="inlineStr">
-        <is>
-          <t>Çifte Şans</t>
-        </is>
-      </c>
-      <c r="H48" s="53" t="inlineStr">
-        <is>
-          <t>1X</t>
-        </is>
-      </c>
-      <c r="I48" s="55" t="n">
-        <v>81.40000000000001</v>
-      </c>
+      <c r="A48" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  19.10.2026</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="n"/>
+      <c r="C48" s="6" t="n"/>
+      <c r="D48" s="6" t="n"/>
+      <c r="E48" s="6" t="n"/>
+      <c r="F48" s="6" t="n"/>
+      <c r="G48" s="6" t="n"/>
+      <c r="H48" s="6" t="n"/>
+      <c r="I48" s="6" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="53" t="inlineStr">
-        <is>
-          <t>18.10.2026</t>
-        </is>
-      </c>
-      <c r="B49" s="53" t="inlineStr">
-        <is>
-          <t>21:45</t>
-        </is>
-      </c>
-      <c r="C49" s="53" t="inlineStr">
-        <is>
-          <t>Fransa</t>
-        </is>
-      </c>
-      <c r="D49" s="53" t="inlineStr">
-        <is>
-          <t>Ligue 1</t>
-        </is>
-      </c>
-      <c r="E49" s="54" t="inlineStr">
-        <is>
-          <t>Olympique Lyonnais</t>
-        </is>
-      </c>
-      <c r="F49" s="54" t="inlineStr">
-        <is>
-          <t>OGC Nice</t>
-        </is>
-      </c>
-      <c r="G49" s="53" t="inlineStr">
-        <is>
-          <t>Çifte Şans</t>
-        </is>
-      </c>
-      <c r="H49" s="53" t="inlineStr">
-        <is>
-          <t>1X</t>
-        </is>
-      </c>
-      <c r="I49" s="55" t="n">
-        <v>81.2</v>
+      <c r="A49" s="45" t="inlineStr">
+        <is>
+          <t>19.10.2026</t>
+        </is>
+      </c>
+      <c r="B49" s="45" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="C49" s="45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D49" s="45" t="inlineStr">
+        <is>
+          <t>MLS</t>
+        </is>
+      </c>
+      <c r="E49" s="51" t="inlineStr">
+        <is>
+          <t>FC Cincinnati</t>
+        </is>
+      </c>
+      <c r="F49" s="51" t="inlineStr">
+        <is>
+          <t>Columbus Crew</t>
+        </is>
+      </c>
+      <c r="G49" s="45" t="inlineStr">
+        <is>
+          <t>1.5 Üst</t>
+        </is>
+      </c>
+      <c r="H49" s="45" t="inlineStr">
+        <is>
+          <t>Üst</t>
+        </is>
+      </c>
+      <c r="I49" s="52" t="n">
+        <v>94.2</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  19.10.2026</t>
-        </is>
-      </c>
-      <c r="B50" s="6" t="n"/>
-      <c r="C50" s="6" t="n"/>
-      <c r="D50" s="6" t="n"/>
-      <c r="E50" s="6" t="n"/>
-      <c r="F50" s="6" t="n"/>
-      <c r="G50" s="6" t="n"/>
-      <c r="H50" s="6" t="n"/>
-      <c r="I50" s="6" t="n"/>
+      <c r="A50" s="53" t="inlineStr">
+        <is>
+          <t>19.10.2026</t>
+        </is>
+      </c>
+      <c r="B50" s="53" t="inlineStr">
+        <is>
+          <t>02:15</t>
+        </is>
+      </c>
+      <c r="C50" s="53" t="inlineStr">
+        <is>
+          <t>Arjantin</t>
+        </is>
+      </c>
+      <c r="D50" s="53" t="inlineStr">
+        <is>
+          <t>Liga Profesional (Arjantin)</t>
+        </is>
+      </c>
+      <c r="E50" s="54" t="inlineStr">
+        <is>
+          <t>Belgrano</t>
+        </is>
+      </c>
+      <c r="F50" s="54" t="inlineStr">
+        <is>
+          <t>River Plate</t>
+        </is>
+      </c>
+      <c r="G50" s="53" t="inlineStr">
+        <is>
+          <t>Çifte Şans</t>
+        </is>
+      </c>
+      <c r="H50" s="53" t="inlineStr">
+        <is>
+          <t>1X</t>
+        </is>
+      </c>
+      <c r="I50" s="55" t="n">
+        <v>83.7</v>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="45" t="inlineStr">
+      <c r="A51" s="53" t="inlineStr">
         <is>
           <t>19.10.2026</t>
         </is>
       </c>
-      <c r="B51" s="45" t="inlineStr">
+      <c r="B51" s="53" t="inlineStr">
         <is>
           <t>00:00</t>
         </is>
       </c>
-      <c r="C51" s="45" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D51" s="45" t="inlineStr">
-        <is>
-          <t>MLS</t>
-        </is>
-      </c>
-      <c r="E51" s="51" t="inlineStr">
-        <is>
-          <t>FC Cincinnati</t>
-        </is>
-      </c>
-      <c r="F51" s="51" t="inlineStr">
-        <is>
-          <t>Columbus Crew</t>
-        </is>
-      </c>
-      <c r="G51" s="45" t="inlineStr">
-        <is>
-          <t>1.5 Üst</t>
-        </is>
-      </c>
-      <c r="H51" s="45" t="inlineStr">
-        <is>
-          <t>Üst</t>
-        </is>
-      </c>
-      <c r="I51" s="52" t="n">
-        <v>94.2</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="53" t="inlineStr">
-        <is>
-          <t>19.10.2026</t>
-        </is>
-      </c>
-      <c r="B52" s="53" t="inlineStr">
-        <is>
-          <t>02:15</t>
-        </is>
-      </c>
-      <c r="C52" s="53" t="inlineStr">
+      <c r="C51" s="53" t="inlineStr">
         <is>
           <t>Arjantin</t>
         </is>
       </c>
-      <c r="D52" s="53" t="inlineStr">
+      <c r="D51" s="53" t="inlineStr">
         <is>
           <t>Liga Profesional (Arjantin)</t>
         </is>
       </c>
-      <c r="E52" s="54" t="inlineStr">
-        <is>
-          <t>Belgrano</t>
-        </is>
-      </c>
-      <c r="F52" s="54" t="inlineStr">
-        <is>
-          <t>River Plate</t>
-        </is>
-      </c>
-      <c r="G52" s="53" t="inlineStr">
+      <c r="E51" s="54" t="inlineStr">
+        <is>
+          <t>Estudiantes L.P.</t>
+        </is>
+      </c>
+      <c r="F51" s="54" t="inlineStr">
+        <is>
+          <t>San Lorenzo</t>
+        </is>
+      </c>
+      <c r="G51" s="53" t="inlineStr">
         <is>
           <t>Çifte Şans</t>
         </is>
       </c>
-      <c r="H52" s="53" t="inlineStr">
+      <c r="H51" s="53" t="inlineStr">
         <is>
           <t>1X</t>
         </is>
       </c>
-      <c r="I52" s="55" t="n">
-        <v>83.7</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="53" t="inlineStr">
-        <is>
-          <t>19.10.2026</t>
-        </is>
-      </c>
-      <c r="B53" s="53" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="C53" s="53" t="inlineStr">
-        <is>
-          <t>Arjantin</t>
-        </is>
-      </c>
-      <c r="D53" s="53" t="inlineStr">
-        <is>
-          <t>Liga Profesional (Arjantin)</t>
-        </is>
-      </c>
-      <c r="E53" s="54" t="inlineStr">
-        <is>
-          <t>Estudiantes L.P.</t>
-        </is>
-      </c>
-      <c r="F53" s="54" t="inlineStr">
-        <is>
-          <t>San Lorenzo</t>
-        </is>
-      </c>
-      <c r="G53" s="53" t="inlineStr">
-        <is>
-          <t>Çifte Şans</t>
-        </is>
-      </c>
-      <c r="H53" s="53" t="inlineStr">
-        <is>
-          <t>1X</t>
-        </is>
-      </c>
-      <c r="I53" s="55" t="n">
+      <c r="I51" s="55" t="n">
         <v>82.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I53"/>
+  <autoFilter ref="A1:I51"/>
   <mergeCells count="4">
-    <mergeCell ref="A30:I30"/>
-    <mergeCell ref="A50:I50"/>
+    <mergeCell ref="A29:I29"/>
+    <mergeCell ref="A48:I48"/>
     <mergeCell ref="A8:I8"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
@@ -24602,7 +24541,7 @@
     <row r="3">
       <c r="A3" s="57" t="inlineStr">
         <is>
-          <t>Oluşturulma zamanı: 16.10.2026 13:37</t>
+          <t>Oluşturulma zamanı: 16.10.2026 18:36</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Güncelle: otomatik GitHub Actions güncellemesi (2026-10-17 10:32 UTC)
</commit_message>
<xml_diff>
--- a/maclar_ve_tahminler.xlsx
+++ b/maclar_ve_tahminler.xlsx
@@ -3132,59 +3132,63 @@
         </is>
       </c>
       <c r="N18" s="43" t="n">
-        <v>61.3</v>
+        <v>63.2</v>
       </c>
       <c r="O18" s="43" t="n">
-        <v>21.1</v>
+        <v>20.8</v>
       </c>
       <c r="P18" s="43" t="n">
-        <v>17.5</v>
+        <v>16</v>
       </c>
       <c r="Q18" s="44" t="n">
         <v>1.9</v>
       </c>
       <c r="R18" s="44" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.59</v>
       </c>
       <c r="S18" s="43" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="T18" s="43" t="n">
         <v>50.6</v>
       </c>
-      <c r="T18" s="43" t="n">
-        <v>49.4</v>
-      </c>
       <c r="U18" s="43" t="n">
-        <v>49.1</v>
+        <v>46.8</v>
       </c>
       <c r="V18" s="43" t="n">
-        <v>50.9</v>
+        <v>53.2</v>
       </c>
       <c r="W18" s="43" t="n">
-        <v>72.09999999999999</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="X18" s="43" t="n">
-        <v>82.5</v>
+        <v>84</v>
       </c>
       <c r="Y18" s="43" t="n">
-        <v>38.7</v>
+        <v>36.8</v>
       </c>
       <c r="Z18" s="43" t="n">
-        <v>78.90000000000001</v>
+        <v>79.2</v>
       </c>
       <c r="AA18" s="43" t="n">
-        <v>47.1</v>
+        <v>48.5</v>
       </c>
       <c r="AB18" s="43" t="n">
-        <v>40</v>
+        <v>40.5</v>
       </c>
       <c r="AC18" s="43" t="n">
-        <v>12.9</v>
+        <v>11</v>
       </c>
       <c r="AD18" s="45" t="inlineStr">
         <is>
-          <t>1-0 (%15)</t>
-        </is>
-      </c>
-      <c r="AE18" s="40" t="n"/>
+          <t>1-0 (%17)</t>
+        </is>
+      </c>
+      <c r="AE18" s="40" t="inlineStr">
+        <is>
+          <t>Dep kilit oyuncu eksik (Abdullahi A.) -&gt; hücum -%15</t>
+        </is>
+      </c>
       <c r="AF18" s="40" t="inlineStr">
         <is>
           <t>Mertoglu E.</t>
@@ -3202,7 +3206,8 @@
       </c>
       <c r="AI18" s="40" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Kesin) Taskiran, Ovacikli, Gerxhaliu, Yumlu, Mujakic, Giorbelidze, Baiye, Owusu, Rodriguez, Tozlu, Cardoso
+DEP: (Kesin) Bilgin, Michalak, El Yamiq, Jules, Yasar, Giordano, Massanga Matondo, Taskin, Raux Yao, Boutobba, Barasi</t>
         </is>
       </c>
     </row>
@@ -3338,12 +3343,13 @@
       </c>
       <c r="AH19" s="46" t="inlineStr">
         <is>
-          <t>14°C, Hafif yağmur, 7 km/sa</t>
+          <t>14°C, Hafif yağmur, 11 km/sa</t>
         </is>
       </c>
       <c r="AI19" s="46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Kesin) Hellstern, Reich, Heuer, Blank, Itter, Banse, Will, Klaus, Appelkamp, Pohlmann, Sillah
+DEP: (Kesin) Hoffmann, Aydin, Ehlers, Frenkert, Di Michele Sanchez, Opoku, Di Benedetto, Flick, Marie, Sturm, Urbich</t>
         </is>
       </c>
     </row>
@@ -3414,59 +3420,63 @@
         </is>
       </c>
       <c r="N20" s="43" t="n">
-        <v>51.1</v>
+        <v>47</v>
       </c>
       <c r="O20" s="43" t="n">
-        <v>27.2</v>
+        <v>29.3</v>
       </c>
       <c r="P20" s="43" t="n">
-        <v>21.7</v>
+        <v>23.7</v>
       </c>
       <c r="Q20" s="44" t="n">
-        <v>1.26</v>
+        <v>1.07</v>
       </c>
       <c r="R20" s="44" t="n">
         <v>0.63</v>
       </c>
       <c r="S20" s="43" t="n">
-        <v>41.7</v>
+        <v>38.9</v>
       </c>
       <c r="T20" s="43" t="n">
-        <v>58.3</v>
+        <v>61.1</v>
       </c>
       <c r="U20" s="43" t="n">
-        <v>44.6</v>
+        <v>43</v>
       </c>
       <c r="V20" s="43" t="n">
-        <v>55.4</v>
+        <v>57</v>
       </c>
       <c r="W20" s="43" t="n">
-        <v>55.7</v>
+        <v>50</v>
       </c>
       <c r="X20" s="43" t="n">
-        <v>78.3</v>
+        <v>76.3</v>
       </c>
       <c r="Y20" s="43" t="n">
-        <v>48.9</v>
+        <v>53</v>
       </c>
       <c r="Z20" s="43" t="n">
-        <v>72.8</v>
+        <v>70.7</v>
       </c>
       <c r="AA20" s="43" t="n">
-        <v>35.1</v>
+        <v>30.7</v>
       </c>
       <c r="AB20" s="43" t="n">
-        <v>49.8</v>
+        <v>53</v>
       </c>
       <c r="AC20" s="43" t="n">
-        <v>15.2</v>
+        <v>16.3</v>
       </c>
       <c r="AD20" s="45" t="inlineStr">
         <is>
           <t>1-0 (%20)</t>
         </is>
       </c>
-      <c r="AE20" s="40" t="n"/>
+      <c r="AE20" s="40" t="inlineStr">
+        <is>
+          <t>Ev kilit oyuncu eksik (Tazemeta T.) -&gt; hücum -%15</t>
+        </is>
+      </c>
       <c r="AF20" s="40" t="inlineStr">
         <is>
           <t>Haslberger W.</t>
@@ -3479,12 +3489,13 @@
       </c>
       <c r="AH20" s="40" t="inlineStr">
         <is>
-          <t>11°C, Hafif yağmur, 8 km/sa</t>
+          <t>11°C, Hafif yağmur, 5 km/sa</t>
         </is>
       </c>
       <c r="AI20" s="40" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Kesin) Krahl, Elvedi, Gyamfi, Murphy, Joly, Sauer, Sahin, Haas, Skytta, Kanate, Lukovic
+DEP: (Kesin) Horn, Klaiber, Steinwender, Mets, Wittek, Meyer, Pannewig, Rasmussen, Miyoshi, Holtmann, Hofmann</t>
         </is>
       </c>
     </row>
@@ -3555,59 +3566,63 @@
         </is>
       </c>
       <c r="N21" s="43" t="n">
-        <v>59.8</v>
+        <v>63.1</v>
       </c>
       <c r="O21" s="43" t="n">
-        <v>18.6</v>
+        <v>17.9</v>
       </c>
       <c r="P21" s="43" t="n">
-        <v>21.6</v>
+        <v>19</v>
       </c>
       <c r="Q21" s="44" t="n">
         <v>3.19</v>
       </c>
       <c r="R21" s="44" t="n">
-        <v>1.71</v>
+        <v>1.45</v>
       </c>
       <c r="S21" s="43" t="n">
-        <v>71.40000000000001</v>
+        <v>69.5</v>
       </c>
       <c r="T21" s="43" t="n">
-        <v>28.6</v>
+        <v>30.5</v>
       </c>
       <c r="U21" s="43" t="n">
-        <v>68.09999999999999</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="V21" s="43" t="n">
-        <v>31.9</v>
+        <v>34.9</v>
       </c>
       <c r="W21" s="43" t="n">
-        <v>95.3</v>
+        <v>94.2</v>
       </c>
       <c r="X21" s="43" t="n">
-        <v>78.40000000000001</v>
+        <v>81</v>
       </c>
       <c r="Y21" s="43" t="n">
-        <v>40.2</v>
+        <v>36.9</v>
       </c>
       <c r="Z21" s="43" t="n">
-        <v>81.40000000000001</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="AA21" s="43" t="n">
-        <v>52.9</v>
+        <v>56</v>
       </c>
       <c r="AB21" s="43" t="n">
         <v>27</v>
       </c>
       <c r="AC21" s="43" t="n">
-        <v>20.1</v>
+        <v>16.9</v>
       </c>
       <c r="AD21" s="45" t="inlineStr">
         <is>
-          <t>3-1 (%7)</t>
-        </is>
-      </c>
-      <c r="AE21" s="46" t="n"/>
+          <t>3-1 (%8)</t>
+        </is>
+      </c>
+      <c r="AE21" s="46" t="inlineStr">
+        <is>
+          <t>Dep kilit oyuncu eksik (Zivzivadze B.) -&gt; hücum -%15</t>
+        </is>
+      </c>
       <c r="AF21" s="46" t="inlineStr">
         <is>
           <t>Bauer T.</t>
@@ -3620,12 +3635,13 @@
       </c>
       <c r="AH21" s="46" t="inlineStr">
         <is>
-          <t>11°C, Hafif yağmur, 12 km/sa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AI21" s="46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Kesin) Wellenreuther, Kumbedi, Wahl, Cleiton, Maehle, Gerhardt, Vini Souza, Damar, Bernhardsson, Glatzel, Reese
+DEP: (Kesin) Dahne, Mhamdi, Mainka, Fohrenbach, Heule, Hennrich, Schoppner, Niehues, Conteh, Kaufmann Sorensen, Vogt</t>
         </is>
       </c>
     </row>
@@ -3761,12 +3777,13 @@
       </c>
       <c r="AH22" s="40" t="inlineStr">
         <is>
-          <t>11°C, Açık, 9 km/sa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AI22" s="40" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Kesin) Pickford, Maitland-Niles, Tarkowski, Branthwaite, Mykolenko, Garner, Armstrong, Rohl, Dewsbury-Hall, Grealish, Barry
+DEP: (Kesin) Martinez, Acheampong, Lacroix, Colwill, Neto, Henderson, Caicedo, Hato, Palmer, Rogers, Joao Pedro</t>
         </is>
       </c>
     </row>
@@ -3978,59 +3995,63 @@
         </is>
       </c>
       <c r="N24" s="43" t="n">
-        <v>45.5</v>
+        <v>48</v>
       </c>
       <c r="O24" s="43" t="n">
-        <v>28.8</v>
+        <v>29</v>
       </c>
       <c r="P24" s="43" t="n">
-        <v>25.6</v>
+        <v>23</v>
       </c>
       <c r="Q24" s="44" t="n">
         <v>1.38</v>
       </c>
       <c r="R24" s="44" t="n">
-        <v>0.9</v>
+        <v>0.76</v>
       </c>
       <c r="S24" s="43" t="n">
-        <v>46.9</v>
+        <v>45.1</v>
       </c>
       <c r="T24" s="43" t="n">
-        <v>53.1</v>
+        <v>54.9</v>
       </c>
       <c r="U24" s="43" t="n">
-        <v>50.9</v>
+        <v>48.7</v>
       </c>
       <c r="V24" s="43" t="n">
-        <v>49.1</v>
+        <v>51.3</v>
       </c>
       <c r="W24" s="43" t="n">
-        <v>67.2</v>
+        <v>63.9</v>
       </c>
       <c r="X24" s="43" t="n">
-        <v>74.40000000000001</v>
+        <v>77</v>
       </c>
       <c r="Y24" s="43" t="n">
-        <v>54.5</v>
+        <v>52</v>
       </c>
       <c r="Z24" s="43" t="n">
-        <v>71.2</v>
+        <v>71</v>
       </c>
       <c r="AA24" s="43" t="n">
-        <v>34.5</v>
+        <v>36.1</v>
       </c>
       <c r="AB24" s="43" t="n">
-        <v>45.4</v>
+        <v>46.7</v>
       </c>
       <c r="AC24" s="43" t="n">
-        <v>20</v>
+        <v>17.2</v>
       </c>
       <c r="AD24" s="45" t="inlineStr">
         <is>
-          <t>1-1 (%13)</t>
-        </is>
-      </c>
-      <c r="AE24" s="40" t="n"/>
+          <t>1-0 (%15)</t>
+        </is>
+      </c>
+      <c r="AE24" s="40" t="inlineStr">
+        <is>
+          <t>Dep kilit oyuncu eksik (Baghdadi S.) -&gt; hücum -%15</t>
+        </is>
+      </c>
       <c r="AF24" s="40" t="inlineStr">
         <is>
           <t>Angoula G.</t>
@@ -4048,7 +4069,8 @@
       </c>
       <c r="AI24" s="40" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Tahmini) Fischer, Sarr, Devenish, Ruiz, Miguel, Deminguet, Munongo, Abuashvili, Toure, Kadamani, Fall
+DEP: (Tahmini) Jeannin, N'Gatta, Peybernes, Agouzoul, Gomis, Diawara, Masson, Nomel, Demoncy, Gomel, Djoco</t>
         </is>
       </c>
     </row>
@@ -4189,7 +4211,8 @@
       </c>
       <c r="AI25" s="46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: -
+DEP: -</t>
         </is>
       </c>
     </row>
@@ -4260,59 +4283,63 @@
         </is>
       </c>
       <c r="N26" s="43" t="n">
-        <v>30.8</v>
+        <v>30.3</v>
       </c>
       <c r="O26" s="43" t="n">
-        <v>27.9</v>
+        <v>29.9</v>
       </c>
       <c r="P26" s="43" t="n">
-        <v>41.3</v>
+        <v>39.9</v>
       </c>
       <c r="Q26" s="44" t="n">
-        <v>1.39</v>
+        <v>1.18</v>
       </c>
       <c r="R26" s="44" t="n">
-        <v>1.74</v>
+        <v>1.48</v>
       </c>
       <c r="S26" s="43" t="n">
-        <v>56.4</v>
+        <v>51.4</v>
       </c>
       <c r="T26" s="43" t="n">
-        <v>43.6</v>
+        <v>48.6</v>
       </c>
       <c r="U26" s="43" t="n">
-        <v>59.9</v>
+        <v>55.9</v>
       </c>
       <c r="V26" s="43" t="n">
-        <v>40.1</v>
+        <v>44.1</v>
       </c>
       <c r="W26" s="43" t="n">
-        <v>83.40000000000001</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="X26" s="43" t="n">
-        <v>58.7</v>
+        <v>60.1</v>
       </c>
       <c r="Y26" s="43" t="n">
-        <v>69.2</v>
+        <v>69.7</v>
       </c>
       <c r="Z26" s="43" t="n">
-        <v>72.09999999999999</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="AA26" s="43" t="n">
-        <v>27.1</v>
+        <v>25.7</v>
       </c>
       <c r="AB26" s="43" t="n">
-        <v>35.6</v>
+        <v>39.3</v>
       </c>
       <c r="AC26" s="43" t="n">
-        <v>37.3</v>
+        <v>35</v>
       </c>
       <c r="AD26" s="45" t="inlineStr">
         <is>
-          <t>1-1 (%12)</t>
-        </is>
-      </c>
-      <c r="AE26" s="40" t="n"/>
+          <t>1-1 (%14)</t>
+        </is>
+      </c>
+      <c r="AE26" s="40" t="inlineStr">
+        <is>
+          <t>Ev kilit oyuncu eksik (Sagrado R.) -&gt; hücum -%15 | Dep kilit oyuncu eksik (De Bruyne K.) -&gt; hücum -%15</t>
+        </is>
+      </c>
       <c r="AF26" s="40" t="inlineStr">
         <is>
           <t>Sacchi J. L.</t>
@@ -4330,7 +4357,8 @@
       </c>
       <c r="AI26" s="40" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Tahmini) Stankovic, Schingtienne, Juan Jesus, Moreno, Hainaut, Perez, Basic, Sohm, Haps, Yeboah, Adams
+DEP: (Tahmini) Meret, Beukema, Rrahmani, Badiashile, Di Lorenzo, Gilmour, Lobotka, Spinazzola, Giovane, McTominay, Hojlund</t>
         </is>
       </c>
     </row>
@@ -4401,59 +4429,63 @@
         </is>
       </c>
       <c r="N27" s="43" t="n">
-        <v>66.5</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="O27" s="43" t="n">
-        <v>18.1</v>
+        <v>17.6</v>
       </c>
       <c r="P27" s="43" t="n">
-        <v>15.4</v>
+        <v>14</v>
       </c>
       <c r="Q27" s="44" t="n">
         <v>2.35</v>
       </c>
       <c r="R27" s="44" t="n">
-        <v>0.77</v>
+        <v>0.66</v>
       </c>
       <c r="S27" s="43" t="n">
-        <v>56.3</v>
+        <v>55.1</v>
       </c>
       <c r="T27" s="43" t="n">
-        <v>43.7</v>
+        <v>44.9</v>
       </c>
       <c r="U27" s="43" t="n">
-        <v>52.3</v>
+        <v>49.8</v>
       </c>
       <c r="V27" s="43" t="n">
-        <v>47.7</v>
+        <v>50.2</v>
       </c>
       <c r="W27" s="43" t="n">
-        <v>81.09999999999999</v>
+        <v>79.5</v>
       </c>
       <c r="X27" s="43" t="n">
-        <v>84.59999999999999</v>
+        <v>86</v>
       </c>
       <c r="Y27" s="43" t="n">
-        <v>33.5</v>
+        <v>31.6</v>
       </c>
       <c r="Z27" s="43" t="n">
-        <v>81.90000000000001</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="AA27" s="43" t="n">
-        <v>53.5</v>
+        <v>55.1</v>
       </c>
       <c r="AB27" s="43" t="n">
-        <v>34.4</v>
+        <v>34.6</v>
       </c>
       <c r="AC27" s="43" t="n">
-        <v>12.1</v>
+        <v>10.3</v>
       </c>
       <c r="AD27" s="45" t="inlineStr">
         <is>
-          <t>2-0 (%12)</t>
-        </is>
-      </c>
-      <c r="AE27" s="46" t="n"/>
+          <t>2-0 (%14)</t>
+        </is>
+      </c>
+      <c r="AE27" s="46" t="inlineStr">
+        <is>
+          <t>Dep kilit oyuncu eksik (Colley E.) -&gt; hücum -%15</t>
+        </is>
+      </c>
       <c r="AF27" s="46" t="inlineStr">
         <is>
           <t>Ergun O.</t>
@@ -4471,7 +4503,8 @@
       </c>
       <c r="AI27" s="46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV: (Tahmini) Lafont, Krasniqi, Yesil, Bates, Meras, Raveloson, Soyalp, Ballet, Saba, Khalil, Orban
+DEP: (Tahmini) Gungordu, Andzouana, Baniya, Bosluk, Masuaku, Jevtovic, Ibrahimoglu, Turuc, Toth, Goncalves, Muleka</t>
         </is>
       </c>
     </row>
@@ -17461,27 +17494,27 @@
       </c>
       <c r="B4" s="45" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="C4" s="45" t="inlineStr">
         <is>
-          <t>Almanya</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D4" s="45" t="inlineStr">
         <is>
-          <t>2. Bundesliga</t>
+          <t>MLS</t>
         </is>
       </c>
       <c r="E4" s="51" t="inlineStr">
         <is>
-          <t>Wolfsburg</t>
+          <t>Minnesota United</t>
         </is>
       </c>
       <c r="F4" s="51" t="inlineStr">
         <is>
-          <t>Heidenheim</t>
+          <t>St. Louis City</t>
         </is>
       </c>
       <c r="G4" s="45" t="inlineStr">
@@ -17495,7 +17528,7 @@
         </is>
       </c>
       <c r="I4" s="52" t="n">
-        <v>95.3</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5">
@@ -17506,7 +17539,7 @@
       </c>
       <c r="B5" s="45" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C5" s="45" t="inlineStr">
@@ -17521,12 +17554,12 @@
       </c>
       <c r="E5" s="51" t="inlineStr">
         <is>
-          <t>Minnesota United</t>
+          <t>Philadelphia Union</t>
         </is>
       </c>
       <c r="F5" s="51" t="inlineStr">
         <is>
-          <t>St. Louis City</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="G5" s="45" t="inlineStr">
@@ -17540,7 +17573,7 @@
         </is>
       </c>
       <c r="I5" s="52" t="n">
-        <v>95</v>
+        <v>94.7</v>
       </c>
     </row>
     <row r="6">
@@ -17551,27 +17584,27 @@
       </c>
       <c r="B6" s="45" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C6" s="45" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D6" s="45" t="inlineStr">
         <is>
-          <t>MLS</t>
+          <t>2. Bundesliga</t>
         </is>
       </c>
       <c r="E6" s="51" t="inlineStr">
         <is>
-          <t>Philadelphia Union</t>
+          <t>Wolfsburg</t>
         </is>
       </c>
       <c r="F6" s="51" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Heidenheim</t>
         </is>
       </c>
       <c r="G6" s="45" t="inlineStr">
@@ -17585,7 +17618,7 @@
         </is>
       </c>
       <c r="I6" s="52" t="n">
-        <v>94.7</v>
+        <v>94.2</v>
       </c>
     </row>
     <row r="7">
@@ -17911,27 +17944,27 @@
       </c>
       <c r="B14" s="53" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C14" s="53" t="inlineStr">
         <is>
-          <t>Almanya</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="D14" s="53" t="inlineStr">
         <is>
-          <t>Bundesliga</t>
+          <t>Süper Lig</t>
         </is>
       </c>
       <c r="E14" s="54" t="inlineStr">
         <is>
-          <t>SV Werder Bremen</t>
+          <t>Amedspor</t>
         </is>
       </c>
       <c r="F14" s="54" t="inlineStr">
         <is>
-          <t>SC Paderborn 07</t>
+          <t>Konyaspor</t>
         </is>
       </c>
       <c r="G14" s="53" t="inlineStr">
@@ -17945,7 +17978,7 @@
         </is>
       </c>
       <c r="I14" s="55" t="n">
-        <v>85.7</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15">
@@ -17956,27 +17989,27 @@
       </c>
       <c r="B15" s="53" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C15" s="53" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D15" s="53" t="inlineStr">
         <is>
-          <t>MLS</t>
+          <t>Bundesliga</t>
         </is>
       </c>
       <c r="E15" s="54" t="inlineStr">
         <is>
-          <t>Philadelphia Union</t>
+          <t>SV Werder Bremen</t>
         </is>
       </c>
       <c r="F15" s="54" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>SC Paderborn 07</t>
         </is>
       </c>
       <c r="G15" s="53" t="inlineStr">
@@ -17990,7 +18023,7 @@
         </is>
       </c>
       <c r="I15" s="55" t="n">
-        <v>84.7</v>
+        <v>85.7</v>
       </c>
     </row>
     <row r="16">
@@ -18001,27 +18034,27 @@
       </c>
       <c r="B16" s="53" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C16" s="53" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D16" s="53" t="inlineStr">
         <is>
-          <t>Süper Lig</t>
+          <t>MLS</t>
         </is>
       </c>
       <c r="E16" s="54" t="inlineStr">
         <is>
-          <t>Amedspor</t>
+          <t>Philadelphia Union</t>
         </is>
       </c>
       <c r="F16" s="54" t="inlineStr">
         <is>
-          <t>Konyaspor</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="G16" s="53" t="inlineStr">
@@ -18035,7 +18068,7 @@
         </is>
       </c>
       <c r="I16" s="55" t="n">
-        <v>84.59999999999999</v>
+        <v>84.7</v>
       </c>
     </row>
     <row r="17">
@@ -18080,7 +18113,7 @@
         </is>
       </c>
       <c r="I17" s="55" t="n">
-        <v>82.5</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18">
@@ -18091,27 +18124,27 @@
       </c>
       <c r="B18" s="53" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C18" s="53" t="inlineStr">
         <is>
-          <t>Fransa</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D18" s="53" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>2. Bundesliga</t>
         </is>
       </c>
       <c r="E18" s="54" t="inlineStr">
         <is>
-          <t>Lille OSC</t>
+          <t>Wolfsburg</t>
         </is>
       </c>
       <c r="F18" s="54" t="inlineStr">
         <is>
-          <t>Stade Brestois 29</t>
+          <t>Heidenheim</t>
         </is>
       </c>
       <c r="G18" s="53" t="inlineStr">
@@ -18121,11 +18154,11 @@
       </c>
       <c r="H18" s="53" t="inlineStr">
         <is>
-          <t>1X</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I18" s="55" t="n">
-        <v>81.8</v>
+        <v>82.09999999999999</v>
       </c>
     </row>
     <row r="19">
@@ -18136,27 +18169,27 @@
       </c>
       <c r="B19" s="53" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="C19" s="53" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Fransa</t>
         </is>
       </c>
       <c r="D19" s="53" t="inlineStr">
         <is>
-          <t>Süper Lig</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="E19" s="54" t="inlineStr">
         <is>
-          <t>Fenerbahce</t>
+          <t>Lille OSC</t>
         </is>
       </c>
       <c r="F19" s="54" t="inlineStr">
         <is>
-          <t>Alanyaspor</t>
+          <t>Stade Brestois 29</t>
         </is>
       </c>
       <c r="G19" s="53" t="inlineStr">
@@ -18170,7 +18203,7 @@
         </is>
       </c>
       <c r="I19" s="55" t="n">
-        <v>81.5</v>
+        <v>81.8</v>
       </c>
     </row>
     <row r="20">
@@ -18181,27 +18214,27 @@
       </c>
       <c r="B20" s="53" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C20" s="53" t="inlineStr">
         <is>
-          <t>Almanya</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="D20" s="53" t="inlineStr">
         <is>
-          <t>2. Bundesliga</t>
+          <t>Süper Lig</t>
         </is>
       </c>
       <c r="E20" s="54" t="inlineStr">
         <is>
-          <t>Wolfsburg</t>
+          <t>Fenerbahce</t>
         </is>
       </c>
       <c r="F20" s="54" t="inlineStr">
         <is>
-          <t>Heidenheim</t>
+          <t>Alanyaspor</t>
         </is>
       </c>
       <c r="G20" s="53" t="inlineStr">
@@ -18211,11 +18244,11 @@
       </c>
       <c r="H20" s="53" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>1X</t>
         </is>
       </c>
       <c r="I20" s="55" t="n">
-        <v>81.40000000000001</v>
+        <v>81.5</v>
       </c>
     </row>
     <row r="21">
@@ -19695,7 +19728,7 @@
     <row r="3">
       <c r="A3" s="57" t="inlineStr">
         <is>
-          <t>Oluşturulma zamanı: 17.10.2026 08:33</t>
+          <t>Oluşturulma zamanı: 17.10.2026 13:32</t>
         </is>
       </c>
     </row>

</xml_diff>